<commit_message>
Actualización automática 2026-01-09 16:30:07
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -720,7 +720,7 @@
         <v>0</v>
       </c>
       <c r="M4" s="2" t="n">
-        <v>51.96</v>
+        <v>181.88</v>
       </c>
       <c r="N4" s="2" t="n">
         <v>0</v>
@@ -4015,7 +4015,7 @@
         <v>13723.92</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>113.02</v>
+        <v>242.94</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>15000</v>
@@ -5517,7 +5517,7 @@
         <v>113883.77</v>
       </c>
       <c r="F60" s="6" t="n">
-        <v>10313.58</v>
+        <v>10443.5</v>
       </c>
       <c r="G60" s="6" t="n">
         <v>115950</v>

</xml_diff>

<commit_message>
Actualización automática 2026-01-19 17:30:09
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -2248,7 +2248,7 @@
         <v>0</v>
       </c>
       <c r="M29" s="2" t="n">
-        <v>0</v>
+        <v>5897.23</v>
       </c>
       <c r="N29" s="2" t="n">
         <v>0</v>
@@ -2257,7 +2257,7 @@
         <v>0</v>
       </c>
       <c r="P29" s="2" t="n">
-        <v>116.86</v>
+        <v>140.23</v>
       </c>
       <c r="Q29" s="2" t="n">
         <v>0</v>
@@ -2701,7 +2701,7 @@
         <v>0</v>
       </c>
       <c r="D37" s="2" t="n">
-        <v>0</v>
+        <v>915.84</v>
       </c>
       <c r="E37" s="2" t="n">
         <v>0</v>
@@ -3313,7 +3313,7 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>0</v>
+        <v>853.2</v>
       </c>
       <c r="I47" s="2" t="n">
         <v>0</v>
@@ -3328,7 +3328,7 @@
         <v>0</v>
       </c>
       <c r="M47" s="2" t="n">
-        <v>0</v>
+        <v>1260.23</v>
       </c>
       <c r="N47" s="2" t="n">
         <v>0</v>
@@ -3688,7 +3688,7 @@
         <v>0</v>
       </c>
       <c r="M53" s="2" t="n">
-        <v>66.09999999999999</v>
+        <v>336.6</v>
       </c>
       <c r="N53" s="2" t="n">
         <v>0</v>
@@ -3834,7 +3834,7 @@
       </c>
       <c r="D56" s="4" t="inlineStr">
         <is>
-          <t>6 de 54</t>
+          <t>7 de 54</t>
         </is>
       </c>
       <c r="E56" s="4" t="inlineStr">
@@ -3854,24 +3854,24 @@
       </c>
       <c r="H56" s="4" t="inlineStr">
         <is>
+          <t>3 de 54</t>
+        </is>
+      </c>
+      <c r="I56" s="4" t="inlineStr">
+        <is>
+          <t>1 de 54</t>
+        </is>
+      </c>
+      <c r="J56" s="4" t="inlineStr">
+        <is>
+          <t>0 de 54</t>
+        </is>
+      </c>
+      <c r="K56" s="4" t="inlineStr">
+        <is>
           <t>2 de 54</t>
         </is>
       </c>
-      <c r="I56" s="4" t="inlineStr">
-        <is>
-          <t>1 de 54</t>
-        </is>
-      </c>
-      <c r="J56" s="4" t="inlineStr">
-        <is>
-          <t>0 de 54</t>
-        </is>
-      </c>
-      <c r="K56" s="4" t="inlineStr">
-        <is>
-          <t>2 de 54</t>
-        </is>
-      </c>
       <c r="L56" s="4" t="inlineStr">
         <is>
           <t>3 de 54</t>
@@ -3879,7 +3879,7 @@
       </c>
       <c r="M56" s="4" t="inlineStr">
         <is>
-          <t>11 de 54</t>
+          <t>13 de 54</t>
         </is>
       </c>
       <c r="N56" s="4" t="inlineStr">
@@ -4718,7 +4718,7 @@
         <v>8513.129999999999</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>610.15</v>
+        <v>6530.75</v>
       </c>
       <c r="G29" s="2" t="n">
         <v>6000</v>
@@ -4934,7 +4934,7 @@
         <v>7074.68</v>
       </c>
       <c r="F37" s="2" t="n">
-        <v>4345.85</v>
+        <v>5261.69</v>
       </c>
       <c r="G37" s="2" t="n">
         <v>8000</v>
@@ -5204,7 +5204,7 @@
         <v>794.5599999999999</v>
       </c>
       <c r="F47" s="2" t="n">
-        <v>0</v>
+        <v>2113.43</v>
       </c>
       <c r="G47" s="2" t="n">
         <v>1500</v>
@@ -5420,7 +5420,7 @@
         <v>1657.97</v>
       </c>
       <c r="F55" s="2" t="n">
-        <v>66.09999999999999</v>
+        <v>336.6</v>
       </c>
       <c r="G55" s="2" t="n">
         <v>500</v>
@@ -5447,7 +5447,7 @@
         <v>1657.97</v>
       </c>
       <c r="F56" s="2" t="n">
-        <v>66.09999999999999</v>
+        <v>336.6</v>
       </c>
       <c r="G56" s="2" t="n">
         <v>1000</v>
@@ -5545,7 +5545,7 @@
         <v>113883.77</v>
       </c>
       <c r="F60" s="5" t="n">
-        <v>26448.35</v>
+        <v>35939.22</v>
       </c>
       <c r="G60" s="5" t="n">
         <v>115950</v>
@@ -5569,7 +5569,7 @@
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="23" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
     <col width="27" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -5644,13 +5644,13 @@
         <v>8826</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>4321.44</v>
+        <v>5237.28</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>4504.56</v>
+        <v>3588.72</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>0.4896261046906866</v>
+        <v>0.5933922501699523</v>
       </c>
     </row>
     <row r="4">
@@ -5716,13 +5716,13 @@
         <v>1275</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>869.4</v>
+        <v>1722.6</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>405.6</v>
+        <v>-447.5999999999999</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>0.6818823529411765</v>
+        <v>1.351058823529412</v>
       </c>
     </row>
     <row r="7">
@@ -5764,13 +5764,13 @@
         <v>250</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>360.92</v>
+        <v>384.29</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>-110.92</v>
+        <v>-134.29</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>1.44368</v>
+        <v>1.53716</v>
       </c>
     </row>
     <row r="9">
@@ -5860,13 +5860,13 @@
         <v>57320</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>12808.36</v>
+        <v>20236.32</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>44511.64</v>
+        <v>37083.68</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0.223453593859037</v>
+        <v>0.3530411723656665</v>
       </c>
     </row>
     <row r="13">
@@ -5927,13 +5927,13 @@
         <v>90296.82000000001</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>26355.25</v>
+        <v>35575.62</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>63941.56999999999</v>
+        <v>54721.2</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.2918735122676523</v>
+        <v>0.3939853031369211</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-01-21 16:30:13
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -661,7 +661,7 @@
         <v>0</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>0</v>
+        <v>396</v>
       </c>
       <c r="E3" s="2" t="n">
         <v>0</v>
@@ -748,7 +748,7 @@
         <v>0</v>
       </c>
       <c r="M4" s="2" t="n">
-        <v>347.72</v>
+        <v>540.46</v>
       </c>
       <c r="N4" s="2" t="n">
         <v>0</v>
@@ -2236,7 +2236,7 @@
         <v>0</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>0</v>
+        <v>165.6</v>
       </c>
       <c r="J29" s="2" t="n">
         <v>0</v>
@@ -2638,7 +2638,7 @@
         </is>
       </c>
       <c r="C36" s="2" t="n">
-        <v>0</v>
+        <v>388.8</v>
       </c>
       <c r="D36" s="2" t="n">
         <v>0</v>
@@ -2668,7 +2668,7 @@
         <v>565.25</v>
       </c>
       <c r="M36" s="2" t="n">
-        <v>1878.05</v>
+        <v>1904.62</v>
       </c>
       <c r="N36" s="2" t="n">
         <v>0</v>
@@ -2941,7 +2941,7 @@
         <v>0</v>
       </c>
       <c r="D41" s="2" t="n">
-        <v>0</v>
+        <v>305.28</v>
       </c>
       <c r="E41" s="2" t="n">
         <v>0</v>
@@ -2968,7 +2968,7 @@
         <v>0</v>
       </c>
       <c r="M41" s="2" t="n">
-        <v>0</v>
+        <v>158.98</v>
       </c>
       <c r="N41" s="2" t="n">
         <v>0</v>
@@ -2980,7 +2980,7 @@
         <v>0</v>
       </c>
       <c r="Q41" s="2" t="n">
-        <v>0</v>
+        <v>669.0599999999999</v>
       </c>
       <c r="R41" s="2" t="n">
         <v>0</v>
@@ -3268,7 +3268,7 @@
         <v>0</v>
       </c>
       <c r="M46" s="2" t="n">
-        <v>0</v>
+        <v>2709</v>
       </c>
       <c r="N46" s="2" t="n">
         <v>0</v>
@@ -3829,77 +3829,77 @@
     <row r="56">
       <c r="C56" s="4" t="inlineStr">
         <is>
+          <t>1 de 54</t>
+        </is>
+      </c>
+      <c r="D56" s="4" t="inlineStr">
+        <is>
+          <t>9 de 54</t>
+        </is>
+      </c>
+      <c r="E56" s="4" t="inlineStr">
+        <is>
+          <t>2 de 54</t>
+        </is>
+      </c>
+      <c r="F56" s="4" t="inlineStr">
+        <is>
           <t>0 de 54</t>
         </is>
       </c>
-      <c r="D56" s="4" t="inlineStr">
-        <is>
-          <t>7 de 54</t>
-        </is>
-      </c>
-      <c r="E56" s="4" t="inlineStr">
+      <c r="G56" s="4" t="inlineStr">
+        <is>
+          <t>0 de 54</t>
+        </is>
+      </c>
+      <c r="H56" s="4" t="inlineStr">
+        <is>
+          <t>3 de 54</t>
+        </is>
+      </c>
+      <c r="I56" s="4" t="inlineStr">
         <is>
           <t>2 de 54</t>
         </is>
       </c>
-      <c r="F56" s="4" t="inlineStr">
+      <c r="J56" s="4" t="inlineStr">
         <is>
           <t>0 de 54</t>
         </is>
       </c>
-      <c r="G56" s="4" t="inlineStr">
+      <c r="K56" s="4" t="inlineStr">
+        <is>
+          <t>2 de 54</t>
+        </is>
+      </c>
+      <c r="L56" s="4" t="inlineStr">
+        <is>
+          <t>3 de 54</t>
+        </is>
+      </c>
+      <c r="M56" s="4" t="inlineStr">
+        <is>
+          <t>15 de 54</t>
+        </is>
+      </c>
+      <c r="N56" s="4" t="inlineStr">
         <is>
           <t>0 de 54</t>
         </is>
       </c>
-      <c r="H56" s="4" t="inlineStr">
-        <is>
-          <t>3 de 54</t>
-        </is>
-      </c>
-      <c r="I56" s="4" t="inlineStr">
-        <is>
-          <t>1 de 54</t>
-        </is>
-      </c>
-      <c r="J56" s="4" t="inlineStr">
+      <c r="O56" s="4" t="inlineStr">
         <is>
           <t>0 de 54</t>
         </is>
       </c>
-      <c r="K56" s="4" t="inlineStr">
+      <c r="P56" s="4" t="inlineStr">
         <is>
           <t>2 de 54</t>
         </is>
       </c>
-      <c r="L56" s="4" t="inlineStr">
-        <is>
-          <t>3 de 54</t>
-        </is>
-      </c>
-      <c r="M56" s="4" t="inlineStr">
-        <is>
-          <t>13 de 54</t>
-        </is>
-      </c>
-      <c r="N56" s="4" t="inlineStr">
-        <is>
-          <t>0 de 54</t>
-        </is>
-      </c>
-      <c r="O56" s="4" t="inlineStr">
-        <is>
-          <t>0 de 54</t>
-        </is>
-      </c>
-      <c r="P56" s="4" t="inlineStr">
-        <is>
-          <t>2 de 54</t>
-        </is>
-      </c>
       <c r="Q56" s="4" t="inlineStr">
         <is>
-          <t>3 de 54</t>
+          <t>4 de 54</t>
         </is>
       </c>
       <c r="R56" s="4" t="inlineStr">
@@ -4016,7 +4016,7 @@
         <v>1237.68</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>244.06</v>
+        <v>640.0599999999999</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>1000</v>
@@ -4043,7 +4043,7 @@
         <v>13723.92</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>408.78</v>
+        <v>601.52</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>15000</v>
@@ -4718,7 +4718,7 @@
         <v>8513.129999999999</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>6530.75</v>
+        <v>6696.35</v>
       </c>
       <c r="G29" s="2" t="n">
         <v>6000</v>
@@ -4907,7 +4907,7 @@
         <v>17009.67</v>
       </c>
       <c r="F36" s="2" t="n">
-        <v>4227.46</v>
+        <v>4642.83</v>
       </c>
       <c r="G36" s="2" t="n">
         <v>10000</v>
@@ -5042,7 +5042,7 @@
         <v>32.53</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>0</v>
+        <v>1133.32</v>
       </c>
       <c r="G41" s="2" t="n">
         <v>1000</v>
@@ -5177,7 +5177,7 @@
         <v>0</v>
       </c>
       <c r="F46" s="2" t="n">
-        <v>1613.52</v>
+        <v>4322.52</v>
       </c>
       <c r="G46" s="2" t="n">
         <v>1500</v>
@@ -5545,7 +5545,7 @@
         <v>113883.77</v>
       </c>
       <c r="F60" s="5" t="n">
-        <v>35939.22</v>
+        <v>40951.25</v>
       </c>
       <c r="G60" s="5" t="n">
         <v>115950</v>
@@ -5620,13 +5620,13 @@
         <v>1036</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0</v>
+        <v>388.8</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>1036</v>
+        <v>647.2</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>0</v>
+        <v>0.3752895752895753</v>
       </c>
     </row>
     <row r="3">
@@ -5644,13 +5644,13 @@
         <v>8826</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>5237.28</v>
+        <v>5938.56</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>3588.72</v>
+        <v>2887.44</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>0.5933922501699523</v>
+        <v>0.6728484024473148</v>
       </c>
     </row>
     <row r="4">
@@ -5740,13 +5740,13 @@
         <v>974.4</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>132.3</v>
+        <v>297.9</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>842.0999999999999</v>
+        <v>676.5</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>0.1357758620689655</v>
+        <v>0.3057266009852216</v>
       </c>
     </row>
     <row r="8">
@@ -5788,10 +5788,10 @@
         <v>0</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>3644.53</v>
+        <v>4313.59</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>-3644.53</v>
+        <v>-4313.59</v>
       </c>
       <c r="F9" s="3" t="n">
         <v>0</v>
@@ -5860,13 +5860,13 @@
         <v>57320</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>20236.32</v>
+        <v>23323.61</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>37083.68</v>
+        <v>33996.39</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0.3530411723656665</v>
+        <v>0.4069017794836008</v>
       </c>
     </row>
     <row r="13">
@@ -5927,13 +5927,13 @@
         <v>90296.82000000001</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>35575.62</v>
+        <v>40587.65</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>54721.2</v>
+        <v>49709.17</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.3939853031369211</v>
+        <v>0.449491466033909</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-01-30 08:30:12
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -1288,7 +1288,7 @@
         <v>0</v>
       </c>
       <c r="M13" s="2" t="n">
-        <v>-345.98</v>
+        <v>-1064.83</v>
       </c>
       <c r="N13" s="2" t="n">
         <v>0</v>
@@ -1444,7 +1444,7 @@
         <v>0</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>0</v>
+        <v>661.13</v>
       </c>
       <c r="F16" s="2" t="n">
         <v>0</v>
@@ -1465,10 +1465,10 @@
         <v>0</v>
       </c>
       <c r="L16" s="2" t="n">
-        <v>0</v>
+        <v>623.74</v>
       </c>
       <c r="M16" s="2" t="n">
-        <v>1110.9</v>
+        <v>1709.94</v>
       </c>
       <c r="N16" s="2" t="n">
         <v>0</v>
@@ -1828,7 +1828,7 @@
         <v>0</v>
       </c>
       <c r="M22" s="2" t="n">
-        <v>0</v>
+        <v>6.12</v>
       </c>
       <c r="N22" s="2" t="n">
         <v>0</v>
@@ -2224,7 +2224,7 @@
         <v>475.2</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>0</v>
+        <v>55.65</v>
       </c>
       <c r="F29" s="2" t="n">
         <v>0</v>
@@ -2242,13 +2242,13 @@
         <v>0</v>
       </c>
       <c r="K29" s="2" t="n">
-        <v>18.09</v>
+        <v>19.62</v>
       </c>
       <c r="L29" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M29" s="2" t="n">
-        <v>5897.23</v>
+        <v>6106.39</v>
       </c>
       <c r="N29" s="2" t="n">
         <v>0</v>
@@ -2662,10 +2662,10 @@
         <v>0</v>
       </c>
       <c r="K36" s="2" t="n">
-        <v>203.04</v>
+        <v>172.58</v>
       </c>
       <c r="L36" s="2" t="n">
-        <v>565.25</v>
+        <v>2604.12</v>
       </c>
       <c r="M36" s="2" t="n">
         <v>1787.67</v>
@@ -3256,7 +3256,7 @@
         <v>0</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>205.2</v>
+        <v>820.8</v>
       </c>
       <c r="J46" s="2" t="n">
         <v>0</v>
@@ -3839,47 +3839,47 @@
       </c>
       <c r="E56" s="4" t="inlineStr">
         <is>
+          <t>5 de 54</t>
+        </is>
+      </c>
+      <c r="F56" s="4" t="inlineStr">
+        <is>
+          <t>0 de 54</t>
+        </is>
+      </c>
+      <c r="G56" s="4" t="inlineStr">
+        <is>
+          <t>0 de 54</t>
+        </is>
+      </c>
+      <c r="H56" s="4" t="inlineStr">
+        <is>
           <t>3 de 54</t>
         </is>
       </c>
-      <c r="F56" s="4" t="inlineStr">
-        <is>
-          <t>0 de 54</t>
-        </is>
-      </c>
-      <c r="G56" s="4" t="inlineStr">
-        <is>
-          <t>0 de 54</t>
-        </is>
-      </c>
-      <c r="H56" s="4" t="inlineStr">
+      <c r="I56" s="4" t="inlineStr">
+        <is>
+          <t>2 de 54</t>
+        </is>
+      </c>
+      <c r="J56" s="4" t="inlineStr">
+        <is>
+          <t>1 de 54</t>
+        </is>
+      </c>
+      <c r="K56" s="4" t="inlineStr">
         <is>
           <t>3 de 54</t>
         </is>
       </c>
-      <c r="I56" s="4" t="inlineStr">
-        <is>
-          <t>2 de 54</t>
-        </is>
-      </c>
-      <c r="J56" s="4" t="inlineStr">
-        <is>
-          <t>1 de 54</t>
-        </is>
-      </c>
-      <c r="K56" s="4" t="inlineStr">
-        <is>
-          <t>3 de 54</t>
-        </is>
-      </c>
       <c r="L56" s="4" t="inlineStr">
         <is>
-          <t>4 de 54</t>
+          <t>5 de 54</t>
         </is>
       </c>
       <c r="M56" s="4" t="inlineStr">
         <is>
-          <t>16 de 54</t>
+          <t>17 de 54</t>
         </is>
       </c>
       <c r="N56" s="4" t="inlineStr">
@@ -3927,7 +3927,7 @@
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -4286,7 +4286,7 @@
         <v>3046.3</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>-345.98</v>
+        <v>-1064.83</v>
       </c>
       <c r="G13" s="2" t="n">
         <v>6000</v>
@@ -4367,7 +4367,7 @@
         <v>6914.1</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>1110.9</v>
+        <v>2994.81</v>
       </c>
       <c r="G16" s="2" t="n">
         <v>6000</v>
@@ -4529,7 +4529,7 @@
         <v>0</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>253.8</v>
+        <v>259.92</v>
       </c>
       <c r="G22" s="2" t="n">
         <v>0</v>
@@ -4718,7 +4718,7 @@
         <v>8513.129999999999</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>6696.35</v>
+        <v>6962.69</v>
       </c>
       <c r="G29" s="2" t="n">
         <v>6000</v>
@@ -4907,7 +4907,7 @@
         <v>17009.67</v>
       </c>
       <c r="F36" s="2" t="n">
-        <v>7448.76</v>
+        <v>9457.17</v>
       </c>
       <c r="G36" s="2" t="n">
         <v>10000</v>
@@ -5042,7 +5042,7 @@
         <v>32.53</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>1133.32</v>
+        <v>1579.36</v>
       </c>
       <c r="G41" s="2" t="n">
         <v>1000</v>
@@ -5177,7 +5177,7 @@
         <v>0</v>
       </c>
       <c r="F46" s="2" t="n">
-        <v>4736.54</v>
+        <v>5352.14</v>
       </c>
       <c r="G46" s="2" t="n">
         <v>1500</v>
@@ -5545,7 +5545,7 @@
         <v>113883.77</v>
       </c>
       <c r="F60" s="5" t="n">
-        <v>51512.48</v>
+        <v>56020.05</v>
       </c>
       <c r="G60" s="5" t="n">
         <v>115950</v>
@@ -5569,7 +5569,7 @@
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="23" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
     <col width="27" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -5668,13 +5668,13 @@
         <v>369.6</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>367.05</v>
+        <v>1083.83</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>2.550000000000011</v>
+        <v>-714.2299999999999</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>0.9931006493506493</v>
+        <v>2.932440476190476</v>
       </c>
     </row>
     <row r="5">
@@ -5740,13 +5740,13 @@
         <v>974.4</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>297.9</v>
+        <v>913.5</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>676.5</v>
+        <v>60.89999999999998</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>0.3057266009852216</v>
+        <v>0.9375</v>
       </c>
     </row>
     <row r="8">
@@ -5812,13 +5812,13 @@
         <v>2850</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>248.13</v>
+        <v>219.2</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>2601.87</v>
+        <v>2630.8</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>0.08706315789473684</v>
+        <v>0.07691228070175438</v>
       </c>
     </row>
     <row r="11">
@@ -5836,13 +5836,13 @@
         <v>4200</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>6677.6</v>
+        <v>7123.64</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>-2477.6</v>
+        <v>-2923.64</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>1.589904761904762</v>
+        <v>1.696104761904762</v>
       </c>
     </row>
     <row r="12">
@@ -5860,13 +5860,13 @@
         <v>13321</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>5981.91</v>
+        <v>8644.52</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>7339.09</v>
+        <v>4676.48</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0.4490586292320397</v>
+        <v>0.6489392688236619</v>
       </c>
     </row>
     <row r="13">
@@ -5884,13 +5884,13 @@
         <v>57320</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>24273.66</v>
+        <v>24369.13</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>33046.34</v>
+        <v>32950.87</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.4234762735519889</v>
+        <v>0.4251418353105373</v>
       </c>
     </row>
     <row r="14">
@@ -5951,13 +5951,13 @@
         <v>94496.82000000001</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>51070.25999999999</v>
+        <v>55577.83</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>43426.56</v>
+        <v>38918.99000000001</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.5404442181228954</v>
+        <v>0.5881449767304339</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-02-04 17:30:15
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -724,7 +724,7 @@
         <v>0</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>0</v>
+        <v>250.11</v>
       </c>
       <c r="F4" s="2" t="n">
         <v>0</v>
@@ -1441,7 +1441,7 @@
         <v>0</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>0</v>
+        <v>1188</v>
       </c>
       <c r="E16" s="2" t="n">
         <v>0</v>
@@ -1468,7 +1468,7 @@
         <v>0</v>
       </c>
       <c r="M16" s="2" t="n">
-        <v>0</v>
+        <v>3079.58</v>
       </c>
       <c r="N16" s="2" t="n">
         <v>0</v>
@@ -1936,7 +1936,7 @@
         <v>205.2</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>0</v>
+        <v>118.8</v>
       </c>
       <c r="J24" s="2" t="n">
         <v>0</v>
@@ -3688,7 +3688,7 @@
         <v>0</v>
       </c>
       <c r="M53" s="2" t="n">
-        <v>0</v>
+        <v>524.88</v>
       </c>
       <c r="N53" s="2" t="n">
         <v>0</v>
@@ -3697,7 +3697,7 @@
         <v>0</v>
       </c>
       <c r="P53" s="2" t="n">
-        <v>0</v>
+        <v>724.52</v>
       </c>
       <c r="Q53" s="2" t="n">
         <v>0</v>
@@ -3834,67 +3834,67 @@
       </c>
       <c r="D56" s="4" t="inlineStr">
         <is>
+          <t>1 de 54</t>
+        </is>
+      </c>
+      <c r="E56" s="4" t="inlineStr">
+        <is>
+          <t>1 de 54</t>
+        </is>
+      </c>
+      <c r="F56" s="4" t="inlineStr">
+        <is>
           <t>0 de 54</t>
         </is>
       </c>
-      <c r="E56" s="4" t="inlineStr">
+      <c r="G56" s="4" t="inlineStr">
         <is>
           <t>0 de 54</t>
         </is>
       </c>
-      <c r="F56" s="4" t="inlineStr">
+      <c r="H56" s="4" t="inlineStr">
+        <is>
+          <t>1 de 54</t>
+        </is>
+      </c>
+      <c r="I56" s="4" t="inlineStr">
+        <is>
+          <t>1 de 54</t>
+        </is>
+      </c>
+      <c r="J56" s="4" t="inlineStr">
         <is>
           <t>0 de 54</t>
         </is>
       </c>
-      <c r="G56" s="4" t="inlineStr">
+      <c r="K56" s="4" t="inlineStr">
+        <is>
+          <t>1 de 54</t>
+        </is>
+      </c>
+      <c r="L56" s="4" t="inlineStr">
+        <is>
+          <t>1 de 54</t>
+        </is>
+      </c>
+      <c r="M56" s="4" t="inlineStr">
+        <is>
+          <t>5 de 54</t>
+        </is>
+      </c>
+      <c r="N56" s="4" t="inlineStr">
         <is>
           <t>0 de 54</t>
         </is>
       </c>
-      <c r="H56" s="4" t="inlineStr">
+      <c r="O56" s="4" t="inlineStr">
+        <is>
+          <t>0 de 54</t>
+        </is>
+      </c>
+      <c r="P56" s="4" t="inlineStr">
         <is>
           <t>1 de 54</t>
-        </is>
-      </c>
-      <c r="I56" s="4" t="inlineStr">
-        <is>
-          <t>0 de 54</t>
-        </is>
-      </c>
-      <c r="J56" s="4" t="inlineStr">
-        <is>
-          <t>0 de 54</t>
-        </is>
-      </c>
-      <c r="K56" s="4" t="inlineStr">
-        <is>
-          <t>1 de 54</t>
-        </is>
-      </c>
-      <c r="L56" s="4" t="inlineStr">
-        <is>
-          <t>1 de 54</t>
-        </is>
-      </c>
-      <c r="M56" s="4" t="inlineStr">
-        <is>
-          <t>3 de 54</t>
-        </is>
-      </c>
-      <c r="N56" s="4" t="inlineStr">
-        <is>
-          <t>0 de 54</t>
-        </is>
-      </c>
-      <c r="O56" s="4" t="inlineStr">
-        <is>
-          <t>0 de 54</t>
-        </is>
-      </c>
-      <c r="P56" s="4" t="inlineStr">
-        <is>
-          <t>0 de 54</t>
         </is>
       </c>
       <c r="Q56" s="4" t="inlineStr">
@@ -4043,7 +4043,7 @@
         <v>689.65</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>48.19</v>
+        <v>298.3</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>15000</v>
@@ -4367,7 +4367,7 @@
         <v>2994.81</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>0</v>
+        <v>4267.58</v>
       </c>
       <c r="G16" s="2" t="n">
         <v>6000</v>
@@ -4583,7 +4583,7 @@
         <v>3774.95</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>5560.92</v>
+        <v>5679.72</v>
       </c>
       <c r="G24" s="2" t="n">
         <v>15000</v>
@@ -5420,7 +5420,7 @@
         <v>336.6</v>
       </c>
       <c r="F55" s="2" t="n">
-        <v>0</v>
+        <v>1249.4</v>
       </c>
       <c r="G55" s="2" t="n">
         <v>500</v>
@@ -5447,7 +5447,7 @@
         <v>336.6</v>
       </c>
       <c r="F56" s="2" t="n">
-        <v>0</v>
+        <v>1249.4</v>
       </c>
       <c r="G56" s="2" t="n">
         <v>1000</v>
@@ -5545,7 +5545,7 @@
         <v>79907.13</v>
       </c>
       <c r="F60" s="5" t="n">
-        <v>9808.549999999999</v>
+        <v>16943.84</v>
       </c>
       <c r="G60" s="5" t="n">
         <v>115950</v>

</xml_diff>

<commit_message>
Actualización automática 2026-02-06 15:30:21
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -748,7 +748,7 @@
         <v>0</v>
       </c>
       <c r="M4" s="2" t="n">
-        <v>48.19</v>
+        <v>72.28</v>
       </c>
       <c r="N4" s="2" t="n">
         <v>0</v>
@@ -2368,7 +2368,7 @@
         <v>0</v>
       </c>
       <c r="M31" s="2" t="n">
-        <v>0</v>
+        <v>72.48999999999999</v>
       </c>
       <c r="N31" s="2" t="n">
         <v>0</v>
@@ -3879,7 +3879,7 @@
       </c>
       <c r="M56" s="4" t="inlineStr">
         <is>
-          <t>6 de 54</t>
+          <t>7 de 54</t>
         </is>
       </c>
       <c r="N56" s="4" t="inlineStr">
@@ -4043,7 +4043,7 @@
         <v>689.65</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>298.3</v>
+        <v>322.39</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>15000</v>
@@ -4772,7 +4772,7 @@
         <v>0</v>
       </c>
       <c r="F31" s="2" t="n">
-        <v>0</v>
+        <v>72.48999999999999</v>
       </c>
       <c r="G31" s="2" t="n">
         <v>1500</v>
@@ -5545,7 +5545,7 @@
         <v>79907.13</v>
       </c>
       <c r="F60" s="5" t="n">
-        <v>16997.45</v>
+        <v>17094.03</v>
       </c>
       <c r="G60" s="5" t="n">
         <v>115950</v>
@@ -5884,13 +5884,13 @@
         <v>49256</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>9131.43</v>
+        <v>9228.01</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>40124.57</v>
+        <v>40027.99</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.1853871609550106</v>
+        <v>0.1873479373071301</v>
       </c>
     </row>
     <row r="14">
@@ -5951,13 +5951,13 @@
         <v>82482.82000000001</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>15748.05</v>
+        <v>15844.63</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>66734.76999999999</v>
+        <v>66638.19</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.1909252132747159</v>
+        <v>0.1920961237746236</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-02-10 08:30:16
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -748,7 +748,7 @@
         <v>0</v>
       </c>
       <c r="M4" s="2" t="n">
-        <v>72.28</v>
+        <v>402.76</v>
       </c>
       <c r="N4" s="2" t="n">
         <v>0</v>
@@ -778,10 +778,10 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>0</v>
+        <v>388.8</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>0</v>
+        <v>534.24</v>
       </c>
       <c r="E5" s="2" t="n">
         <v>0</v>
@@ -805,7 +805,7 @@
         <v>0</v>
       </c>
       <c r="L5" s="2" t="n">
-        <v>0</v>
+        <v>253.44</v>
       </c>
       <c r="M5" s="2" t="n">
         <v>0</v>
@@ -1168,7 +1168,7 @@
         <v>0</v>
       </c>
       <c r="M11" s="2" t="n">
-        <v>0</v>
+        <v>3036.01</v>
       </c>
       <c r="N11" s="2" t="n">
         <v>0</v>
@@ -2041,7 +2041,7 @@
         <v>0</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>0</v>
+        <v>1555.2</v>
       </c>
       <c r="E26" s="2" t="n">
         <v>0</v>
@@ -3829,57 +3829,57 @@
     <row r="56">
       <c r="C56" s="4" t="inlineStr">
         <is>
+          <t>1 de 54</t>
+        </is>
+      </c>
+      <c r="D56" s="4" t="inlineStr">
+        <is>
+          <t>3 de 54</t>
+        </is>
+      </c>
+      <c r="E56" s="4" t="inlineStr">
+        <is>
+          <t>1 de 54</t>
+        </is>
+      </c>
+      <c r="F56" s="4" t="inlineStr">
+        <is>
           <t>0 de 54</t>
         </is>
       </c>
-      <c r="D56" s="4" t="inlineStr">
+      <c r="G56" s="4" t="inlineStr">
+        <is>
+          <t>0 de 54</t>
+        </is>
+      </c>
+      <c r="H56" s="4" t="inlineStr">
         <is>
           <t>1 de 54</t>
         </is>
       </c>
-      <c r="E56" s="4" t="inlineStr">
+      <c r="I56" s="4" t="inlineStr">
         <is>
           <t>1 de 54</t>
         </is>
       </c>
-      <c r="F56" s="4" t="inlineStr">
+      <c r="J56" s="4" t="inlineStr">
         <is>
           <t>0 de 54</t>
         </is>
       </c>
-      <c r="G56" s="4" t="inlineStr">
-        <is>
-          <t>0 de 54</t>
-        </is>
-      </c>
-      <c r="H56" s="4" t="inlineStr">
+      <c r="K56" s="4" t="inlineStr">
         <is>
           <t>1 de 54</t>
         </is>
       </c>
-      <c r="I56" s="4" t="inlineStr">
-        <is>
-          <t>1 de 54</t>
-        </is>
-      </c>
-      <c r="J56" s="4" t="inlineStr">
-        <is>
-          <t>0 de 54</t>
-        </is>
-      </c>
-      <c r="K56" s="4" t="inlineStr">
-        <is>
-          <t>1 de 54</t>
-        </is>
-      </c>
       <c r="L56" s="4" t="inlineStr">
         <is>
-          <t>1 de 54</t>
+          <t>2 de 54</t>
         </is>
       </c>
       <c r="M56" s="4" t="inlineStr">
         <is>
-          <t>8 de 54</t>
+          <t>9 de 54</t>
         </is>
       </c>
       <c r="N56" s="4" t="inlineStr">
@@ -4043,7 +4043,7 @@
         <v>689.65</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>322.39</v>
+        <v>652.87</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>15000</v>
@@ -4070,7 +4070,7 @@
         <v>10936.72</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>0</v>
+        <v>1176.48</v>
       </c>
       <c r="G5" s="2" t="n">
         <v>10000</v>
@@ -4232,7 +4232,7 @@
         <v>6.12</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>0</v>
+        <v>3036.01</v>
       </c>
       <c r="G11" s="2" t="n">
         <v>500</v>
@@ -4637,7 +4637,7 @@
         <v>615.6</v>
       </c>
       <c r="F26" s="2" t="n">
-        <v>0</v>
+        <v>1555.2</v>
       </c>
       <c r="G26" s="2" t="n">
         <v>500</v>
@@ -5545,7 +5545,7 @@
         <v>79907.13</v>
       </c>
       <c r="F60" s="5" t="n">
-        <v>18859.18</v>
+        <v>24957.35</v>
       </c>
       <c r="G60" s="5" t="n">
         <v>115950</v>
@@ -5569,7 +5569,7 @@
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="5" max="5"/>
     <col width="25" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -5620,13 +5620,13 @@
         <v>1036</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0</v>
+        <v>388.8</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>1036</v>
+        <v>647.2</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>0</v>
+        <v>0.3752895752895753</v>
       </c>
     </row>
     <row r="3">
@@ -5644,13 +5644,13 @@
         <v>8826</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>1188</v>
+        <v>3277.44</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>7638</v>
+        <v>5548.559999999999</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>0.1346023113528212</v>
+        <v>0.3713392250169952</v>
       </c>
     </row>
     <row r="4">
@@ -5860,13 +5860,13 @@
         <v>13321</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>3977.71</v>
+        <v>4231.15</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>9343.290000000001</v>
+        <v>9089.85</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0.2986044591246904</v>
+        <v>0.3176300578034682</v>
       </c>
     </row>
     <row r="13">
@@ -5884,13 +5884,13 @@
         <v>49256</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>10993.16</v>
+        <v>14359.65</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>38262.84</v>
+        <v>34896.35</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.2231841806074387</v>
+        <v>0.2915309809972389</v>
       </c>
     </row>
     <row r="14">
@@ -5951,13 +5951,13 @@
         <v>82482.82000000001</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>17609.78</v>
+        <v>23707.95</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>64873.03999999999</v>
+        <v>58774.87</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.2134963377828255</v>
+        <v>0.2874289458095637</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-02-10 12:30:21
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -1288,7 +1288,7 @@
         <v>0</v>
       </c>
       <c r="M13" s="2" t="n">
-        <v>-311.04</v>
+        <v>-1617.41</v>
       </c>
       <c r="N13" s="2" t="n">
         <v>0</v>
@@ -3927,7 +3927,7 @@
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -4286,7 +4286,7 @@
         <v>-1064.83</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>-311.04</v>
+        <v>-1617.41</v>
       </c>
       <c r="G13" s="2" t="n">
         <v>6000</v>
@@ -5545,7 +5545,7 @@
         <v>79907.13</v>
       </c>
       <c r="F60" s="5" t="n">
-        <v>24957.35</v>
+        <v>23650.98</v>
       </c>
       <c r="G60" s="5" t="n">
         <v>115950</v>
@@ -5884,13 +5884,13 @@
         <v>49256</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>14359.65</v>
+        <v>13053.28</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>34896.35</v>
+        <v>36202.72</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.2915309809972389</v>
+        <v>0.2650089329218775</v>
       </c>
     </row>
     <row r="14">
@@ -5951,13 +5951,13 @@
         <v>82482.82000000001</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>23707.95</v>
+        <v>22401.58</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>58774.87</v>
+        <v>60081.24</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.2874289458095637</v>
+        <v>0.2715908597693435</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-02-10 17:30:21
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -3208,7 +3208,7 @@
         <v>0</v>
       </c>
       <c r="M45" s="2" t="n">
-        <v>0</v>
+        <v>65.8</v>
       </c>
       <c r="N45" s="2" t="n">
         <v>0</v>
@@ -3879,7 +3879,7 @@
       </c>
       <c r="M56" s="4" t="inlineStr">
         <is>
-          <t>9 de 54</t>
+          <t>10 de 54</t>
         </is>
       </c>
       <c r="N56" s="4" t="inlineStr">
@@ -5150,7 +5150,7 @@
         <v>0</v>
       </c>
       <c r="F45" s="2" t="n">
-        <v>0</v>
+        <v>65.8</v>
       </c>
       <c r="G45" s="2" t="n">
         <v>300</v>
@@ -5545,7 +5545,7 @@
         <v>79907.13</v>
       </c>
       <c r="F60" s="5" t="n">
-        <v>23650.98</v>
+        <v>23716.78</v>
       </c>
       <c r="G60" s="5" t="n">
         <v>115950</v>
@@ -5884,13 +5884,13 @@
         <v>49256</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>13053.28</v>
+        <v>13119.08</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>36202.72</v>
+        <v>36136.92</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.2650089329218775</v>
+        <v>0.266344810784473</v>
       </c>
     </row>
     <row r="14">
@@ -5951,13 +5951,13 @@
         <v>82482.82000000001</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>22401.58</v>
+        <v>22467.38</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>60081.24</v>
+        <v>60015.44</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.2715908597693435</v>
+        <v>0.2723886016506225</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-02-11 08:30:21
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -2188,7 +2188,7 @@
         <v>0</v>
       </c>
       <c r="M28" s="2" t="n">
-        <v>0</v>
+        <v>65.8</v>
       </c>
       <c r="N28" s="2" t="n">
         <v>0</v>
@@ -3879,7 +3879,7 @@
       </c>
       <c r="M56" s="4" t="inlineStr">
         <is>
-          <t>10 de 54</t>
+          <t>11 de 54</t>
         </is>
       </c>
       <c r="N56" s="4" t="inlineStr">
@@ -4691,7 +4691,7 @@
         <v>1342.12</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>0</v>
+        <v>65.8</v>
       </c>
       <c r="G28" s="2" t="n">
         <v>1500</v>
@@ -5545,7 +5545,7 @@
         <v>79907.13</v>
       </c>
       <c r="F60" s="5" t="n">
-        <v>23716.78</v>
+        <v>23782.58</v>
       </c>
       <c r="G60" s="5" t="n">
         <v>115950</v>
@@ -5884,13 +5884,13 @@
         <v>49256</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>13119.08</v>
+        <v>13184.88</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>36136.92</v>
+        <v>36071.12</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.266344810784473</v>
+        <v>0.2676806886470683</v>
       </c>
     </row>
     <row r="14">
@@ -5951,13 +5951,13 @@
         <v>82482.82000000001</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>22467.38</v>
+        <v>22533.18</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>60015.44</v>
+        <v>59949.64</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.2723886016506225</v>
+        <v>0.2731863435319015</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-02-11 15:30:20
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -1108,7 +1108,7 @@
         <v>0</v>
       </c>
       <c r="M10" s="2" t="n">
-        <v>0</v>
+        <v>37.51</v>
       </c>
       <c r="N10" s="2" t="n">
         <v>0</v>
@@ -1708,7 +1708,7 @@
         <v>0</v>
       </c>
       <c r="M20" s="2" t="n">
-        <v>0</v>
+        <v>37.51</v>
       </c>
       <c r="N20" s="2" t="n">
         <v>0</v>
@@ -3628,7 +3628,7 @@
         <v>0</v>
       </c>
       <c r="M52" s="2" t="n">
-        <v>0</v>
+        <v>1111.96</v>
       </c>
       <c r="N52" s="2" t="n">
         <v>0</v>
@@ -3637,7 +3637,7 @@
         <v>0</v>
       </c>
       <c r="P52" s="2" t="n">
-        <v>0</v>
+        <v>491.17</v>
       </c>
       <c r="Q52" s="2" t="n">
         <v>0</v>
@@ -3879,7 +3879,7 @@
       </c>
       <c r="M56" s="4" t="inlineStr">
         <is>
-          <t>11 de 54</t>
+          <t>14 de 54</t>
         </is>
       </c>
       <c r="N56" s="4" t="inlineStr">
@@ -3894,7 +3894,7 @@
       </c>
       <c r="P56" s="4" t="inlineStr">
         <is>
-          <t>1 de 54</t>
+          <t>2 de 54</t>
         </is>
       </c>
       <c r="Q56" s="4" t="inlineStr">
@@ -4205,7 +4205,7 @@
         <v>0</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>0</v>
+        <v>37.51</v>
       </c>
       <c r="G10" s="2" t="n">
         <v>1000</v>
@@ -4475,7 +4475,7 @@
         <v>0</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>0</v>
+        <v>37.51</v>
       </c>
       <c r="G20" s="2" t="n">
         <v>500</v>
@@ -5366,7 +5366,7 @@
         <v>105.62</v>
       </c>
       <c r="F53" s="2" t="n">
-        <v>0</v>
+        <v>1603.13</v>
       </c>
       <c r="G53" s="2" t="n">
         <v>1500</v>
@@ -5393,7 +5393,7 @@
         <v>105.62</v>
       </c>
       <c r="F54" s="2" t="n">
-        <v>0</v>
+        <v>1603.13</v>
       </c>
       <c r="G54" s="2" t="n">
         <v>1650</v>
@@ -5545,7 +5545,7 @@
         <v>79907.13</v>
       </c>
       <c r="F60" s="5" t="n">
-        <v>23748.88</v>
+        <v>27030.16</v>
       </c>
       <c r="G60" s="5" t="n">
         <v>115950</v>
@@ -5764,13 +5764,13 @@
         <v>250</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>724.52</v>
+        <v>1215.69</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>-474.52</v>
+        <v>-965.6900000000001</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>2.89808</v>
+        <v>4.862760000000001</v>
       </c>
     </row>
     <row r="9">
@@ -5884,13 +5884,13 @@
         <v>49256</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>13151.18</v>
+        <v>14338.16</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>36104.82</v>
+        <v>34917.84</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.2669965080396297</v>
+        <v>0.2910946889719019</v>
       </c>
     </row>
     <row r="14">
@@ -5951,13 +5951,13 @@
         <v>82482.82000000001</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>22499.48</v>
+        <v>24177.63</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>59983.34</v>
+        <v>58305.19</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.272777773601824</v>
+        <v>0.2931232225086388</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-02-12 17:30:19
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -748,7 +748,7 @@
         <v>0</v>
       </c>
       <c r="M4" s="2" t="n">
-        <v>402.76</v>
+        <v>512.92</v>
       </c>
       <c r="N4" s="2" t="n">
         <v>0</v>
@@ -1288,7 +1288,7 @@
         <v>0</v>
       </c>
       <c r="M13" s="2" t="n">
-        <v>-1617.41</v>
+        <v>-1721.09</v>
       </c>
       <c r="N13" s="2" t="n">
         <v>0</v>
@@ -2728,7 +2728,7 @@
         <v>0</v>
       </c>
       <c r="M37" s="2" t="n">
-        <v>0</v>
+        <v>529.92</v>
       </c>
       <c r="N37" s="2" t="n">
         <v>0</v>
@@ -3879,7 +3879,7 @@
       </c>
       <c r="M56" s="4" t="inlineStr">
         <is>
-          <t>14 de 54</t>
+          <t>15 de 54</t>
         </is>
       </c>
       <c r="N56" s="4" t="inlineStr">
@@ -4043,7 +4043,7 @@
         <v>689.65</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>652.87</v>
+        <v>763.03</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>15000</v>
@@ -4286,7 +4286,7 @@
         <v>-1064.83</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>-1617.41</v>
+        <v>-1721.09</v>
       </c>
       <c r="G13" s="2" t="n">
         <v>6000</v>
@@ -4718,7 +4718,7 @@
         <v>6962.69</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>0</v>
+        <v>26.1</v>
       </c>
       <c r="G29" s="2" t="n">
         <v>6000</v>
@@ -4934,7 +4934,7 @@
         <v>7485.63</v>
       </c>
       <c r="F37" s="2" t="n">
-        <v>0</v>
+        <v>529.92</v>
       </c>
       <c r="G37" s="2" t="n">
         <v>8000</v>
@@ -5545,7 +5545,7 @@
         <v>79907.13</v>
       </c>
       <c r="F60" s="5" t="n">
-        <v>27030.16</v>
+        <v>27592.66</v>
       </c>
       <c r="G60" s="5" t="n">
         <v>115950</v>
@@ -5836,13 +5836,13 @@
         <v>550</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>0</v>
+        <v>26.1</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>550</v>
+        <v>523.9</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>0</v>
+        <v>0.04745454545454546</v>
       </c>
     </row>
     <row r="12">
@@ -5884,13 +5884,13 @@
         <v>49256</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>14338.16</v>
+        <v>14874.56</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>34917.84</v>
+        <v>34381.44</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.2910946889719019</v>
+        <v>0.3019847328244274</v>
       </c>
     </row>
     <row r="14">
@@ -5951,13 +5951,13 @@
         <v>82482.82000000001</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>24177.63</v>
+        <v>24740.13</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>58305.19</v>
+        <v>57742.69</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.2931232225086388</v>
+        <v>0.2999428244572627</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-02-18 09:30:21
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -2728,7 +2728,7 @@
         <v>0</v>
       </c>
       <c r="M37" s="2" t="n">
-        <v>529.92</v>
+        <v>513.0700000000001</v>
       </c>
       <c r="N37" s="2" t="n">
         <v>0</v>
@@ -4934,7 +4934,7 @@
         <v>7485.63</v>
       </c>
       <c r="F37" s="2" t="n">
-        <v>529.92</v>
+        <v>513.0700000000001</v>
       </c>
       <c r="G37" s="2" t="n">
         <v>8000</v>
@@ -5545,7 +5545,7 @@
         <v>79907.13</v>
       </c>
       <c r="F60" s="5" t="n">
-        <v>27592.66</v>
+        <v>27575.81</v>
       </c>
       <c r="G60" s="5" t="n">
         <v>115950</v>
@@ -5884,13 +5884,13 @@
         <v>49256</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>14874.56</v>
+        <v>14857.71</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>34381.44</v>
+        <v>34398.29</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.3019847328244274</v>
+        <v>0.3016426425207081</v>
       </c>
     </row>
     <row r="14">
@@ -5951,13 +5951,13 @@
         <v>82482.82000000001</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>24740.13</v>
+        <v>24723.28</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>57742.69</v>
+        <v>57759.54</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.2999428244572627</v>
+        <v>0.2997385394922239</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-02-18 17:30:21
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -781,7 +781,7 @@
         <v>388.8</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>534.24</v>
+        <v>2914.1</v>
       </c>
       <c r="E5" s="2" t="n">
         <v>0</v>
@@ -1921,7 +1921,7 @@
         <v>0</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>0</v>
+        <v>381.6</v>
       </c>
       <c r="E24" s="2" t="n">
         <v>0</v>
@@ -1936,7 +1936,7 @@
         <v>205.2</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>118.8</v>
+        <v>275.4</v>
       </c>
       <c r="J24" s="2" t="n">
         <v>0</v>
@@ -1948,7 +1948,7 @@
         <v>0</v>
       </c>
       <c r="M24" s="2" t="n">
-        <v>5203.44</v>
+        <v>5209.15</v>
       </c>
       <c r="N24" s="2" t="n">
         <v>0</v>
@@ -2248,7 +2248,7 @@
         <v>0</v>
       </c>
       <c r="M29" s="2" t="n">
-        <v>0</v>
+        <v>231.34</v>
       </c>
       <c r="N29" s="2" t="n">
         <v>0</v>
@@ -2668,7 +2668,7 @@
         <v>3977.71</v>
       </c>
       <c r="M36" s="2" t="n">
-        <v>0</v>
+        <v>10552.61</v>
       </c>
       <c r="N36" s="2" t="n">
         <v>0</v>
@@ -3834,7 +3834,7 @@
       </c>
       <c r="D56" s="4" t="inlineStr">
         <is>
-          <t>3 de 54</t>
+          <t>4 de 54</t>
         </is>
       </c>
       <c r="E56" s="4" t="inlineStr">
@@ -3879,7 +3879,7 @@
       </c>
       <c r="M56" s="4" t="inlineStr">
         <is>
-          <t>15 de 54</t>
+          <t>17 de 54</t>
         </is>
       </c>
       <c r="N56" s="4" t="inlineStr">
@@ -4070,7 +4070,7 @@
         <v>10936.72</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>1176.48</v>
+        <v>3556.34</v>
       </c>
       <c r="G5" s="2" t="n">
         <v>10000</v>
@@ -4583,7 +4583,7 @@
         <v>3774.95</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>5679.72</v>
+        <v>6223.63</v>
       </c>
       <c r="G24" s="2" t="n">
         <v>15000</v>
@@ -4718,7 +4718,7 @@
         <v>6962.69</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>26.1</v>
+        <v>257.44</v>
       </c>
       <c r="G29" s="2" t="n">
         <v>6000</v>
@@ -4907,7 +4907,7 @@
         <v>9478.459999999999</v>
       </c>
       <c r="F36" s="2" t="n">
-        <v>3977.71</v>
+        <v>14530.32</v>
       </c>
       <c r="G36" s="2" t="n">
         <v>10000</v>
@@ -5545,7 +5545,7 @@
         <v>79907.13</v>
       </c>
       <c r="F60" s="5" t="n">
-        <v>27575.81</v>
+        <v>41283.53</v>
       </c>
       <c r="G60" s="5" t="n">
         <v>115950</v>
@@ -5569,7 +5569,7 @@
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="23" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
     <col width="25" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -5644,13 +5644,13 @@
         <v>8826</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>3277.44</v>
+        <v>6038.9</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>5548.559999999999</v>
+        <v>2787.1</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>0.3713392250169952</v>
+        <v>0.6842170858826195</v>
       </c>
     </row>
     <row r="4">
@@ -5740,13 +5740,13 @@
         <v>974.4</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>118.8</v>
+        <v>275.4</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>855.6</v>
+        <v>699</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>0.1219211822660099</v>
+        <v>0.2826354679802955</v>
       </c>
     </row>
     <row r="8">
@@ -5884,13 +5884,13 @@
         <v>49256</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>14857.71</v>
+        <v>25647.37</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>34398.29</v>
+        <v>23608.63</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.3016426425207081</v>
+        <v>0.5206953467597856</v>
       </c>
     </row>
     <row r="14">
@@ -5951,13 +5951,13 @@
         <v>82482.82000000001</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>24723.28</v>
+        <v>38431</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>57759.54</v>
+        <v>44051.82</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.2997385394922239</v>
+        <v>0.465927328866787</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-02-19 09:30:23
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -1468,7 +1468,7 @@
         <v>0</v>
       </c>
       <c r="M16" s="2" t="n">
-        <v>3079.58</v>
+        <v>8559.67</v>
       </c>
       <c r="N16" s="2" t="n">
         <v>0</v>
@@ -2668,7 +2668,7 @@
         <v>3977.71</v>
       </c>
       <c r="M36" s="2" t="n">
-        <v>10552.61</v>
+        <v>18648.64</v>
       </c>
       <c r="N36" s="2" t="n">
         <v>0</v>
@@ -4367,7 +4367,7 @@
         <v>2994.81</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>4267.58</v>
+        <v>9747.67</v>
       </c>
       <c r="G16" s="2" t="n">
         <v>6000</v>
@@ -4907,7 +4907,7 @@
         <v>9478.459999999999</v>
       </c>
       <c r="F36" s="2" t="n">
-        <v>14530.32</v>
+        <v>22626.35</v>
       </c>
       <c r="G36" s="2" t="n">
         <v>10000</v>
@@ -5545,7 +5545,7 @@
         <v>79907.13</v>
       </c>
       <c r="F60" s="5" t="n">
-        <v>41283.53</v>
+        <v>54859.65</v>
       </c>
       <c r="G60" s="5" t="n">
         <v>115950</v>
@@ -5884,13 +5884,13 @@
         <v>49256</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>25647.37</v>
+        <v>39223.49</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>23608.63</v>
+        <v>10032.51</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.5206953467597856</v>
+        <v>0.7963190271235991</v>
       </c>
     </row>
     <row r="14">
@@ -5951,13 +5951,13 @@
         <v>82482.82000000001</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>38431</v>
+        <v>52007.12</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>44051.82</v>
+        <v>30475.7</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.465927328866787</v>
+        <v>0.6305206344787919</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-02-19 14:30:22
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -1948,7 +1948,7 @@
         <v>0</v>
       </c>
       <c r="M24" s="2" t="n">
-        <v>5209.15</v>
+        <v>5714.1</v>
       </c>
       <c r="N24" s="2" t="n">
         <v>0</v>
@@ -3628,7 +3628,7 @@
         <v>0</v>
       </c>
       <c r="M52" s="2" t="n">
-        <v>1111.96</v>
+        <v>1883.08</v>
       </c>
       <c r="N52" s="2" t="n">
         <v>0</v>
@@ -4583,7 +4583,7 @@
         <v>3774.95</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>6223.63</v>
+        <v>6728.58</v>
       </c>
       <c r="G24" s="2" t="n">
         <v>15000</v>
@@ -5366,7 +5366,7 @@
         <v>105.62</v>
       </c>
       <c r="F53" s="2" t="n">
-        <v>1603.13</v>
+        <v>2374.25</v>
       </c>
       <c r="G53" s="2" t="n">
         <v>1500</v>
@@ -5393,7 +5393,7 @@
         <v>105.62</v>
       </c>
       <c r="F54" s="2" t="n">
-        <v>1603.13</v>
+        <v>2374.25</v>
       </c>
       <c r="G54" s="2" t="n">
         <v>1650</v>
@@ -5545,7 +5545,7 @@
         <v>79907.13</v>
       </c>
       <c r="F60" s="5" t="n">
-        <v>53926.53</v>
+        <v>55973.72</v>
       </c>
       <c r="G60" s="5" t="n">
         <v>115950</v>
@@ -5569,7 +5569,7 @@
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="5" max="5"/>
     <col width="25" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -5884,13 +5884,13 @@
         <v>49256</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>38290.37</v>
+        <v>39566.44</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>10965.63</v>
+        <v>9689.559999999998</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.7773747360727628</v>
+        <v>0.8032816306642846</v>
       </c>
     </row>
     <row r="14">
@@ -5951,13 +5951,13 @@
         <v>82482.82000000001</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>51074</v>
+        <v>52350.07</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>31408.82</v>
+        <v>30132.75</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.6192077331982587</v>
+        <v>0.6346784700135131</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-02-24 17:30:23
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -1033,10 +1033,10 @@
         <v>0</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>0</v>
+        <v>615.6</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>0</v>
+        <v>156.6</v>
       </c>
       <c r="J9" s="2" t="n">
         <v>0</v>
@@ -1228,7 +1228,7 @@
         <v>0</v>
       </c>
       <c r="M12" s="2" t="n">
-        <v>0</v>
+        <v>1836.35</v>
       </c>
       <c r="N12" s="2" t="n">
         <v>0</v>
@@ -1888,7 +1888,7 @@
         <v>0</v>
       </c>
       <c r="M23" s="2" t="n">
-        <v>-33.7</v>
+        <v>-0.25</v>
       </c>
       <c r="N23" s="2" t="n">
         <v>0</v>
@@ -1948,7 +1948,7 @@
         <v>0</v>
       </c>
       <c r="M24" s="2" t="n">
-        <v>5714.1</v>
+        <v>5741.39</v>
       </c>
       <c r="N24" s="2" t="n">
         <v>0</v>
@@ -2662,10 +2662,10 @@
         <v>0</v>
       </c>
       <c r="K36" s="2" t="n">
-        <v>0</v>
+        <v>406.08</v>
       </c>
       <c r="L36" s="2" t="n">
-        <v>3977.71</v>
+        <v>5390.83</v>
       </c>
       <c r="M36" s="2" t="n">
         <v>18648.64</v>
@@ -3854,14 +3854,14 @@
       </c>
       <c r="H56" s="4" t="inlineStr">
         <is>
+          <t>3 de 54</t>
+        </is>
+      </c>
+      <c r="I56" s="4" t="inlineStr">
+        <is>
           <t>2 de 54</t>
         </is>
       </c>
-      <c r="I56" s="4" t="inlineStr">
-        <is>
-          <t>1 de 54</t>
-        </is>
-      </c>
       <c r="J56" s="4" t="inlineStr">
         <is>
           <t>0 de 54</t>
@@ -3869,7 +3869,7 @@
       </c>
       <c r="K56" s="4" t="inlineStr">
         <is>
-          <t>1 de 54</t>
+          <t>2 de 54</t>
         </is>
       </c>
       <c r="L56" s="4" t="inlineStr">
@@ -3879,7 +3879,7 @@
       </c>
       <c r="M56" s="4" t="inlineStr">
         <is>
-          <t>16 de 54</t>
+          <t>17 de 54</t>
         </is>
       </c>
       <c r="N56" s="4" t="inlineStr">
@@ -4178,7 +4178,7 @@
         <v>6.12</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>0</v>
+        <v>772.2</v>
       </c>
       <c r="G9" s="2" t="n">
         <v>1500</v>
@@ -4259,7 +4259,7 @@
         <v>3948.01</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>0</v>
+        <v>1836.35</v>
       </c>
       <c r="G12" s="2" t="n">
         <v>3000</v>
@@ -4556,7 +4556,7 @@
         <v>2531.23</v>
       </c>
       <c r="F23" s="2" t="n">
-        <v>-33.7</v>
+        <v>-0.25</v>
       </c>
       <c r="G23" s="2" t="n">
         <v>0</v>
@@ -4583,7 +4583,7 @@
         <v>3774.95</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>6728.58</v>
+        <v>6755.87</v>
       </c>
       <c r="G24" s="2" t="n">
         <v>15000</v>
@@ -4907,7 +4907,7 @@
         <v>9478.459999999999</v>
       </c>
       <c r="F36" s="2" t="n">
-        <v>22626.35</v>
+        <v>24445.55</v>
       </c>
       <c r="G36" s="2" t="n">
         <v>10000</v>
@@ -5545,7 +5545,7 @@
         <v>79907.13</v>
       </c>
       <c r="F60" s="5" t="n">
-        <v>57569.06</v>
+        <v>62057.55</v>
       </c>
       <c r="G60" s="5" t="n">
         <v>115950</v>
@@ -5716,13 +5716,13 @@
         <v>975</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>987.3</v>
+        <v>1602.9</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>-12.29999999999995</v>
+        <v>-627.9000000000001</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>1.012615384615384</v>
+        <v>1.644</v>
       </c>
     </row>
     <row r="7">
@@ -5740,13 +5740,13 @@
         <v>974.4</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>275.4</v>
+        <v>432</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>699</v>
+        <v>542.4</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>0.2826354679802955</v>
+        <v>0.4433497536945813</v>
       </c>
     </row>
     <row r="8">
@@ -5812,13 +5812,13 @@
         <v>2850</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>152.28</v>
+        <v>558.36</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>2697.72</v>
+        <v>2291.64</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>0.05343157894736842</v>
+        <v>0.1959157894736842</v>
       </c>
     </row>
     <row r="11">
@@ -5860,13 +5860,13 @@
         <v>13321</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>4231.15</v>
+        <v>5644.27</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>9089.85</v>
+        <v>7676.73</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0.3176300578034682</v>
+        <v>0.4237121837699873</v>
       </c>
     </row>
     <row r="13">
@@ -5884,13 +5884,13 @@
         <v>49256</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>40250.08</v>
+        <v>42147.17</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>9005.919999999998</v>
+        <v>7108.830000000002</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.8171609550105571</v>
+        <v>0.8556758567484164</v>
       </c>
     </row>
     <row r="14">
@@ -5951,13 +5951,13 @@
         <v>82482.82000000001</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>53945.41</v>
+        <v>58433.9</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>28537.41</v>
+        <v>24048.92</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.6540199522761224</v>
+        <v>0.7084372236545743</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-02-26 12:30:23
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -1948,7 +1948,7 @@
         <v>0</v>
       </c>
       <c r="M24" s="2" t="n">
-        <v>5741.39</v>
+        <v>12413.2</v>
       </c>
       <c r="N24" s="2" t="n">
         <v>0</v>
@@ -4583,7 +4583,7 @@
         <v>3774.95</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>6755.87</v>
+        <v>13427.68</v>
       </c>
       <c r="G24" s="2" t="n">
         <v>15000</v>
@@ -5545,7 +5545,7 @@
         <v>79907.13</v>
       </c>
       <c r="F60" s="5" t="n">
-        <v>62285.21</v>
+        <v>68957.02</v>
       </c>
       <c r="G60" s="5" t="n">
         <v>115950</v>
@@ -5884,13 +5884,13 @@
         <v>49256</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>42216.03</v>
+        <v>48887.84</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>7039.970000000001</v>
+        <v>368.1600000000035</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.8570738590222511</v>
+        <v>0.992525580639922</v>
       </c>
     </row>
     <row r="14">
@@ -5951,13 +5951,13 @@
         <v>82482.82000000001</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>58592.7</v>
+        <v>65264.50999999999</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>23890.12</v>
+        <v>17218.31</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.7103624730580258</v>
+        <v>0.7912497414613127</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-02-26 15:30:20
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -745,10 +745,10 @@
         <v>0</v>
       </c>
       <c r="L4" s="2" t="n">
-        <v>0</v>
+        <v>89.56</v>
       </c>
       <c r="M4" s="2" t="n">
-        <v>512.92</v>
+        <v>698.9</v>
       </c>
       <c r="N4" s="2" t="n">
         <v>0</v>
@@ -3874,7 +3874,7 @@
       </c>
       <c r="L56" s="4" t="inlineStr">
         <is>
-          <t>2 de 54</t>
+          <t>3 de 54</t>
         </is>
       </c>
       <c r="M56" s="4" t="inlineStr">
@@ -4043,7 +4043,7 @@
         <v>689.65</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>763.03</v>
+        <v>1038.57</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>15000</v>
@@ -5545,7 +5545,7 @@
         <v>79907.13</v>
       </c>
       <c r="F60" s="5" t="n">
-        <v>68957.02</v>
+        <v>69232.56</v>
       </c>
       <c r="G60" s="5" t="n">
         <v>115950</v>
@@ -5860,13 +5860,13 @@
         <v>13321</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>5644.27</v>
+        <v>5733.83</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>7676.73</v>
+        <v>7587.17</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0.4237121837699873</v>
+        <v>0.4304354027475415</v>
       </c>
     </row>
     <row r="13">
@@ -5884,13 +5884,13 @@
         <v>49256</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>48887.84</v>
+        <v>49073.82</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>368.1600000000035</v>
+        <v>182.1800000000003</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.992525580639922</v>
+        <v>0.9963013643007959</v>
       </c>
     </row>
     <row r="14">
@@ -5951,13 +5951,13 @@
         <v>82482.82000000001</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>65264.50999999999</v>
+        <v>65540.05</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>17218.31</v>
+        <v>16942.77</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.7912497414613127</v>
+        <v>0.7945903158985107</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-02-27 12:30:23
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -748,7 +748,7 @@
         <v>89.56</v>
       </c>
       <c r="M4" s="2" t="n">
-        <v>698.9</v>
+        <v>1073.44</v>
       </c>
       <c r="N4" s="2" t="n">
         <v>0</v>
@@ -805,7 +805,7 @@
         <v>0</v>
       </c>
       <c r="L5" s="2" t="n">
-        <v>253.44</v>
+        <v>810.25</v>
       </c>
       <c r="M5" s="2" t="n">
         <v>0</v>
@@ -1444,7 +1444,7 @@
         <v>1188</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>0</v>
+        <v>568.79</v>
       </c>
       <c r="F16" s="2" t="n">
         <v>0</v>
@@ -2701,7 +2701,7 @@
         <v>0</v>
       </c>
       <c r="D37" s="2" t="n">
-        <v>158.4</v>
+        <v>554.4</v>
       </c>
       <c r="E37" s="2" t="n">
         <v>0</v>
@@ -3688,7 +3688,7 @@
         <v>0</v>
       </c>
       <c r="M53" s="2" t="n">
-        <v>593.74</v>
+        <v>1165.28</v>
       </c>
       <c r="N53" s="2" t="n">
         <v>0</v>
@@ -3839,7 +3839,7 @@
       </c>
       <c r="E56" s="4" t="inlineStr">
         <is>
-          <t>1 de 54</t>
+          <t>2 de 54</t>
         </is>
       </c>
       <c r="F56" s="4" t="inlineStr">
@@ -4043,7 +4043,7 @@
         <v>689.65</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>1038.57</v>
+        <v>1413.11</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>15000</v>
@@ -4070,7 +4070,7 @@
         <v>10936.72</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>3556.34</v>
+        <v>4113.15</v>
       </c>
       <c r="G5" s="2" t="n">
         <v>10000</v>
@@ -4367,7 +4367,7 @@
         <v>2994.81</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>10555.7</v>
+        <v>11124.49</v>
       </c>
       <c r="G16" s="2" t="n">
         <v>6000</v>
@@ -4934,7 +4934,7 @@
         <v>7485.63</v>
       </c>
       <c r="F37" s="2" t="n">
-        <v>671.47</v>
+        <v>1067.47</v>
       </c>
       <c r="G37" s="2" t="n">
         <v>8000</v>
@@ -5420,7 +5420,7 @@
         <v>336.6</v>
       </c>
       <c r="F55" s="2" t="n">
-        <v>1318.26</v>
+        <v>1889.8</v>
       </c>
       <c r="G55" s="2" t="n">
         <v>500</v>
@@ -5447,7 +5447,7 @@
         <v>336.6</v>
       </c>
       <c r="F56" s="2" t="n">
-        <v>1318.26</v>
+        <v>1889.8</v>
       </c>
       <c r="G56" s="2" t="n">
         <v>1000</v>
@@ -5545,7 +5545,7 @@
         <v>79907.13</v>
       </c>
       <c r="F60" s="5" t="n">
-        <v>69390.96000000001</v>
+        <v>72430.17999999999</v>
       </c>
       <c r="G60" s="5" t="n">
         <v>115950</v>
@@ -5568,7 +5568,7 @@
     <col width="32" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="25" customWidth="1" min="6" max="6"/>
   </cols>
@@ -5644,13 +5644,13 @@
         <v>8826</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>6197.3</v>
+        <v>6593.3</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>2628.7</v>
+        <v>2232.7</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>0.7021640607296624</v>
+        <v>0.7470314978472694</v>
       </c>
     </row>
     <row r="4">
@@ -5668,13 +5668,13 @@
         <v>369.6</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>250.11</v>
+        <v>818.9</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>119.49</v>
+        <v>-449.3</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>0.6767045454545455</v>
+        <v>2.215638528138528</v>
       </c>
     </row>
     <row r="5">
@@ -5860,13 +5860,13 @@
         <v>13321</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>5733.83</v>
+        <v>6290.64</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>7587.17</v>
+        <v>7030.36</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0.4304354027475415</v>
+        <v>0.4722348172059155</v>
       </c>
     </row>
     <row r="13">
@@ -5884,13 +5884,13 @@
         <v>49256</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>49073.82</v>
+        <v>50019.9</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>182.1800000000003</v>
+        <v>-763.9000000000015</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.9963013643007959</v>
+        <v>1.015508770505116</v>
       </c>
     </row>
     <row r="14">
@@ -5951,13 +5951,13 @@
         <v>82482.82000000001</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>65698.45</v>
+        <v>68166.13</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>16784.37</v>
+        <v>14316.69</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.7965107158072432</v>
+        <v>0.8264282186278306</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-03-04 15:30:27
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -748,7 +748,7 @@
         <v>0</v>
       </c>
       <c r="M4" s="2" t="n">
-        <v>0</v>
+        <v>345.38</v>
       </c>
       <c r="N4" s="2" t="n">
         <v>0</v>
@@ -3879,7 +3879,7 @@
       </c>
       <c r="M56" s="4" t="inlineStr">
         <is>
-          <t>5 de 54</t>
+          <t>6 de 54</t>
         </is>
       </c>
       <c r="N56" s="4" t="inlineStr">
@@ -4043,7 +4043,7 @@
         <v>1611.4</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>0</v>
+        <v>345.38</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>15000</v>
@@ -5545,7 +5545,7 @@
         <v>76363.98</v>
       </c>
       <c r="F60" s="5" t="n">
-        <v>2516.63</v>
+        <v>2862.01</v>
       </c>
       <c r="G60" s="5" t="n">
         <v>115950</v>
@@ -5884,13 +5884,13 @@
         <v>65052</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>821.9</v>
+        <v>1167.28</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>64230.1</v>
+        <v>63884.72</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.01263450777839267</v>
+        <v>0.01794379880710816</v>
       </c>
     </row>
     <row r="14">
@@ -5927,13 +5927,13 @@
         <v>82783.32000000001</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>2411.66</v>
+        <v>2757.04</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>80371.66</v>
+        <v>80026.28</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.02913219716242354</v>
+        <v>0.03330429366688845</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-03-05 17:30:24
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -3688,7 +3688,7 @@
         <v>0</v>
       </c>
       <c r="M53" s="2" t="n">
-        <v>104.97</v>
+        <v>864.6900000000001</v>
       </c>
       <c r="N53" s="2" t="n">
         <v>0</v>
@@ -5420,7 +5420,7 @@
         <v>1915.78</v>
       </c>
       <c r="F55" s="2" t="n">
-        <v>104.97</v>
+        <v>864.6900000000001</v>
       </c>
       <c r="G55" s="2" t="n">
         <v>500</v>
@@ -5447,7 +5447,7 @@
         <v>1915.78</v>
       </c>
       <c r="F56" s="2" t="n">
-        <v>104.97</v>
+        <v>864.6900000000001</v>
       </c>
       <c r="G56" s="2" t="n">
         <v>1000</v>
@@ -5545,7 +5545,7 @@
         <v>76363.98</v>
       </c>
       <c r="F60" s="5" t="n">
-        <v>2862.01</v>
+        <v>4381.45</v>
       </c>
       <c r="G60" s="5" t="n">
         <v>115950</v>
@@ -5884,13 +5884,13 @@
         <v>65052</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>1167.28</v>
+        <v>1927</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>63884.72</v>
+        <v>63125</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.01794379880710816</v>
+        <v>0.02962245588144869</v>
       </c>
     </row>
     <row r="14">
@@ -5927,13 +5927,13 @@
         <v>82783.32000000001</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>2757.04</v>
+        <v>3516.76</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>80026.28</v>
+        <v>79266.56</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.03330429366688845</v>
+        <v>0.04248150472824719</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-03-06 09:30:20
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -3208,7 +3208,7 @@
         <v>0</v>
       </c>
       <c r="M45" s="2" t="n">
-        <v>0</v>
+        <v>821.0599999999999</v>
       </c>
       <c r="N45" s="2" t="n">
         <v>0</v>
@@ -3879,7 +3879,7 @@
       </c>
       <c r="M56" s="4" t="inlineStr">
         <is>
-          <t>6 de 54</t>
+          <t>7 de 54</t>
         </is>
       </c>
       <c r="N56" s="4" t="inlineStr">
@@ -5150,7 +5150,7 @@
         <v>65.8</v>
       </c>
       <c r="F45" s="2" t="n">
-        <v>0</v>
+        <v>821.0599999999999</v>
       </c>
       <c r="G45" s="2" t="n">
         <v>300</v>
@@ -5545,7 +5545,7 @@
         <v>76363.98</v>
       </c>
       <c r="F60" s="5" t="n">
-        <v>5418.59</v>
+        <v>6239.65</v>
       </c>
       <c r="G60" s="5" t="n">
         <v>115950</v>
@@ -5884,13 +5884,13 @@
         <v>65052</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>2123.73</v>
+        <v>2944.79</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>62928.27</v>
+        <v>62107.21</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.03264665190924184</v>
+        <v>0.04526824694090881</v>
       </c>
     </row>
     <row r="14">
@@ -5927,13 +5927,13 @@
         <v>82783.32000000001</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>4357.17</v>
+        <v>5178.23</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>78426.14999999999</v>
+        <v>77605.09</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.0526334290530991</v>
+        <v>0.0625516106384716</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-03-10 11:30:23
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -721,7 +721,7 @@
         <v>0</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>0</v>
+        <v>95.04000000000001</v>
       </c>
       <c r="E4" s="2" t="n">
         <v>0</v>
@@ -3834,7 +3834,7 @@
       </c>
       <c r="D56" s="4" t="inlineStr">
         <is>
-          <t>4 de 54</t>
+          <t>5 de 54</t>
         </is>
       </c>
       <c r="E56" s="4" t="inlineStr">
@@ -4043,7 +4043,7 @@
         <v>1611.4</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>345.38</v>
+        <v>440.42</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>15000</v>
@@ -5545,7 +5545,7 @@
         <v>76363.98</v>
       </c>
       <c r="F60" s="5" t="n">
-        <v>6137.93</v>
+        <v>6232.97</v>
       </c>
       <c r="G60" s="5" t="n">
         <v>115950</v>
@@ -5644,13 +5644,13 @@
         <v>6600</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>1558.08</v>
+        <v>1653.12</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>5041.92</v>
+        <v>4946.88</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>0.2360727272727273</v>
+        <v>0.2504727272727272</v>
       </c>
     </row>
     <row r="4">
@@ -5927,13 +5927,13 @@
         <v>82783.32000000001</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>5117.33</v>
+        <v>5212.37</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>77665.98999999999</v>
+        <v>77570.95</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.06181595519483876</v>
+        <v>0.06296401255711899</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-03-11 08:30:19
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -1948,7 +1948,7 @@
         <v>506.88</v>
       </c>
       <c r="M24" s="2" t="n">
-        <v>415.76</v>
+        <v>398.91</v>
       </c>
       <c r="N24" s="2" t="n">
         <v>0</v>
@@ -4583,7 +4583,7 @@
         <v>13411.91</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>1304.24</v>
+        <v>1287.39</v>
       </c>
       <c r="G24" s="2" t="n">
         <v>15000</v>
@@ -5545,7 +5545,7 @@
         <v>76363.98</v>
       </c>
       <c r="F60" s="5" t="n">
-        <v>12627.72</v>
+        <v>12610.87</v>
       </c>
       <c r="G60" s="5" t="n">
         <v>115950</v>
@@ -5884,13 +5884,13 @@
         <v>65052</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>4080.43</v>
+        <v>4063.58</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>60971.57</v>
+        <v>60988.42</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.06272566562134907</v>
+        <v>0.06246664207095862</v>
       </c>
     </row>
     <row r="14">
@@ -5927,13 +5927,13 @@
         <v>82783.32000000001</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>11607.12</v>
+        <v>11590.27</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>71176.2</v>
+        <v>71193.05</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.1402108540706026</v>
+        <v>0.1400073106514694</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-03-12 17:31:01
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -901,7 +901,7 @@
         <v>0</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>0</v>
+        <v>79.2</v>
       </c>
       <c r="E7" s="2" t="n">
         <v>0</v>
@@ -1948,7 +1948,7 @@
         <v>506.88</v>
       </c>
       <c r="M24" s="2" t="n">
-        <v>398.91</v>
+        <v>441.68</v>
       </c>
       <c r="N24" s="2" t="n">
         <v>0</v>
@@ -2665,10 +2665,10 @@
         <v>0</v>
       </c>
       <c r="L36" s="2" t="n">
-        <v>0</v>
+        <v>317.95</v>
       </c>
       <c r="M36" s="2" t="n">
-        <v>0</v>
+        <v>120.46</v>
       </c>
       <c r="N36" s="2" t="n">
         <v>0</v>
@@ -2725,7 +2725,7 @@
         <v>0</v>
       </c>
       <c r="L37" s="2" t="n">
-        <v>0</v>
+        <v>565.25</v>
       </c>
       <c r="M37" s="2" t="n">
         <v>0</v>
@@ -3834,52 +3834,52 @@
       </c>
       <c r="D56" s="4" t="inlineStr">
         <is>
+          <t>6 de 54</t>
+        </is>
+      </c>
+      <c r="E56" s="4" t="inlineStr">
+        <is>
+          <t>0 de 54</t>
+        </is>
+      </c>
+      <c r="F56" s="4" t="inlineStr">
+        <is>
+          <t>0 de 54</t>
+        </is>
+      </c>
+      <c r="G56" s="4" t="inlineStr">
+        <is>
+          <t>0 de 54</t>
+        </is>
+      </c>
+      <c r="H56" s="4" t="inlineStr">
+        <is>
+          <t>1 de 54</t>
+        </is>
+      </c>
+      <c r="I56" s="4" t="inlineStr">
+        <is>
+          <t>1 de 54</t>
+        </is>
+      </c>
+      <c r="J56" s="4" t="inlineStr">
+        <is>
+          <t>0 de 54</t>
+        </is>
+      </c>
+      <c r="K56" s="4" t="inlineStr">
+        <is>
+          <t>0 de 54</t>
+        </is>
+      </c>
+      <c r="L56" s="4" t="inlineStr">
+        <is>
           <t>5 de 54</t>
         </is>
       </c>
-      <c r="E56" s="4" t="inlineStr">
-        <is>
-          <t>0 de 54</t>
-        </is>
-      </c>
-      <c r="F56" s="4" t="inlineStr">
-        <is>
-          <t>0 de 54</t>
-        </is>
-      </c>
-      <c r="G56" s="4" t="inlineStr">
-        <is>
-          <t>0 de 54</t>
-        </is>
-      </c>
-      <c r="H56" s="4" t="inlineStr">
-        <is>
-          <t>1 de 54</t>
-        </is>
-      </c>
-      <c r="I56" s="4" t="inlineStr">
-        <is>
-          <t>1 de 54</t>
-        </is>
-      </c>
-      <c r="J56" s="4" t="inlineStr">
-        <is>
-          <t>0 de 54</t>
-        </is>
-      </c>
-      <c r="K56" s="4" t="inlineStr">
-        <is>
-          <t>0 de 54</t>
-        </is>
-      </c>
-      <c r="L56" s="4" t="inlineStr">
-        <is>
-          <t>3 de 54</t>
-        </is>
-      </c>
       <c r="M56" s="4" t="inlineStr">
         <is>
-          <t>7 de 54</t>
+          <t>8 de 54</t>
         </is>
       </c>
       <c r="N56" s="4" t="inlineStr">
@@ -4124,7 +4124,7 @@
         <v>2076.19</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>0</v>
+        <v>79.2</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>1500</v>
@@ -4583,7 +4583,7 @@
         <v>13411.91</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>1287.39</v>
+        <v>1330.16</v>
       </c>
       <c r="G24" s="2" t="n">
         <v>15000</v>
@@ -4907,7 +4907,7 @@
         <v>27766.67</v>
       </c>
       <c r="F36" s="2" t="n">
-        <v>-20.08</v>
+        <v>418.33</v>
       </c>
       <c r="G36" s="2" t="n">
         <v>10000</v>
@@ -4934,7 +4934,7 @@
         <v>1067.47</v>
       </c>
       <c r="F37" s="2" t="n">
-        <v>0</v>
+        <v>565.25</v>
       </c>
       <c r="G37" s="2" t="n">
         <v>8000</v>
@@ -5545,7 +5545,7 @@
         <v>76363.98</v>
       </c>
       <c r="F60" s="5" t="n">
-        <v>13079.16</v>
+        <v>14204.79</v>
       </c>
       <c r="G60" s="5" t="n">
         <v>115950</v>
@@ -5644,13 +5644,13 @@
         <v>6600</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>5460.91</v>
+        <v>5540.11</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>1139.09</v>
+        <v>1059.89</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>0.827410606060606</v>
+        <v>0.839410606060606</v>
       </c>
     </row>
     <row r="4">
@@ -5860,13 +5860,13 @@
         <v>7700</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>1722.26</v>
+        <v>2605.46</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>5977.74</v>
+        <v>5094.54</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0.2236701298701299</v>
+        <v>0.3383714285714286</v>
       </c>
     </row>
     <row r="13">
@@ -5884,13 +5884,13 @@
         <v>65052</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>4151.71</v>
+        <v>4314.94</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>60900.29</v>
+        <v>60737.06</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.06382140441492959</v>
+        <v>0.06633062780544795</v>
       </c>
     </row>
     <row r="14">
@@ -5927,13 +5927,13 @@
         <v>82783.32000000001</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>12058.56</v>
+        <v>13184.19</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>70724.75999999999</v>
+        <v>69599.13</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.1456641265414337</v>
+        <v>0.1592614309259401</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-03-13 08:30:20
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -1948,7 +1948,7 @@
         <v>506.88</v>
       </c>
       <c r="M24" s="2" t="n">
-        <v>441.68</v>
+        <v>727.51</v>
       </c>
       <c r="N24" s="2" t="n">
         <v>0</v>
@@ -4583,7 +4583,7 @@
         <v>13411.91</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>1330.16</v>
+        <v>1615.99</v>
       </c>
       <c r="G24" s="2" t="n">
         <v>15000</v>
@@ -5545,7 +5545,7 @@
         <v>76363.98</v>
       </c>
       <c r="F60" s="5" t="n">
-        <v>14204.79</v>
+        <v>14490.62</v>
       </c>
       <c r="G60" s="5" t="n">
         <v>115950</v>
@@ -5884,13 +5884,13 @@
         <v>65052</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>4314.94</v>
+        <v>4600.77</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>60737.06</v>
+        <v>60451.23</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.06633062780544795</v>
+        <v>0.07072449732521675</v>
       </c>
     </row>
     <row r="14">
@@ -5927,13 +5927,13 @@
         <v>82783.32000000001</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>13184.19</v>
+        <v>13470.02</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>69599.13</v>
+        <v>69313.3</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.1592614309259401</v>
+        <v>0.1627141796197591</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-03-13 10:30:23
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -2677,7 +2677,7 @@
         <v>0</v>
       </c>
       <c r="P36" s="2" t="n">
-        <v>-20.08</v>
+        <v>-22.59</v>
       </c>
       <c r="Q36" s="2" t="n">
         <v>0</v>
@@ -4907,7 +4907,7 @@
         <v>27766.67</v>
       </c>
       <c r="F36" s="2" t="n">
-        <v>418.33</v>
+        <v>415.82</v>
       </c>
       <c r="G36" s="2" t="n">
         <v>10000</v>
@@ -5545,7 +5545,7 @@
         <v>76363.98</v>
       </c>
       <c r="F60" s="5" t="n">
-        <v>14490.62</v>
+        <v>14488.11</v>
       </c>
       <c r="G60" s="5" t="n">
         <v>115950</v>
@@ -5764,13 +5764,13 @@
         <v>250</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>316.88</v>
+        <v>314.37</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>-66.88</v>
+        <v>-64.37</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>1.26752</v>
+        <v>1.25748</v>
       </c>
     </row>
     <row r="9">
@@ -5927,13 +5927,13 @@
         <v>82783.32000000001</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>13470.02</v>
+        <v>13467.51</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>69313.3</v>
+        <v>69315.81</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.1627141796197591</v>
+        <v>0.1626838595021316</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-03-17 10:30:19
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -1948,7 +1948,7 @@
         <v>506.88</v>
       </c>
       <c r="M24" s="2" t="n">
-        <v>727.51</v>
+        <v>710.66</v>
       </c>
       <c r="N24" s="2" t="n">
         <v>0</v>
@@ -3361,7 +3361,7 @@
         <v>0</v>
       </c>
       <c r="D48" s="2" t="n">
-        <v>2855.07</v>
+        <v>2787.07</v>
       </c>
       <c r="E48" s="2" t="n">
         <v>0</v>
@@ -4583,7 +4583,7 @@
         <v>13411.91</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>1615.99</v>
+        <v>1599.14</v>
       </c>
       <c r="G24" s="2" t="n">
         <v>15000</v>
@@ -5231,7 +5231,7 @@
         <v>0</v>
       </c>
       <c r="F48" s="2" t="n">
-        <v>2855.07</v>
+        <v>2787.07</v>
       </c>
       <c r="G48" s="2" t="n">
         <v>1500</v>
@@ -5545,7 +5545,7 @@
         <v>76363.98</v>
       </c>
       <c r="F60" s="5" t="n">
-        <v>18376.51</v>
+        <v>18291.66</v>
       </c>
       <c r="G60" s="5" t="n">
         <v>115950</v>
@@ -5570,7 +5570,7 @@
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5644,13 +5644,13 @@
         <v>6600</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>5921.71</v>
+        <v>5853.71</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>678.29</v>
+        <v>746.29</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>0.8972287878787879</v>
+        <v>0.8869257575757575</v>
       </c>
     </row>
     <row r="4">
@@ -5884,13 +5884,13 @@
         <v>65052</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>6096.16</v>
+        <v>6079.31</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>58955.84</v>
+        <v>58972.69</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.0937121072372871</v>
+        <v>0.09345308368689664</v>
       </c>
     </row>
     <row r="14">
@@ -5927,13 +5927,13 @@
         <v>82783.32000000001</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>17355.91</v>
+        <v>17271.06</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>65427.41</v>
+        <v>65512.26</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.2096546743957599</v>
+        <v>0.2086297094632107</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-03-18 16:30:22
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -1948,7 +1948,7 @@
         <v>506.88</v>
       </c>
       <c r="M24" s="2" t="n">
-        <v>710.66</v>
+        <v>1822.63</v>
       </c>
       <c r="N24" s="2" t="n">
         <v>0</v>
@@ -4583,7 +4583,7 @@
         <v>13411.91</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>1599.14</v>
+        <v>2711.11</v>
       </c>
       <c r="G24" s="2" t="n">
         <v>15000</v>
@@ -5545,7 +5545,7 @@
         <v>76363.98</v>
       </c>
       <c r="F60" s="5" t="n">
-        <v>18291.66</v>
+        <v>19403.63</v>
       </c>
       <c r="G60" s="5" t="n">
         <v>115950</v>
@@ -5570,7 +5570,7 @@
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5884,13 +5884,13 @@
         <v>65052</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>6079.31</v>
+        <v>7191.28</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>58972.69</v>
+        <v>57860.72</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.09345308368689664</v>
+        <v>0.1105466396113878</v>
       </c>
     </row>
     <row r="14">
@@ -5927,13 +5927,13 @@
         <v>82783.32000000001</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>17271.06</v>
+        <v>18383.03</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>65512.26</v>
+        <v>64400.29</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.2086297094632107</v>
+        <v>0.2220620047613456</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-03-18 17:30:20
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -2221,7 +2221,7 @@
         <v>0</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>1823.92</v>
+        <v>2775.86</v>
       </c>
       <c r="E29" s="2" t="n">
         <v>0</v>
@@ -2233,7 +2233,7 @@
         <v>0</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>142.2</v>
+        <v>782.1</v>
       </c>
       <c r="I29" s="2" t="n">
         <v>0</v>
@@ -4718,7 +4718,7 @@
         <v>257.44</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>1988.15</v>
+        <v>3579.99</v>
       </c>
       <c r="G29" s="2" t="n">
         <v>6000</v>
@@ -5545,7 +5545,7 @@
         <v>76363.98</v>
       </c>
       <c r="F60" s="5" t="n">
-        <v>19403.63</v>
+        <v>20995.47</v>
       </c>
       <c r="G60" s="5" t="n">
         <v>115950</v>
@@ -5644,13 +5644,13 @@
         <v>6600</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>5853.71</v>
+        <v>6805.65</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>746.29</v>
+        <v>-205.6499999999996</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>0.8869257575757575</v>
+        <v>1.031159090909091</v>
       </c>
     </row>
     <row r="4">
@@ -5716,13 +5716,13 @@
         <v>240</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>927</v>
+        <v>1566.9</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>-687</v>
+        <v>-1326.9</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>3.8625</v>
+        <v>6.52875</v>
       </c>
     </row>
     <row r="7">
@@ -5927,13 +5927,13 @@
         <v>82783.32000000001</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>18383.03</v>
+        <v>19974.87</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>64400.29</v>
+        <v>62808.45</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.2220620047613456</v>
+        <v>0.2412909992012884</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-03-19 10:30:22
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -483,7 +483,7 @@
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
     <col width="25" customWidth="1" min="11" max="11"/>
     <col width="24" customWidth="1" min="12" max="12"/>
     <col width="17" customWidth="1" min="13" max="13"/>
@@ -739,7 +739,7 @@
         <v>0</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>0</v>
+        <v>188.6</v>
       </c>
       <c r="K4" s="2" t="n">
         <v>0</v>
@@ -2662,7 +2662,7 @@
         <v>0</v>
       </c>
       <c r="K36" s="2" t="n">
-        <v>0</v>
+        <v>46.44</v>
       </c>
       <c r="L36" s="2" t="n">
         <v>317.95</v>
@@ -3793,7 +3793,7 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>0</v>
+        <v>295.2</v>
       </c>
       <c r="I55" s="2" t="n">
         <v>0</v>
@@ -3854,7 +3854,7 @@
       </c>
       <c r="H56" s="4" t="inlineStr">
         <is>
-          <t>2 de 54</t>
+          <t>3 de 54</t>
         </is>
       </c>
       <c r="I56" s="4" t="inlineStr">
@@ -3864,12 +3864,12 @@
       </c>
       <c r="J56" s="4" t="inlineStr">
         <is>
-          <t>0 de 54</t>
+          <t>1 de 54</t>
         </is>
       </c>
       <c r="K56" s="4" t="inlineStr">
         <is>
-          <t>0 de 54</t>
+          <t>1 de 54</t>
         </is>
       </c>
       <c r="L56" s="4" t="inlineStr">
@@ -4043,7 +4043,7 @@
         <v>1611.4</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>2085.17</v>
+        <v>2273.77</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>15000</v>
@@ -4907,7 +4907,7 @@
         <v>27766.67</v>
       </c>
       <c r="F36" s="2" t="n">
-        <v>415.82</v>
+        <v>462.26</v>
       </c>
       <c r="G36" s="2" t="n">
         <v>10000</v>
@@ -5501,7 +5501,7 @@
         <v>0</v>
       </c>
       <c r="F58" s="2" t="n">
-        <v>0</v>
+        <v>295.2</v>
       </c>
       <c r="G58" s="2" t="n">
         <v>1000</v>
@@ -5528,7 +5528,7 @@
         <v>0</v>
       </c>
       <c r="F59" s="2" t="n">
-        <v>0</v>
+        <v>295.2</v>
       </c>
       <c r="G59" s="2" t="n">
         <v>0</v>
@@ -5545,7 +5545,7 @@
         <v>76363.98</v>
       </c>
       <c r="F60" s="5" t="n">
-        <v>20995.47</v>
+        <v>21820.91</v>
       </c>
       <c r="G60" s="5" t="n">
         <v>115950</v>
@@ -5716,13 +5716,13 @@
         <v>240</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>1566.9</v>
+        <v>1862.1</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>-1326.9</v>
+        <v>-1622.1</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>6.52875</v>
+        <v>7.75875</v>
       </c>
     </row>
     <row r="7">
@@ -5788,10 +5788,10 @@
         <v>0</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0</v>
+        <v>188.6</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>0</v>
+        <v>-188.6</v>
       </c>
       <c r="F9" s="3" t="n">
         <v>0</v>
@@ -5812,13 +5812,13 @@
         <v>728</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0</v>
+        <v>46.44</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>728</v>
+        <v>681.5599999999999</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>0</v>
+        <v>0.06379120879120879</v>
       </c>
     </row>
     <row r="11">
@@ -5927,13 +5927,13 @@
         <v>82783.32000000001</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>19974.87</v>
+        <v>20505.11</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>62808.45</v>
+        <v>62278.21</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.2412909992012884</v>
+        <v>0.2476961542494309</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-03-20 09:30:19
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -748,7 +748,7 @@
         <v>380.16</v>
       </c>
       <c r="M4" s="2" t="n">
-        <v>1609.97</v>
+        <v>1979.33</v>
       </c>
       <c r="N4" s="2" t="n">
         <v>0</v>
@@ -4043,7 +4043,7 @@
         <v>1611.4</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>2273.77</v>
+        <v>2643.13</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>15000</v>
@@ -5545,7 +5545,7 @@
         <v>76363.98</v>
       </c>
       <c r="F60" s="5" t="n">
-        <v>21820.91</v>
+        <v>22190.27</v>
       </c>
       <c r="G60" s="5" t="n">
         <v>115950</v>
@@ -5884,13 +5884,13 @@
         <v>65052</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>7191.28</v>
+        <v>7560.64</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>57860.72</v>
+        <v>57491.36</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.1105466396113878</v>
+        <v>0.1162245588144869</v>
       </c>
     </row>
     <row r="14">
@@ -5927,13 +5927,13 @@
         <v>82783.32000000001</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>20505.11</v>
+        <v>20874.47</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>62278.21</v>
+        <v>61908.85</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.2476961542494309</v>
+        <v>0.2521579226346564</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-03-23 15:30:24
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -2188,7 +2188,7 @@
         <v>0</v>
       </c>
       <c r="M28" s="2" t="n">
-        <v>0</v>
+        <v>1701.31</v>
       </c>
       <c r="N28" s="2" t="n">
         <v>0</v>
@@ -3879,7 +3879,7 @@
       </c>
       <c r="M56" s="4" t="inlineStr">
         <is>
-          <t>10 de 54</t>
+          <t>11 de 54</t>
         </is>
       </c>
       <c r="N56" s="4" t="inlineStr">
@@ -4691,7 +4691,7 @@
         <v>847.9</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>0</v>
+        <v>1701.31</v>
       </c>
       <c r="G28" s="2" t="n">
         <v>1500</v>
@@ -5545,7 +5545,7 @@
         <v>76363.98</v>
       </c>
       <c r="F60" s="5" t="n">
-        <v>22388.56</v>
+        <v>24089.87</v>
       </c>
       <c r="G60" s="5" t="n">
         <v>115950</v>
@@ -5884,13 +5884,13 @@
         <v>65052</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>7758.93</v>
+        <v>9460.24</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>57293.07</v>
+        <v>55591.76</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.1192727356576277</v>
+        <v>0.1454258131955974</v>
       </c>
     </row>
     <row r="14">
@@ -5927,13 +5927,13 @@
         <v>82783.32000000001</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>21072.76</v>
+        <v>22774.07</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>61710.56</v>
+        <v>60009.25</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.2545532119272337</v>
+        <v>0.2751045742064947</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-03-24 17:30:21
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -2248,7 +2248,7 @@
         <v>0</v>
       </c>
       <c r="M29" s="2" t="n">
-        <v>22.03</v>
+        <v>229.91</v>
       </c>
       <c r="N29" s="2" t="n">
         <v>0</v>
@@ -4718,7 +4718,7 @@
         <v>257.44</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>3579.99</v>
+        <v>3787.87</v>
       </c>
       <c r="G29" s="2" t="n">
         <v>6000</v>
@@ -5545,7 +5545,7 @@
         <v>76363.98</v>
       </c>
       <c r="F60" s="5" t="n">
-        <v>24155.45</v>
+        <v>24363.33</v>
       </c>
       <c r="G60" s="5" t="n">
         <v>115950</v>
@@ -5884,13 +5884,13 @@
         <v>65052</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>9460.24</v>
+        <v>9668.120000000001</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>55591.76</v>
+        <v>55383.88</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.1454258131955974</v>
+        <v>0.1486214105638566</v>
       </c>
     </row>
     <row r="14">
@@ -5927,13 +5927,13 @@
         <v>82783.32000000001</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>22839.65</v>
+        <v>23047.53000000001</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>59943.67000000001</v>
+        <v>59735.79</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.2758967627778156</v>
+        <v>0.2784078966632409</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-03-25 15:30:19
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -724,7 +724,7 @@
         <v>95.04000000000001</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>0</v>
+        <v>74.29000000000001</v>
       </c>
       <c r="F4" s="2" t="n">
         <v>0</v>
@@ -751,7 +751,7 @@
         <v>1979.33</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>0</v>
+        <v>234.47</v>
       </c>
       <c r="O4" s="2" t="n">
         <v>0</v>
@@ -808,7 +808,7 @@
         <v>835.22</v>
       </c>
       <c r="M5" s="2" t="n">
-        <v>33.05</v>
+        <v>444.4</v>
       </c>
       <c r="N5" s="2" t="n">
         <v>0</v>
@@ -2242,7 +2242,7 @@
         <v>0</v>
       </c>
       <c r="K29" s="2" t="n">
-        <v>0</v>
+        <v>459.86</v>
       </c>
       <c r="L29" s="2" t="n">
         <v>0</v>
@@ -3025,7 +3025,7 @@
         <v>0</v>
       </c>
       <c r="L42" s="2" t="n">
-        <v>0</v>
+        <v>253.44</v>
       </c>
       <c r="M42" s="2" t="n">
         <v>0</v>
@@ -3688,7 +3688,7 @@
         <v>0</v>
       </c>
       <c r="M53" s="2" t="n">
-        <v>1020.6</v>
+        <v>1296.86</v>
       </c>
       <c r="N53" s="2" t="n">
         <v>0</v>
@@ -3839,19 +3839,19 @@
       </c>
       <c r="E56" s="4" t="inlineStr">
         <is>
+          <t>1 de 54</t>
+        </is>
+      </c>
+      <c r="F56" s="4" t="inlineStr">
+        <is>
           <t>0 de 54</t>
         </is>
       </c>
-      <c r="F56" s="4" t="inlineStr">
+      <c r="G56" s="4" t="inlineStr">
         <is>
           <t>0 de 54</t>
         </is>
       </c>
-      <c r="G56" s="4" t="inlineStr">
-        <is>
-          <t>0 de 54</t>
-        </is>
-      </c>
       <c r="H56" s="4" t="inlineStr">
         <is>
           <t>3 de 54</t>
@@ -3869,22 +3869,22 @@
       </c>
       <c r="K56" s="4" t="inlineStr">
         <is>
+          <t>2 de 54</t>
+        </is>
+      </c>
+      <c r="L56" s="4" t="inlineStr">
+        <is>
+          <t>6 de 54</t>
+        </is>
+      </c>
+      <c r="M56" s="4" t="inlineStr">
+        <is>
+          <t>11 de 54</t>
+        </is>
+      </c>
+      <c r="N56" s="4" t="inlineStr">
+        <is>
           <t>1 de 54</t>
-        </is>
-      </c>
-      <c r="L56" s="4" t="inlineStr">
-        <is>
-          <t>5 de 54</t>
-        </is>
-      </c>
-      <c r="M56" s="4" t="inlineStr">
-        <is>
-          <t>11 de 54</t>
-        </is>
-      </c>
-      <c r="N56" s="4" t="inlineStr">
-        <is>
-          <t>0 de 54</t>
         </is>
       </c>
       <c r="O56" s="4" t="inlineStr">
@@ -4043,7 +4043,7 @@
         <v>1611.4</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>2635.61</v>
+        <v>2944.37</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>15000</v>
@@ -4070,7 +4070,7 @@
         <v>4113.15</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>1036.75</v>
+        <v>1448.1</v>
       </c>
       <c r="G5" s="2" t="n">
         <v>10000</v>
@@ -4718,7 +4718,7 @@
         <v>257.44</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>3787.87</v>
+        <v>4247.73</v>
       </c>
       <c r="G29" s="2" t="n">
         <v>6000</v>
@@ -5042,7 +5042,7 @@
         <v>0</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>669.0599999999999</v>
+        <v>1338.12</v>
       </c>
       <c r="G41" s="2" t="n">
         <v>1000</v>
@@ -5069,7 +5069,7 @@
         <v>0</v>
       </c>
       <c r="F42" s="2" t="n">
-        <v>0</v>
+        <v>1562.76</v>
       </c>
       <c r="G42" s="2" t="n">
         <v>2000</v>
@@ -5420,7 +5420,7 @@
         <v>1915.78</v>
       </c>
       <c r="F55" s="2" t="n">
-        <v>1020.6</v>
+        <v>1296.86</v>
       </c>
       <c r="G55" s="2" t="n">
         <v>500</v>
@@ -5447,7 +5447,7 @@
         <v>1915.78</v>
       </c>
       <c r="F56" s="2" t="n">
-        <v>1020.6</v>
+        <v>1296.86</v>
       </c>
       <c r="G56" s="2" t="n">
         <v>1000</v>
@@ -5545,7 +5545,7 @@
         <v>76363.98</v>
       </c>
       <c r="F60" s="5" t="n">
-        <v>24458.37</v>
+        <v>28422.68</v>
       </c>
       <c r="G60" s="5" t="n">
         <v>115950</v>
@@ -5568,7 +5568,7 @@
     <col width="32" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
@@ -5668,13 +5668,13 @@
         <v>199.5</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>0</v>
+        <v>74.29000000000001</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>199.5</v>
+        <v>125.21</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>0</v>
+        <v>0.3723809523809524</v>
       </c>
     </row>
     <row r="5">
@@ -5812,13 +5812,13 @@
         <v>728</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>46.44</v>
+        <v>506.3</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>681.5599999999999</v>
+        <v>221.7</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>0.06379120879120879</v>
+        <v>0.6954670329670329</v>
       </c>
     </row>
     <row r="11">
@@ -5836,13 +5836,13 @@
         <v>350</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>1226.61</v>
+        <v>3204.99</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>-876.6099999999999</v>
+        <v>-2854.99</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>3.504599999999999</v>
+        <v>9.157114285714284</v>
       </c>
     </row>
     <row r="12">
@@ -5860,13 +5860,13 @@
         <v>7700</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>2605.46</v>
+        <v>2858.9</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>5094.54</v>
+        <v>4841.1</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0.3383714285714286</v>
+        <v>0.3712857142857143</v>
       </c>
     </row>
     <row r="13">
@@ -5884,13 +5884,13 @@
         <v>65052</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>9668.120000000001</v>
+        <v>10355.73</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>55383.88</v>
+        <v>54696.27</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.1486214105638566</v>
+        <v>0.1591915698210662</v>
       </c>
     </row>
     <row r="14">
@@ -5908,13 +5908,13 @@
         <v>402</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>0</v>
+        <v>234.47</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>402</v>
+        <v>167.53</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0</v>
+        <v>0.5832587064676616</v>
       </c>
     </row>
     <row r="15">
@@ -5927,13 +5927,13 @@
         <v>82783.32000000001</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>23142.57</v>
+        <v>26830.62</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>59640.75</v>
+        <v>55952.7</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.2795559540255211</v>
+        <v>0.3241065953866069</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-03-25 16:30:20
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -3022,7 +3022,7 @@
         <v>0</v>
       </c>
       <c r="K42" s="2" t="n">
-        <v>0</v>
+        <v>304.56</v>
       </c>
       <c r="L42" s="2" t="n">
         <v>253.44</v>
@@ -3031,7 +3031,7 @@
         <v>0</v>
       </c>
       <c r="N42" s="2" t="n">
-        <v>0</v>
+        <v>135.79</v>
       </c>
       <c r="O42" s="2" t="n">
         <v>0</v>
@@ -3869,22 +3869,22 @@
       </c>
       <c r="K56" s="4" t="inlineStr">
         <is>
+          <t>3 de 54</t>
+        </is>
+      </c>
+      <c r="L56" s="4" t="inlineStr">
+        <is>
+          <t>6 de 54</t>
+        </is>
+      </c>
+      <c r="M56" s="4" t="inlineStr">
+        <is>
+          <t>11 de 54</t>
+        </is>
+      </c>
+      <c r="N56" s="4" t="inlineStr">
+        <is>
           <t>2 de 54</t>
-        </is>
-      </c>
-      <c r="L56" s="4" t="inlineStr">
-        <is>
-          <t>6 de 54</t>
-        </is>
-      </c>
-      <c r="M56" s="4" t="inlineStr">
-        <is>
-          <t>11 de 54</t>
-        </is>
-      </c>
-      <c r="N56" s="4" t="inlineStr">
-        <is>
-          <t>1 de 54</t>
         </is>
       </c>
       <c r="O56" s="4" t="inlineStr">
@@ -5069,7 +5069,7 @@
         <v>0</v>
       </c>
       <c r="F42" s="2" t="n">
-        <v>1562.76</v>
+        <v>2003.11</v>
       </c>
       <c r="G42" s="2" t="n">
         <v>2000</v>
@@ -5545,7 +5545,7 @@
         <v>76363.98</v>
       </c>
       <c r="F60" s="5" t="n">
-        <v>28422.68</v>
+        <v>28863.03</v>
       </c>
       <c r="G60" s="5" t="n">
         <v>115950</v>
@@ -5812,13 +5812,13 @@
         <v>728</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>506.3</v>
+        <v>810.86</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>221.7</v>
+        <v>-82.86000000000001</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>0.6954670329670329</v>
+        <v>1.113818681318681</v>
       </c>
     </row>
     <row r="11">
@@ -5908,13 +5908,13 @@
         <v>402</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>234.47</v>
+        <v>370.26</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>167.53</v>
+        <v>31.74000000000001</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.5832587064676616</v>
+        <v>0.9210447761194029</v>
       </c>
     </row>
     <row r="15">
@@ -5927,13 +5927,13 @@
         <v>82783.32000000001</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>26830.62</v>
+        <v>27270.97</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>55952.7</v>
+        <v>55512.35</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.3241065953866069</v>
+        <v>0.3294259036723823</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-03-25 17:30:20
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -1456,7 +1456,7 @@
         <v>0</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>0</v>
+        <v>151.2</v>
       </c>
       <c r="J16" s="2" t="n">
         <v>0</v>
@@ -1468,7 +1468,7 @@
         <v>0</v>
       </c>
       <c r="M16" s="2" t="n">
-        <v>0</v>
+        <v>2709.07</v>
       </c>
       <c r="N16" s="2" t="n">
         <v>0</v>
@@ -3859,7 +3859,7 @@
       </c>
       <c r="I56" s="4" t="inlineStr">
         <is>
-          <t>2 de 54</t>
+          <t>3 de 54</t>
         </is>
       </c>
       <c r="J56" s="4" t="inlineStr">
@@ -3879,7 +3879,7 @@
       </c>
       <c r="M56" s="4" t="inlineStr">
         <is>
-          <t>11 de 54</t>
+          <t>12 de 54</t>
         </is>
       </c>
       <c r="N56" s="4" t="inlineStr">
@@ -4367,7 +4367,7 @@
         <v>11341.48</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>0</v>
+        <v>2860.27</v>
       </c>
       <c r="G16" s="2" t="n">
         <v>6000</v>
@@ -5545,7 +5545,7 @@
         <v>76363.98</v>
       </c>
       <c r="F60" s="5" t="n">
-        <v>28863.03</v>
+        <v>31723.3</v>
       </c>
       <c r="G60" s="5" t="n">
         <v>115950</v>
@@ -5568,7 +5568,7 @@
     <col width="32" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
@@ -5740,13 +5740,13 @@
         <v>653</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>337.7</v>
+        <v>488.9</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>315.3</v>
+        <v>164.1</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>0.5171516079632466</v>
+        <v>0.748698315467075</v>
       </c>
     </row>
     <row r="8">
@@ -5884,13 +5884,13 @@
         <v>65052</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>10355.73</v>
+        <v>13064.8</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>54696.27</v>
+        <v>51987.2</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.1591915698210662</v>
+        <v>0.2008362540736641</v>
       </c>
     </row>
     <row r="14">
@@ -5927,13 +5927,13 @@
         <v>82783.32000000001</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>27270.97</v>
+        <v>30131.24</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>55512.35</v>
+        <v>52652.07999999999</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.3294259036723823</v>
+        <v>0.363977187675005</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-03-26 16:30:23
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -745,7 +745,7 @@
         <v>0</v>
       </c>
       <c r="L4" s="2" t="n">
-        <v>380.16</v>
+        <v>698.11</v>
       </c>
       <c r="M4" s="2" t="n">
         <v>1979.33</v>
@@ -4043,7 +4043,7 @@
         <v>1611.4</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>2944.37</v>
+        <v>3262.32</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>15000</v>
@@ -5545,7 +5545,7 @@
         <v>76363.98</v>
       </c>
       <c r="F60" s="5" t="n">
-        <v>31723.3</v>
+        <v>32041.25</v>
       </c>
       <c r="G60" s="5" t="n">
         <v>115950</v>
@@ -5860,13 +5860,13 @@
         <v>7700</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>2858.9</v>
+        <v>3176.85</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>4841.1</v>
+        <v>4523.15</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0.3712857142857143</v>
+        <v>0.412577922077922</v>
       </c>
     </row>
     <row r="13">
@@ -5927,13 +5927,13 @@
         <v>82783.32000000001</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>30131.24</v>
+        <v>30449.19</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>52652.07999999999</v>
+        <v>52334.13</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.363977187675005</v>
+        <v>0.3678179372366317</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-03-30 08:30:21
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -748,7 +748,7 @@
         <v>698.11</v>
       </c>
       <c r="M4" s="2" t="n">
-        <v>1979.33</v>
+        <v>3476.65</v>
       </c>
       <c r="N4" s="2" t="n">
         <v>234.47</v>
@@ -781,7 +781,7 @@
         <v>0</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>0</v>
+        <v>316.8</v>
       </c>
       <c r="E5" s="2" t="n">
         <v>0</v>
@@ -805,10 +805,10 @@
         <v>0</v>
       </c>
       <c r="L5" s="2" t="n">
-        <v>835.22</v>
+        <v>3013.41</v>
       </c>
       <c r="M5" s="2" t="n">
-        <v>444.4</v>
+        <v>2258.37</v>
       </c>
       <c r="N5" s="2" t="n">
         <v>0</v>
@@ -1645,7 +1645,7 @@
         <v>0</v>
       </c>
       <c r="L19" s="2" t="n">
-        <v>0</v>
+        <v>443.44</v>
       </c>
       <c r="M19" s="2" t="n">
         <v>0</v>
@@ -3834,47 +3834,47 @@
       </c>
       <c r="D56" s="4" t="inlineStr">
         <is>
+          <t>8 de 54</t>
+        </is>
+      </c>
+      <c r="E56" s="4" t="inlineStr">
+        <is>
+          <t>1 de 54</t>
+        </is>
+      </c>
+      <c r="F56" s="4" t="inlineStr">
+        <is>
+          <t>0 de 54</t>
+        </is>
+      </c>
+      <c r="G56" s="4" t="inlineStr">
+        <is>
+          <t>0 de 54</t>
+        </is>
+      </c>
+      <c r="H56" s="4" t="inlineStr">
+        <is>
+          <t>3 de 54</t>
+        </is>
+      </c>
+      <c r="I56" s="4" t="inlineStr">
+        <is>
+          <t>3 de 54</t>
+        </is>
+      </c>
+      <c r="J56" s="4" t="inlineStr">
+        <is>
+          <t>1 de 54</t>
+        </is>
+      </c>
+      <c r="K56" s="4" t="inlineStr">
+        <is>
+          <t>3 de 54</t>
+        </is>
+      </c>
+      <c r="L56" s="4" t="inlineStr">
+        <is>
           <t>7 de 54</t>
-        </is>
-      </c>
-      <c r="E56" s="4" t="inlineStr">
-        <is>
-          <t>1 de 54</t>
-        </is>
-      </c>
-      <c r="F56" s="4" t="inlineStr">
-        <is>
-          <t>0 de 54</t>
-        </is>
-      </c>
-      <c r="G56" s="4" t="inlineStr">
-        <is>
-          <t>0 de 54</t>
-        </is>
-      </c>
-      <c r="H56" s="4" t="inlineStr">
-        <is>
-          <t>3 de 54</t>
-        </is>
-      </c>
-      <c r="I56" s="4" t="inlineStr">
-        <is>
-          <t>3 de 54</t>
-        </is>
-      </c>
-      <c r="J56" s="4" t="inlineStr">
-        <is>
-          <t>1 de 54</t>
-        </is>
-      </c>
-      <c r="K56" s="4" t="inlineStr">
-        <is>
-          <t>3 de 54</t>
-        </is>
-      </c>
-      <c r="L56" s="4" t="inlineStr">
-        <is>
-          <t>6 de 54</t>
         </is>
       </c>
       <c r="M56" s="4" t="inlineStr">
@@ -4043,7 +4043,7 @@
         <v>1611.4</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>3262.32</v>
+        <v>4817.91</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>15000</v>
@@ -4070,7 +4070,7 @@
         <v>4113.15</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>1448.1</v>
+        <v>5757.06</v>
       </c>
       <c r="G5" s="2" t="n">
         <v>10000</v>
@@ -4448,7 +4448,7 @@
         <v>0</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>0</v>
+        <v>443.44</v>
       </c>
       <c r="G19" s="2" t="n">
         <v>1000</v>
@@ -5366,7 +5366,7 @@
         <v>2465.83</v>
       </c>
       <c r="F53" s="2" t="n">
-        <v>0</v>
+        <v>834.48</v>
       </c>
       <c r="G53" s="2" t="n">
         <v>1500</v>
@@ -5393,7 +5393,7 @@
         <v>2465.83</v>
       </c>
       <c r="F54" s="2" t="n">
-        <v>0</v>
+        <v>834.48</v>
       </c>
       <c r="G54" s="2" t="n">
         <v>1650</v>
@@ -5545,7 +5545,7 @@
         <v>76363.98</v>
       </c>
       <c r="F60" s="5" t="n">
-        <v>49059.35</v>
+        <v>57036.3</v>
       </c>
       <c r="G60" s="5" t="n">
         <v>115950</v>
@@ -5644,13 +5644,13 @@
         <v>6600</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>6900.69</v>
+        <v>7217.49</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>-300.6899999999996</v>
+        <v>-617.4899999999998</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>1.045559090909091</v>
+        <v>1.093559090909091</v>
       </c>
     </row>
     <row r="4">
@@ -5836,13 +5836,13 @@
         <v>350</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>3204.99</v>
+        <v>4097.74</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>-2854.99</v>
+        <v>-3747.74</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>9.157114285714284</v>
+        <v>11.70782857142857</v>
       </c>
     </row>
     <row r="12">
@@ -5860,13 +5860,13 @@
         <v>7700</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>8498.129999999999</v>
+        <v>11119.76</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>-798.1299999999992</v>
+        <v>-3419.76</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>1.103653246753247</v>
+        <v>1.444124675324675</v>
       </c>
     </row>
     <row r="13">
@@ -5884,13 +5884,13 @@
         <v>65052</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>24761.62</v>
+        <v>28072.91</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>40290.38</v>
+        <v>36979.09</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.3806434852118305</v>
+        <v>0.4315456865277009</v>
       </c>
     </row>
     <row r="14">
@@ -5927,13 +5927,13 @@
         <v>82783.32000000001</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>47467.29</v>
+        <v>54609.76</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>35316.03</v>
+        <v>28173.56</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.5733919586699349</v>
+        <v>0.6596710545071156</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-03-30 17:30:25
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -2236,7 +2236,7 @@
         <v>782.1</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>0</v>
+        <v>48.6</v>
       </c>
       <c r="J29" s="2" t="n">
         <v>0</v>
@@ -3025,7 +3025,7 @@
         <v>304.56</v>
       </c>
       <c r="L42" s="2" t="n">
-        <v>253.44</v>
+        <v>380.16</v>
       </c>
       <c r="M42" s="2" t="n">
         <v>0</v>
@@ -3859,7 +3859,7 @@
       </c>
       <c r="I56" s="4" t="inlineStr">
         <is>
-          <t>3 de 54</t>
+          <t>4 de 54</t>
         </is>
       </c>
       <c r="J56" s="4" t="inlineStr">
@@ -4718,7 +4718,7 @@
         <v>257.44</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>4247.73</v>
+        <v>4296.33</v>
       </c>
       <c r="G29" s="2" t="n">
         <v>6000</v>
@@ -5069,7 +5069,7 @@
         <v>0</v>
       </c>
       <c r="F42" s="2" t="n">
-        <v>2003.11</v>
+        <v>2129.83</v>
       </c>
       <c r="G42" s="2" t="n">
         <v>2000</v>
@@ -5545,7 +5545,7 @@
         <v>76363.98</v>
       </c>
       <c r="F60" s="5" t="n">
-        <v>57036.3</v>
+        <v>57211.62</v>
       </c>
       <c r="G60" s="5" t="n">
         <v>115950</v>
@@ -5740,13 +5740,13 @@
         <v>653</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>488.9</v>
+        <v>537.5</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>164.1</v>
+        <v>115.5</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>0.748698315467075</v>
+        <v>0.8231240428790199</v>
       </c>
     </row>
     <row r="8">
@@ -5860,13 +5860,13 @@
         <v>7700</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>11119.76</v>
+        <v>11246.48</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>-3419.76</v>
+        <v>-3546.48</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>1.444124675324675</v>
+        <v>1.460581818181818</v>
       </c>
     </row>
     <row r="13">
@@ -5927,13 +5927,13 @@
         <v>82783.32000000001</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>54609.76</v>
+        <v>54785.08</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>28173.56</v>
+        <v>27998.24</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.6596710545071156</v>
+        <v>0.6617888724443522</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-04-07 08:30:17
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -2236,7 +2236,7 @@
         <v>0</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>0</v>
+        <v>435.6</v>
       </c>
       <c r="J29" s="2" t="n">
         <v>0</v>
@@ -3859,7 +3859,7 @@
       </c>
       <c r="I56" s="4" t="inlineStr">
         <is>
-          <t>0 de 54</t>
+          <t>1 de 54</t>
         </is>
       </c>
       <c r="J56" s="4" t="inlineStr">
@@ -4718,7 +4718,7 @@
         <v>8735.280000000001</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>0</v>
+        <v>435.6</v>
       </c>
       <c r="G29" s="2" t="n">
         <v>6000</v>
@@ -5545,7 +5545,7 @@
         <v>79624.92</v>
       </c>
       <c r="F60" s="5" t="n">
-        <v>-64.21000000000001</v>
+        <v>371.39</v>
       </c>
       <c r="G60" s="5" t="n">
         <v>115950</v>

</xml_diff>

<commit_message>
Actualización automática 2026-04-09 08:30:20
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -2677,7 +2677,7 @@
         <v>0</v>
       </c>
       <c r="P36" s="2" t="n">
-        <v>0</v>
+        <v>474.43</v>
       </c>
       <c r="Q36" s="2" t="n">
         <v>0</v>
@@ -3894,7 +3894,7 @@
       </c>
       <c r="P56" s="4" t="inlineStr">
         <is>
-          <t>0 de 54</t>
+          <t>1 de 54</t>
         </is>
       </c>
       <c r="Q56" s="4" t="inlineStr">
@@ -4907,7 +4907,7 @@
         <v>17480.36</v>
       </c>
       <c r="F36" s="2" t="n">
-        <v>0</v>
+        <v>474.43</v>
       </c>
       <c r="G36" s="2" t="n">
         <v>10000</v>
@@ -5545,7 +5545,7 @@
         <v>79624.92</v>
       </c>
       <c r="F60" s="5" t="n">
-        <v>430.97</v>
+        <v>905.4</v>
       </c>
       <c r="G60" s="5" t="n">
         <v>115950</v>

</xml_diff>

<commit_message>
Actualización automática 2026-04-09 17:30:18
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -2428,7 +2428,7 @@
         <v>0</v>
       </c>
       <c r="M32" s="2" t="n">
-        <v>0</v>
+        <v>1508.89</v>
       </c>
       <c r="N32" s="2" t="n">
         <v>0</v>
@@ -3361,7 +3361,7 @@
         <v>0</v>
       </c>
       <c r="D48" s="2" t="n">
-        <v>0</v>
+        <v>2453.44</v>
       </c>
       <c r="E48" s="2" t="n">
         <v>0</v>
@@ -3834,52 +3834,52 @@
       </c>
       <c r="D56" s="4" t="inlineStr">
         <is>
+          <t>2 de 54</t>
+        </is>
+      </c>
+      <c r="E56" s="4" t="inlineStr">
+        <is>
+          <t>0 de 54</t>
+        </is>
+      </c>
+      <c r="F56" s="4" t="inlineStr">
+        <is>
+          <t>0 de 54</t>
+        </is>
+      </c>
+      <c r="G56" s="4" t="inlineStr">
+        <is>
+          <t>0 de 54</t>
+        </is>
+      </c>
+      <c r="H56" s="4" t="inlineStr">
+        <is>
+          <t>0 de 54</t>
+        </is>
+      </c>
+      <c r="I56" s="4" t="inlineStr">
+        <is>
           <t>1 de 54</t>
         </is>
       </c>
-      <c r="E56" s="4" t="inlineStr">
+      <c r="J56" s="4" t="inlineStr">
         <is>
           <t>0 de 54</t>
         </is>
       </c>
-      <c r="F56" s="4" t="inlineStr">
+      <c r="K56" s="4" t="inlineStr">
         <is>
           <t>0 de 54</t>
         </is>
       </c>
-      <c r="G56" s="4" t="inlineStr">
+      <c r="L56" s="4" t="inlineStr">
         <is>
           <t>0 de 54</t>
         </is>
       </c>
-      <c r="H56" s="4" t="inlineStr">
-        <is>
-          <t>0 de 54</t>
-        </is>
-      </c>
-      <c r="I56" s="4" t="inlineStr">
-        <is>
-          <t>1 de 54</t>
-        </is>
-      </c>
-      <c r="J56" s="4" t="inlineStr">
-        <is>
-          <t>0 de 54</t>
-        </is>
-      </c>
-      <c r="K56" s="4" t="inlineStr">
-        <is>
-          <t>0 de 54</t>
-        </is>
-      </c>
-      <c r="L56" s="4" t="inlineStr">
-        <is>
-          <t>0 de 54</t>
-        </is>
-      </c>
       <c r="M56" s="4" t="inlineStr">
         <is>
-          <t>1 de 54</t>
+          <t>2 de 54</t>
         </is>
       </c>
       <c r="N56" s="4" t="inlineStr">
@@ -3927,7 +3927,7 @@
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -4799,7 +4799,7 @@
         <v>264.6</v>
       </c>
       <c r="F32" s="2" t="n">
-        <v>0</v>
+        <v>1508.89</v>
       </c>
       <c r="G32" s="2" t="n">
         <v>3000</v>
@@ -5231,7 +5231,7 @@
         <v>2787.07</v>
       </c>
       <c r="F48" s="2" t="n">
-        <v>0</v>
+        <v>2453.44</v>
       </c>
       <c r="G48" s="2" t="n">
         <v>1500</v>
@@ -5545,7 +5545,7 @@
         <v>79624.92</v>
       </c>
       <c r="F60" s="5" t="n">
-        <v>905.4</v>
+        <v>4867.73</v>
       </c>
       <c r="G60" s="5" t="n">
         <v>115950</v>

</xml_diff>

<commit_message>
Actualización automática 2026-04-13 17:30:23
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -1888,7 +1888,7 @@
         <v>0</v>
       </c>
       <c r="M23" s="2" t="n">
-        <v>0</v>
+        <v>1111.97</v>
       </c>
       <c r="N23" s="2" t="n">
         <v>0</v>
@@ -1948,7 +1948,7 @@
         <v>0</v>
       </c>
       <c r="M24" s="2" t="n">
-        <v>0</v>
+        <v>1206.63</v>
       </c>
       <c r="N24" s="2" t="n">
         <v>0</v>
@@ -3879,7 +3879,7 @@
       </c>
       <c r="M56" s="4" t="inlineStr">
         <is>
-          <t>2 de 54</t>
+          <t>4 de 54</t>
         </is>
       </c>
       <c r="N56" s="4" t="inlineStr">
@@ -4556,7 +4556,7 @@
         <v>0</v>
       </c>
       <c r="F23" s="2" t="n">
-        <v>0</v>
+        <v>1111.97</v>
       </c>
       <c r="G23" s="2" t="n">
         <v>0</v>
@@ -4583,7 +4583,7 @@
         <v>2711.11</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>0</v>
+        <v>1206.63</v>
       </c>
       <c r="G24" s="2" t="n">
         <v>15000</v>
@@ -5545,7 +5545,7 @@
         <v>79624.92</v>
       </c>
       <c r="F60" s="5" t="n">
-        <v>4765.41</v>
+        <v>7084.01</v>
       </c>
       <c r="G60" s="5" t="n">
         <v>115950</v>
@@ -5860,13 +5860,13 @@
         <v>54325</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>1384.93</v>
+        <v>3703.53</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>52940.07</v>
+        <v>50621.47</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0.02549341923607916</v>
+        <v>0.06817358490566038</v>
       </c>
     </row>
     <row r="13">
@@ -5927,13 +5927,13 @@
         <v>73362.32000000001</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>4765.41</v>
+        <v>7084.01</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>68596.91</v>
+        <v>66278.31</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.06495718783157348</v>
+        <v>0.09656196805117395</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-04-14 14:30:18
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -3022,7 +3022,7 @@
         <v>0</v>
       </c>
       <c r="K42" s="2" t="n">
-        <v>0</v>
+        <v>101.52</v>
       </c>
       <c r="L42" s="2" t="n">
         <v>0</v>
@@ -3869,7 +3869,7 @@
       </c>
       <c r="K56" s="4" t="inlineStr">
         <is>
-          <t>0 de 54</t>
+          <t>1 de 54</t>
         </is>
       </c>
       <c r="L56" s="4" t="inlineStr">
@@ -5069,7 +5069,7 @@
         <v>1994.04</v>
       </c>
       <c r="F42" s="2" t="n">
-        <v>0</v>
+        <v>101.52</v>
       </c>
       <c r="G42" s="2" t="n">
         <v>2000</v>
@@ -5545,7 +5545,7 @@
         <v>79624.92</v>
       </c>
       <c r="F60" s="5" t="n">
-        <v>7084.01</v>
+        <v>7185.530000000001</v>
       </c>
       <c r="G60" s="5" t="n">
         <v>115950</v>
@@ -5788,13 +5788,13 @@
         <v>1300</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0</v>
+        <v>101.52</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>1300</v>
+        <v>1198.48</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>0</v>
+        <v>0.07809230769230768</v>
       </c>
     </row>
     <row r="10">
@@ -5927,13 +5927,13 @@
         <v>73362.32000000001</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>7084.01</v>
+        <v>7185.53</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>66278.31</v>
+        <v>66176.79000000001</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.09656196805117395</v>
+        <v>0.09794578470255574</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-04-14 16:30:17
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -748,7 +748,7 @@
         <v>0</v>
       </c>
       <c r="M4" s="2" t="n">
-        <v>42.57</v>
+        <v>334.82</v>
       </c>
       <c r="N4" s="2" t="n">
         <v>0</v>
@@ -4043,7 +4043,7 @@
         <v>4764.43</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>42.57</v>
+        <v>334.82</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>15000</v>
@@ -5545,7 +5545,7 @@
         <v>79624.92</v>
       </c>
       <c r="F60" s="5" t="n">
-        <v>7185.530000000001</v>
+        <v>7477.780000000001</v>
       </c>
       <c r="G60" s="5" t="n">
         <v>115950</v>
@@ -5860,13 +5860,13 @@
         <v>54325</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>3703.53</v>
+        <v>3995.78</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>50621.47</v>
+        <v>50329.22</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0.06817358490566038</v>
+        <v>0.0735532443626323</v>
       </c>
     </row>
     <row r="13">
@@ -5927,13 +5927,13 @@
         <v>73362.32000000001</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>7185.53</v>
+        <v>7477.78</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>66176.79000000001</v>
+        <v>65884.54000000001</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.09794578470255574</v>
+        <v>0.1019294373460381</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-04-15 12:30:18
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -2881,7 +2881,7 @@
         <v>0</v>
       </c>
       <c r="D40" s="2" t="n">
-        <v>0</v>
+        <v>2453.5</v>
       </c>
       <c r="E40" s="2" t="n">
         <v>0</v>
@@ -2908,7 +2908,7 @@
         <v>0</v>
       </c>
       <c r="M40" s="2" t="n">
-        <v>0</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="N40" s="2" t="n">
         <v>0</v>
@@ -3834,7 +3834,7 @@
       </c>
       <c r="D56" s="4" t="inlineStr">
         <is>
-          <t>2 de 54</t>
+          <t>3 de 54</t>
         </is>
       </c>
       <c r="E56" s="4" t="inlineStr">
@@ -3879,7 +3879,7 @@
       </c>
       <c r="M56" s="4" t="inlineStr">
         <is>
-          <t>4 de 54</t>
+          <t>5 de 54</t>
         </is>
       </c>
       <c r="N56" s="4" t="inlineStr">
@@ -5015,7 +5015,7 @@
         <v>224.96</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>0</v>
+        <v>2519.6</v>
       </c>
       <c r="G40" s="2" t="n">
         <v>3500</v>
@@ -5545,7 +5545,7 @@
         <v>79624.92</v>
       </c>
       <c r="F60" s="5" t="n">
-        <v>11559.11</v>
+        <v>14078.71</v>
       </c>
       <c r="G60" s="5" t="n">
         <v>115950</v>
@@ -5644,13 +5644,13 @@
         <v>8373</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>2400.35</v>
+        <v>4853.85</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>5972.65</v>
+        <v>3519.15</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>0.2866774155022095</v>
+        <v>0.5797026155499821</v>
       </c>
     </row>
     <row r="4">
@@ -5860,13 +5860,13 @@
         <v>54325</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>8017.61</v>
+        <v>8083.71</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>46307.39</v>
+        <v>46241.29</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0.1475860101242522</v>
+        <v>0.1488027611596871</v>
       </c>
     </row>
     <row r="13">
@@ -5927,13 +5927,13 @@
         <v>73362.32000000001</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>11559.11</v>
+        <v>14078.71</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>61803.21</v>
+        <v>59283.61</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.1575619473320909</v>
+        <v>0.1919065536640608</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-04-16 08:30:19
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -805,10 +805,10 @@
         <v>0</v>
       </c>
       <c r="L5" s="2" t="n">
-        <v>0</v>
+        <v>1696.3</v>
       </c>
       <c r="M5" s="2" t="n">
-        <v>0</v>
+        <v>52.99</v>
       </c>
       <c r="N5" s="2" t="n">
         <v>0</v>
@@ -1861,7 +1861,7 @@
         <v>0</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>0</v>
+        <v>489.88</v>
       </c>
       <c r="E23" s="2" t="n">
         <v>0</v>
@@ -2248,7 +2248,7 @@
         <v>0</v>
       </c>
       <c r="M29" s="2" t="n">
-        <v>-78.93000000000001</v>
+        <v>25.01</v>
       </c>
       <c r="N29" s="2" t="n">
         <v>0</v>
@@ -2677,7 +2677,7 @@
         <v>0</v>
       </c>
       <c r="P36" s="2" t="n">
-        <v>474.43</v>
+        <v>1558.83</v>
       </c>
       <c r="Q36" s="2" t="n">
         <v>0</v>
@@ -2728,7 +2728,7 @@
         <v>0</v>
       </c>
       <c r="M37" s="2" t="n">
-        <v>0</v>
+        <v>1140.48</v>
       </c>
       <c r="N37" s="2" t="n">
         <v>0</v>
@@ -3328,7 +3328,7 @@
         <v>0</v>
       </c>
       <c r="M47" s="2" t="n">
-        <v>0</v>
+        <v>1786.75</v>
       </c>
       <c r="N47" s="2" t="n">
         <v>0</v>
@@ -3834,7 +3834,7 @@
       </c>
       <c r="D56" s="4" t="inlineStr">
         <is>
-          <t>3 de 54</t>
+          <t>4 de 54</t>
         </is>
       </c>
       <c r="E56" s="4" t="inlineStr">
@@ -3874,12 +3874,12 @@
       </c>
       <c r="L56" s="4" t="inlineStr">
         <is>
-          <t>0 de 54</t>
+          <t>1 de 54</t>
         </is>
       </c>
       <c r="M56" s="4" t="inlineStr">
         <is>
-          <t>5 de 54</t>
+          <t>9 de 54</t>
         </is>
       </c>
       <c r="N56" s="4" t="inlineStr">
@@ -4070,7 +4070,7 @@
         <v>12980.37</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>0</v>
+        <v>1749.29</v>
       </c>
       <c r="G5" s="2" t="n">
         <v>10000</v>
@@ -4556,7 +4556,7 @@
         <v>0</v>
       </c>
       <c r="F23" s="2" t="n">
-        <v>1111.97</v>
+        <v>1601.85</v>
       </c>
       <c r="G23" s="2" t="n">
         <v>0</v>
@@ -4718,7 +4718,7 @@
         <v>8735.280000000001</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>373.68</v>
+        <v>477.62</v>
       </c>
       <c r="G29" s="2" t="n">
         <v>6000</v>
@@ -4907,7 +4907,7 @@
         <v>17480.36</v>
       </c>
       <c r="F36" s="2" t="n">
-        <v>451.04</v>
+        <v>1535.44</v>
       </c>
       <c r="G36" s="2" t="n">
         <v>10000</v>
@@ -4934,7 +4934,7 @@
         <v>565.25</v>
       </c>
       <c r="F37" s="2" t="n">
-        <v>0</v>
+        <v>1140.48</v>
       </c>
       <c r="G37" s="2" t="n">
         <v>8000</v>
@@ -5204,7 +5204,7 @@
         <v>378.38</v>
       </c>
       <c r="F47" s="2" t="n">
-        <v>0</v>
+        <v>1786.75</v>
       </c>
       <c r="G47" s="2" t="n">
         <v>1500</v>
@@ -5545,7 +5545,7 @@
         <v>79624.92</v>
       </c>
       <c r="F60" s="5" t="n">
-        <v>14078.71</v>
+        <v>20433.45</v>
       </c>
       <c r="G60" s="5" t="n">
         <v>115950</v>
@@ -5568,7 +5568,7 @@
     <col width="32" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
     <col width="23" customWidth="1" min="5" max="5"/>
     <col width="25" customWidth="1" min="6" max="6"/>
   </cols>
@@ -5644,13 +5644,13 @@
         <v>8373</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>4853.85</v>
+        <v>5343.73</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>3519.15</v>
+        <v>3029.27</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>0.5797026155499821</v>
+        <v>0.6382097217245909</v>
       </c>
     </row>
     <row r="4">
@@ -5740,13 +5740,13 @@
         <v>250</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>474.43</v>
+        <v>1558.83</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>-224.43</v>
+        <v>-1308.83</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>1.89772</v>
+        <v>6.23532</v>
       </c>
     </row>
     <row r="8">
@@ -5836,13 +5836,13 @@
         <v>7260</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>0</v>
+        <v>1696.3</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>7260</v>
+        <v>5563.7</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>0</v>
+        <v>0.2336501377410468</v>
       </c>
     </row>
     <row r="12">
@@ -5860,13 +5860,13 @@
         <v>54325</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>8083.71</v>
+        <v>11167.87</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>46241.29</v>
+        <v>43157.13</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0.1488027611596871</v>
+        <v>0.2055751495628164</v>
       </c>
     </row>
     <row r="13">
@@ -5927,13 +5927,13 @@
         <v>73362.32000000001</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>14078.71</v>
+        <v>20433.45</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>59283.61</v>
+        <v>52928.87</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.1919065536640608</v>
+        <v>0.2785278600785798</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-04-16 17:04:31
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -2905,7 +2905,7 @@
         <v>0</v>
       </c>
       <c r="L40" s="2" t="n">
-        <v>0</v>
+        <v>909.2</v>
       </c>
       <c r="M40" s="2" t="n">
         <v>66.09999999999999</v>
@@ -3874,7 +3874,7 @@
       </c>
       <c r="L56" s="4" t="inlineStr">
         <is>
-          <t>1 de 54</t>
+          <t>2 de 54</t>
         </is>
       </c>
       <c r="M56" s="4" t="inlineStr">
@@ -3919,7 +3919,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G60"/>
+  <dimension ref="A1:G56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5015,7 +5015,7 @@
         <v>224.96</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>2519.6</v>
+        <v>3428.8</v>
       </c>
       <c r="G40" s="2" t="n">
         <v>3500</v>
@@ -5326,23 +5326,23 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>SOLANO DE LA SALA PAZ GONZALO PATRICIO</t>
+          <t>TORO BLACIO MARIA DEL CISNE</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
-        <v>0</v>
+        <v>105.62</v>
       </c>
       <c r="D52" s="2" t="n">
-        <v>0</v>
+        <v>2465.83</v>
       </c>
       <c r="E52" s="2" t="n">
-        <v>0</v>
+        <v>834.48</v>
       </c>
       <c r="F52" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G52" s="2" t="n">
-        <v>0</v>
+        <v>1650</v>
       </c>
     </row>
     <row r="53">
@@ -5353,23 +5353,23 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>TORO BLACIO MARIA DEL CISNE</t>
+          <t>WONG SANCHEZ CLAUDIA PAULINA</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
-        <v>105.62</v>
+        <v>336.6</v>
       </c>
       <c r="D53" s="2" t="n">
-        <v>2465.83</v>
+        <v>1915.78</v>
       </c>
       <c r="E53" s="2" t="n">
-        <v>834.48</v>
+        <v>1296.86</v>
       </c>
       <c r="F53" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G53" s="2" t="n">
-        <v>1500</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="54">
@@ -5380,23 +5380,23 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>TORO BLACIO MARIA DEL CISNE</t>
+          <t>WONG SANCHEZ PAULA SOFIA</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
-        <v>105.62</v>
+        <v>0</v>
       </c>
       <c r="D54" s="2" t="n">
-        <v>2465.83</v>
+        <v>0</v>
       </c>
       <c r="E54" s="2" t="n">
-        <v>834.48</v>
+        <v>0</v>
       </c>
       <c r="F54" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G54" s="2" t="n">
-        <v>1650</v>
+        <v>0</v>
       </c>
     </row>
     <row r="55">
@@ -5407,148 +5407,40 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>WONG SANCHEZ CLAUDIA PAULINA</t>
+          <t>ZUÑIGA CORONEL MARCIA LUZMILA</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
-        <v>336.6</v>
+        <v>0</v>
       </c>
       <c r="D55" s="2" t="n">
-        <v>1915.78</v>
+        <v>0</v>
       </c>
       <c r="E55" s="2" t="n">
-        <v>1296.86</v>
+        <v>295.2</v>
       </c>
       <c r="F55" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G55" s="2" t="n">
-        <v>500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>GUERRERO FAREZ FABIAN MAURICIO</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>WONG SANCHEZ CLAUDIA PAULINA</t>
-        </is>
-      </c>
-      <c r="C56" s="2" t="n">
-        <v>336.6</v>
-      </c>
-      <c r="D56" s="2" t="n">
-        <v>1915.78</v>
-      </c>
-      <c r="E56" s="2" t="n">
-        <v>1296.86</v>
-      </c>
-      <c r="F56" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G56" s="2" t="n">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>GUERRERO FAREZ FABIAN MAURICIO</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>WONG SANCHEZ PAULA SOFIA</t>
-        </is>
-      </c>
-      <c r="C57" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D57" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E57" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F57" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G57" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>GUERRERO FAREZ FABIAN MAURICIO</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>ZUÑIGA CORONEL MARCIA LUZMILA</t>
-        </is>
-      </c>
-      <c r="C58" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D58" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E58" s="2" t="n">
-        <v>295.2</v>
-      </c>
-      <c r="F58" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G58" s="2" t="n">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>GUERRERO FAREZ FABIAN MAURICIO</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>ZUÑIGA CORONEL MARCIA LUZMILA</t>
-        </is>
-      </c>
-      <c r="C59" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D59" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E59" s="2" t="n">
-        <v>295.2</v>
-      </c>
-      <c r="F59" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G59" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="C60" s="5" t="n">
-        <v>79907.13</v>
-      </c>
-      <c r="D60" s="5" t="n">
-        <v>76363.98</v>
-      </c>
-      <c r="E60" s="5" t="n">
-        <v>79624.92</v>
-      </c>
-      <c r="F60" s="5" t="n">
-        <v>20141.2</v>
-      </c>
-      <c r="G60" s="5" t="n">
-        <v>115950</v>
+      <c r="C56" s="5" t="n">
+        <v>79464.91</v>
+      </c>
+      <c r="D56" s="5" t="n">
+        <v>71982.37</v>
+      </c>
+      <c r="E56" s="5" t="n">
+        <v>77198.38</v>
+      </c>
+      <c r="F56" s="5" t="n">
+        <v>21050.4</v>
+      </c>
+      <c r="G56" s="5" t="n">
+        <v>112950</v>
       </c>
     </row>
   </sheetData>
@@ -5836,13 +5728,13 @@
         <v>7260</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>1696.3</v>
+        <v>2605.5</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>5563.7</v>
+        <v>4654.5</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>0.2336501377410468</v>
+        <v>0.3588842975206611</v>
       </c>
     </row>
     <row r="12">
@@ -5927,13 +5819,13 @@
         <v>73362.32000000001</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>20141.2</v>
+        <v>21050.4</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>53221.12</v>
+        <v>52311.92</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.2745442074350974</v>
+        <v>0.2869374905264719</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-04-17 11:30:19
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R56"/>
+  <dimension ref="A1:R57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2634,7 +2634,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>ORTEGA ROMAN KLEBER ERWIN</t>
+          <t>OJEDA GONZALEZ EDWIN FERNANDO</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
@@ -2668,7 +2668,7 @@
         <v>0</v>
       </c>
       <c r="M36" s="2" t="n">
-        <v>-23.39</v>
+        <v>0</v>
       </c>
       <c r="N36" s="2" t="n">
         <v>0</v>
@@ -2677,7 +2677,7 @@
         <v>0</v>
       </c>
       <c r="P36" s="2" t="n">
-        <v>1558.83</v>
+        <v>0</v>
       </c>
       <c r="Q36" s="2" t="n">
         <v>0</v>
@@ -2694,7 +2694,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>ORTEGA ROMAN LUIS FERNANDO</t>
+          <t>ORTEGA ROMAN KLEBER ERWIN</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
@@ -2728,7 +2728,7 @@
         <v>0</v>
       </c>
       <c r="M37" s="2" t="n">
-        <v>1140.48</v>
+        <v>-23.39</v>
       </c>
       <c r="N37" s="2" t="n">
         <v>0</v>
@@ -2737,7 +2737,7 @@
         <v>0</v>
       </c>
       <c r="P37" s="2" t="n">
-        <v>0</v>
+        <v>1558.83</v>
       </c>
       <c r="Q37" s="2" t="n">
         <v>0</v>
@@ -2754,7 +2754,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>PACHECO NIVICELA DORIS PRICILA</t>
+          <t>ORTEGA ROMAN LUIS FERNANDO</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
@@ -2788,7 +2788,7 @@
         <v>0</v>
       </c>
       <c r="M38" s="2" t="n">
-        <v>0</v>
+        <v>1140.48</v>
       </c>
       <c r="N38" s="2" t="n">
         <v>0</v>
@@ -2814,7 +2814,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>PACHECO NIVICELA SANDRA ELISABETH</t>
+          <t>PACHECO NIVICELA DORIS PRICILA</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
@@ -2874,14 +2874,14 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>PEREZ ROSALES EDGAR RICARDO</t>
+          <t>PACHECO NIVICELA SANDRA ELISABETH</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D40" s="2" t="n">
-        <v>2453.5</v>
+        <v>0</v>
       </c>
       <c r="E40" s="2" t="n">
         <v>0</v>
@@ -2905,10 +2905,10 @@
         <v>0</v>
       </c>
       <c r="L40" s="2" t="n">
-        <v>909.2</v>
+        <v>0</v>
       </c>
       <c r="M40" s="2" t="n">
-        <v>66.09999999999999</v>
+        <v>0</v>
       </c>
       <c r="N40" s="2" t="n">
         <v>0</v>
@@ -2934,14 +2934,14 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>PEÑALOZA LOPEZ RONALD STALIN</t>
+          <t>PEREZ ROSALES EDGAR RICARDO</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D41" s="2" t="n">
-        <v>0</v>
+        <v>2453.5</v>
       </c>
       <c r="E41" s="2" t="n">
         <v>0</v>
@@ -2965,10 +2965,10 @@
         <v>0</v>
       </c>
       <c r="L41" s="2" t="n">
-        <v>0</v>
+        <v>909.2</v>
       </c>
       <c r="M41" s="2" t="n">
-        <v>0</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="N41" s="2" t="n">
         <v>0</v>
@@ -2994,7 +2994,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>QUEZADA VEGA JAIME PATRICIO</t>
+          <t>PEÑALOZA LOPEZ RONALD STALIN</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
@@ -3022,7 +3022,7 @@
         <v>0</v>
       </c>
       <c r="K42" s="2" t="n">
-        <v>101.52</v>
+        <v>0</v>
       </c>
       <c r="L42" s="2" t="n">
         <v>0</v>
@@ -3054,7 +3054,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>QUINCHE ALCIVAR ARGENTINA DEL ROCIO</t>
+          <t>QUEZADA VEGA JAIME PATRICIO</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
@@ -3082,7 +3082,7 @@
         <v>0</v>
       </c>
       <c r="K43" s="2" t="n">
-        <v>0</v>
+        <v>101.52</v>
       </c>
       <c r="L43" s="2" t="n">
         <v>0</v>
@@ -3114,7 +3114,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>RAMIREZ APOLO JOBANI DE JESUS</t>
+          <t>QUINCHE ALCIVAR ARGENTINA DEL ROCIO</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
@@ -3174,7 +3174,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>REYES MOSCOSO NARCISA DE JESUS</t>
+          <t>RAMIREZ APOLO JOBANI DE JESUS</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
@@ -3234,7 +3234,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>ROJAS SANCHEZ LADY MARGOT</t>
+          <t>REYES MOSCOSO NARCISA DE JESUS</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
@@ -3294,7 +3294,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>ROMERO RODAS SILVIA MARELIS</t>
+          <t>ROJAS SANCHEZ LADY MARGOT</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
@@ -3328,7 +3328,7 @@
         <v>0</v>
       </c>
       <c r="M47" s="2" t="n">
-        <v>1786.75</v>
+        <v>0</v>
       </c>
       <c r="N47" s="2" t="n">
         <v>0</v>
@@ -3354,14 +3354,14 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>RUIZ TINIZARAY YOHANNA MARYURI</t>
+          <t>ROMERO RODAS SILVIA MARELIS</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D48" s="2" t="n">
-        <v>2383.34</v>
+        <v>0</v>
       </c>
       <c r="E48" s="2" t="n">
         <v>0</v>
@@ -3388,7 +3388,7 @@
         <v>0</v>
       </c>
       <c r="M48" s="2" t="n">
-        <v>0</v>
+        <v>1786.75</v>
       </c>
       <c r="N48" s="2" t="n">
         <v>0</v>
@@ -3414,14 +3414,14 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>SALAS NOBLECILLA MARIA SUSANA</t>
+          <t>RUIZ TINIZARAY YOHANNA MARYURI</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D49" s="2" t="n">
-        <v>0</v>
+        <v>2383.34</v>
       </c>
       <c r="E49" s="2" t="n">
         <v>0</v>
@@ -3474,7 +3474,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>SALDARRIAGA ECHEVERRIA BRYAN STEVEN</t>
+          <t>SALAS NOBLECILLA MARIA SUSANA</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
@@ -3534,7 +3534,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>SOLANO DE LA SALA PAZ GONZALO PATRICIO</t>
+          <t>SALDARRIAGA ECHEVERRIA BRYAN STEVEN</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
@@ -3594,7 +3594,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>TORO BLACIO MARIA DEL CISNE</t>
+          <t>SOLANO DE LA SALA PAZ GONZALO PATRICIO</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
@@ -3654,7 +3654,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>WONG SANCHEZ CLAUDIA PAULINA</t>
+          <t>TORO BLACIO MARIA DEL CISNE</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
@@ -3714,7 +3714,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>WONG SANCHEZ PAULA SOFIA</t>
+          <t>WONG SANCHEZ CLAUDIA PAULINA</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
@@ -3774,137 +3774,197 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
+          <t>WONG SANCHEZ PAULA SOFIA</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R55" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>GUERRERO FAREZ FABIAN MAURICIO</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
           <t>ZUÑIGA CORONEL MARCIA LUZMILA</t>
         </is>
       </c>
-      <c r="C55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R55" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="C56" s="4" t="inlineStr">
-        <is>
-          <t>1 de 54</t>
-        </is>
-      </c>
-      <c r="D56" s="4" t="inlineStr">
-        <is>
-          <t>4 de 54</t>
-        </is>
-      </c>
-      <c r="E56" s="4" t="inlineStr">
-        <is>
-          <t>0 de 54</t>
-        </is>
-      </c>
-      <c r="F56" s="4" t="inlineStr">
-        <is>
-          <t>0 de 54</t>
-        </is>
-      </c>
-      <c r="G56" s="4" t="inlineStr">
-        <is>
-          <t>0 de 54</t>
-        </is>
-      </c>
-      <c r="H56" s="4" t="inlineStr">
-        <is>
-          <t>0 de 54</t>
-        </is>
-      </c>
-      <c r="I56" s="4" t="inlineStr">
-        <is>
-          <t>1 de 54</t>
-        </is>
-      </c>
-      <c r="J56" s="4" t="inlineStr">
-        <is>
-          <t>0 de 54</t>
-        </is>
-      </c>
-      <c r="K56" s="4" t="inlineStr">
-        <is>
-          <t>1 de 54</t>
-        </is>
-      </c>
-      <c r="L56" s="4" t="inlineStr">
-        <is>
-          <t>2 de 54</t>
-        </is>
-      </c>
-      <c r="M56" s="4" t="inlineStr">
-        <is>
-          <t>9 de 54</t>
-        </is>
-      </c>
-      <c r="N56" s="4" t="inlineStr">
-        <is>
-          <t>0 de 54</t>
-        </is>
-      </c>
-      <c r="O56" s="4" t="inlineStr">
-        <is>
-          <t>0 de 54</t>
-        </is>
-      </c>
-      <c r="P56" s="4" t="inlineStr">
-        <is>
-          <t>1 de 54</t>
-        </is>
-      </c>
-      <c r="Q56" s="4" t="inlineStr">
-        <is>
-          <t>0 de 54</t>
-        </is>
-      </c>
-      <c r="R56" s="4" t="inlineStr">
-        <is>
-          <t>0 de 54</t>
+      <c r="C56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R56" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="C57" s="4" t="inlineStr">
+        <is>
+          <t>1 de 55</t>
+        </is>
+      </c>
+      <c r="D57" s="4" t="inlineStr">
+        <is>
+          <t>4 de 55</t>
+        </is>
+      </c>
+      <c r="E57" s="4" t="inlineStr">
+        <is>
+          <t>0 de 55</t>
+        </is>
+      </c>
+      <c r="F57" s="4" t="inlineStr">
+        <is>
+          <t>0 de 55</t>
+        </is>
+      </c>
+      <c r="G57" s="4" t="inlineStr">
+        <is>
+          <t>0 de 55</t>
+        </is>
+      </c>
+      <c r="H57" s="4" t="inlineStr">
+        <is>
+          <t>0 de 55</t>
+        </is>
+      </c>
+      <c r="I57" s="4" t="inlineStr">
+        <is>
+          <t>1 de 55</t>
+        </is>
+      </c>
+      <c r="J57" s="4" t="inlineStr">
+        <is>
+          <t>0 de 55</t>
+        </is>
+      </c>
+      <c r="K57" s="4" t="inlineStr">
+        <is>
+          <t>1 de 55</t>
+        </is>
+      </c>
+      <c r="L57" s="4" t="inlineStr">
+        <is>
+          <t>2 de 55</t>
+        </is>
+      </c>
+      <c r="M57" s="4" t="inlineStr">
+        <is>
+          <t>9 de 55</t>
+        </is>
+      </c>
+      <c r="N57" s="4" t="inlineStr">
+        <is>
+          <t>0 de 55</t>
+        </is>
+      </c>
+      <c r="O57" s="4" t="inlineStr">
+        <is>
+          <t>0 de 55</t>
+        </is>
+      </c>
+      <c r="P57" s="4" t="inlineStr">
+        <is>
+          <t>1 de 55</t>
+        </is>
+      </c>
+      <c r="Q57" s="4" t="inlineStr">
+        <is>
+          <t>0 de 55</t>
+        </is>
+      </c>
+      <c r="R57" s="4" t="inlineStr">
+        <is>
+          <t>0 de 55</t>
         </is>
       </c>
     </row>
@@ -3919,7 +3979,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G56"/>
+  <dimension ref="A1:G57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4894,23 +4954,23 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>ORTEGA ROMAN KLEBER ERWIN</t>
+          <t>OJEDA GONZALEZ EDWIN FERNANDO</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
-        <v>9478.459999999999</v>
+        <v>0</v>
       </c>
       <c r="D36" s="2" t="n">
-        <v>27766.67</v>
+        <v>0</v>
       </c>
       <c r="E36" s="2" t="n">
-        <v>17480.36</v>
+        <v>0</v>
       </c>
       <c r="F36" s="2" t="n">
-        <v>1535.44</v>
+        <v>0</v>
       </c>
       <c r="G36" s="2" t="n">
-        <v>10000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37">
@@ -4921,23 +4981,23 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>ORTEGA ROMAN LUIS FERNANDO</t>
+          <t>ORTEGA ROMAN KLEBER ERWIN</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
-        <v>7485.63</v>
+        <v>9478.459999999999</v>
       </c>
       <c r="D37" s="2" t="n">
-        <v>1067.47</v>
+        <v>27766.67</v>
       </c>
       <c r="E37" s="2" t="n">
-        <v>565.25</v>
+        <v>17480.36</v>
       </c>
       <c r="F37" s="2" t="n">
-        <v>1140.48</v>
+        <v>1535.44</v>
       </c>
       <c r="G37" s="2" t="n">
-        <v>8000</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="38">
@@ -4948,23 +5008,23 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>PACHECO NIVICELA DORIS PRICILA</t>
+          <t>ORTEGA ROMAN LUIS FERNANDO</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
-        <v>0</v>
+        <v>7485.63</v>
       </c>
       <c r="D38" s="2" t="n">
-        <v>0</v>
+        <v>1067.47</v>
       </c>
       <c r="E38" s="2" t="n">
-        <v>0</v>
+        <v>565.25</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>0</v>
+        <v>1140.48</v>
       </c>
       <c r="G38" s="2" t="n">
-        <v>200</v>
+        <v>8000</v>
       </c>
     </row>
     <row r="39">
@@ -4975,7 +5035,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>PACHECO NIVICELA SANDRA ELISABETH</t>
+          <t>PACHECO NIVICELA DORIS PRICILA</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
@@ -4991,7 +5051,7 @@
         <v>0</v>
       </c>
       <c r="G39" s="2" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
     </row>
     <row r="40">
@@ -5002,23 +5062,23 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>PEREZ ROSALES EDGAR RICARDO</t>
+          <t>PACHECO NIVICELA SANDRA ELISABETH</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D40" s="2" t="n">
-        <v>221.73</v>
+        <v>0</v>
       </c>
       <c r="E40" s="2" t="n">
-        <v>224.96</v>
+        <v>0</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>3428.8</v>
+        <v>0</v>
       </c>
       <c r="G40" s="2" t="n">
-        <v>3500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41">
@@ -5029,23 +5089,23 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>PEÑALOZA LOPEZ RONALD STALIN</t>
+          <t>PEREZ ROSALES EDGAR RICARDO</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
-        <v>1579.36</v>
+        <v>0</v>
       </c>
       <c r="D41" s="2" t="n">
-        <v>0</v>
+        <v>221.73</v>
       </c>
       <c r="E41" s="2" t="n">
-        <v>1338.12</v>
+        <v>224.96</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>0</v>
+        <v>3428.8</v>
       </c>
       <c r="G41" s="2" t="n">
-        <v>1000</v>
+        <v>3500</v>
       </c>
     </row>
     <row r="42">
@@ -5056,23 +5116,23 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>QUEZADA VEGA JAIME PATRICIO</t>
+          <t>PEÑALOZA LOPEZ RONALD STALIN</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
-        <v>0</v>
+        <v>1579.36</v>
       </c>
       <c r="D42" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E42" s="2" t="n">
-        <v>1994.04</v>
+        <v>1338.12</v>
       </c>
       <c r="F42" s="2" t="n">
-        <v>101.52</v>
+        <v>0</v>
       </c>
       <c r="G42" s="2" t="n">
-        <v>2000</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="43">
@@ -5083,7 +5143,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>QUINCHE ALCIVAR ARGENTINA DEL ROCIO</t>
+          <t>QUEZADA VEGA JAIME PATRICIO</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
@@ -5093,13 +5153,13 @@
         <v>0</v>
       </c>
       <c r="E43" s="2" t="n">
-        <v>0</v>
+        <v>1994.04</v>
       </c>
       <c r="F43" s="2" t="n">
-        <v>0</v>
+        <v>101.52</v>
       </c>
       <c r="G43" s="2" t="n">
-        <v>200</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="44">
@@ -5110,7 +5170,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>RAMIREZ APOLO JOBANI DE JESUS</t>
+          <t>QUINCHE ALCIVAR ARGENTINA DEL ROCIO</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
@@ -5126,7 +5186,7 @@
         <v>0</v>
       </c>
       <c r="G44" s="2" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
     </row>
     <row r="45">
@@ -5137,23 +5197,23 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>REYES MOSCOSO NARCISA DE JESUS</t>
+          <t>RAMIREZ APOLO JOBANI DE JESUS</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D45" s="2" t="n">
-        <v>65.8</v>
+        <v>0</v>
       </c>
       <c r="E45" s="2" t="n">
-        <v>821.0599999999999</v>
+        <v>0</v>
       </c>
       <c r="F45" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G45" s="2" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46">
@@ -5164,23 +5224,23 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>ROJAS SANCHEZ LADY MARGOT</t>
+          <t>REYES MOSCOSO NARCISA DE JESUS</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
-        <v>5352.14</v>
+        <v>0</v>
       </c>
       <c r="D46" s="2" t="n">
-        <v>0</v>
+        <v>65.8</v>
       </c>
       <c r="E46" s="2" t="n">
-        <v>1260.23</v>
+        <v>821.0599999999999</v>
       </c>
       <c r="F46" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G46" s="2" t="n">
-        <v>1500</v>
+        <v>300</v>
       </c>
     </row>
     <row r="47">
@@ -5191,20 +5251,20 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>ROMERO RODAS SILVIA MARELIS</t>
+          <t>ROJAS SANCHEZ LADY MARGOT</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
-        <v>2047.8</v>
+        <v>5352.14</v>
       </c>
       <c r="D47" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>378.38</v>
+        <v>1260.23</v>
       </c>
       <c r="F47" s="2" t="n">
-        <v>1786.75</v>
+        <v>0</v>
       </c>
       <c r="G47" s="2" t="n">
         <v>1500</v>
@@ -5218,20 +5278,20 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>RUIZ TINIZARAY YOHANNA MARYURI</t>
+          <t>ROMERO RODAS SILVIA MARELIS</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
-        <v>950.4</v>
+        <v>2047.8</v>
       </c>
       <c r="D48" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>2787.07</v>
+        <v>378.38</v>
       </c>
       <c r="F48" s="2" t="n">
-        <v>2383.34</v>
+        <v>1786.75</v>
       </c>
       <c r="G48" s="2" t="n">
         <v>1500</v>
@@ -5245,23 +5305,23 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>SALAS NOBLECILLA MARIA SUSANA</t>
+          <t>RUIZ TINIZARAY YOHANNA MARYURI</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
-        <v>0</v>
+        <v>950.4</v>
       </c>
       <c r="D49" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E49" s="2" t="n">
-        <v>0</v>
+        <v>2787.07</v>
       </c>
       <c r="F49" s="2" t="n">
-        <v>0</v>
+        <v>2383.34</v>
       </c>
       <c r="G49" s="2" t="n">
-        <v>500</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="50">
@@ -5272,7 +5332,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>SALDARRIAGA ECHEVERRIA BRYAN STEVEN</t>
+          <t>SALAS NOBLECILLA MARIA SUSANA</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
@@ -5282,13 +5342,13 @@
         <v>0</v>
       </c>
       <c r="E50" s="2" t="n">
-        <v>138.2</v>
+        <v>0</v>
       </c>
       <c r="F50" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G50" s="2" t="n">
-        <v>0</v>
+        <v>500</v>
       </c>
     </row>
     <row r="51">
@@ -5299,7 +5359,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>SOLANO DE LA SALA PAZ GONZALO PATRICIO</t>
+          <t>SALDARRIAGA ECHEVERRIA BRYAN STEVEN</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
@@ -5309,7 +5369,7 @@
         <v>0</v>
       </c>
       <c r="E51" s="2" t="n">
-        <v>0</v>
+        <v>138.2</v>
       </c>
       <c r="F51" s="2" t="n">
         <v>0</v>
@@ -5326,23 +5386,23 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>TORO BLACIO MARIA DEL CISNE</t>
+          <t>SOLANO DE LA SALA PAZ GONZALO PATRICIO</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
-        <v>105.62</v>
+        <v>0</v>
       </c>
       <c r="D52" s="2" t="n">
-        <v>2465.83</v>
+        <v>0</v>
       </c>
       <c r="E52" s="2" t="n">
-        <v>834.48</v>
+        <v>0</v>
       </c>
       <c r="F52" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G52" s="2" t="n">
-        <v>1650</v>
+        <v>0</v>
       </c>
     </row>
     <row r="53">
@@ -5353,23 +5413,23 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>WONG SANCHEZ CLAUDIA PAULINA</t>
+          <t>TORO BLACIO MARIA DEL CISNE</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
-        <v>336.6</v>
+        <v>105.62</v>
       </c>
       <c r="D53" s="2" t="n">
-        <v>1915.78</v>
+        <v>2465.83</v>
       </c>
       <c r="E53" s="2" t="n">
-        <v>1296.86</v>
+        <v>834.48</v>
       </c>
       <c r="F53" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G53" s="2" t="n">
-        <v>1000</v>
+        <v>1650</v>
       </c>
     </row>
     <row r="54">
@@ -5380,23 +5440,23 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>WONG SANCHEZ PAULA SOFIA</t>
+          <t>WONG SANCHEZ CLAUDIA PAULINA</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
-        <v>0</v>
+        <v>336.6</v>
       </c>
       <c r="D54" s="2" t="n">
-        <v>0</v>
+        <v>1915.78</v>
       </c>
       <c r="E54" s="2" t="n">
-        <v>0</v>
+        <v>1296.86</v>
       </c>
       <c r="F54" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G54" s="2" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="55">
@@ -5407,39 +5467,66 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
+          <t>WONG SANCHEZ PAULA SOFIA</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G55" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>GUERRERO FAREZ FABIAN MAURICIO</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
           <t>ZUÑIGA CORONEL MARCIA LUZMILA</t>
         </is>
       </c>
-      <c r="C55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E55" s="2" t="n">
+      <c r="C56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E56" s="2" t="n">
         <v>295.2</v>
       </c>
-      <c r="F55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G55" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="C56" s="5" t="n">
+      <c r="F56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G56" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="C57" s="5" t="n">
         <v>79464.91</v>
       </c>
-      <c r="D56" s="5" t="n">
+      <c r="D57" s="5" t="n">
         <v>71982.37</v>
       </c>
-      <c r="E56" s="5" t="n">
+      <c r="E57" s="5" t="n">
         <v>77198.38</v>
       </c>
-      <c r="F56" s="5" t="n">
+      <c r="F57" s="5" t="n">
         <v>21031.31</v>
       </c>
-      <c r="G56" s="5" t="n">
+      <c r="G57" s="5" t="n">
         <v>112950</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática 2026-04-17 17:30:19
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -928,7 +928,7 @@
         <v>0</v>
       </c>
       <c r="M7" s="2" t="n">
-        <v>-40.82</v>
+        <v>1772.92</v>
       </c>
       <c r="N7" s="2" t="n">
         <v>0</v>
@@ -2173,7 +2173,7 @@
         <v>0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>0</v>
+        <v>102.6</v>
       </c>
       <c r="I28" s="2" t="n">
         <v>0</v>
@@ -2188,7 +2188,7 @@
         <v>0</v>
       </c>
       <c r="M28" s="2" t="n">
-        <v>0</v>
+        <v>2952.1</v>
       </c>
       <c r="N28" s="2" t="n">
         <v>0</v>
@@ -3914,24 +3914,24 @@
       </c>
       <c r="H57" s="4" t="inlineStr">
         <is>
+          <t>1 de 55</t>
+        </is>
+      </c>
+      <c r="I57" s="4" t="inlineStr">
+        <is>
+          <t>1 de 55</t>
+        </is>
+      </c>
+      <c r="J57" s="4" t="inlineStr">
+        <is>
           <t>0 de 55</t>
         </is>
       </c>
-      <c r="I57" s="4" t="inlineStr">
+      <c r="K57" s="4" t="inlineStr">
         <is>
           <t>1 de 55</t>
         </is>
       </c>
-      <c r="J57" s="4" t="inlineStr">
-        <is>
-          <t>0 de 55</t>
-        </is>
-      </c>
-      <c r="K57" s="4" t="inlineStr">
-        <is>
-          <t>1 de 55</t>
-        </is>
-      </c>
       <c r="L57" s="4" t="inlineStr">
         <is>
           <t>2 de 55</t>
@@ -3939,7 +3939,7 @@
       </c>
       <c r="M57" s="4" t="inlineStr">
         <is>
-          <t>9 de 55</t>
+          <t>11 de 55</t>
         </is>
       </c>
       <c r="N57" s="4" t="inlineStr">
@@ -4184,7 +4184,7 @@
         <v>4192.73</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>-40.82</v>
+        <v>1772.92</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>1500</v>
@@ -4751,7 +4751,7 @@
         <v>3991.15</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>0</v>
+        <v>3054.7</v>
       </c>
       <c r="G28" s="2" t="n">
         <v>1500</v>
@@ -5524,7 +5524,7 @@
         <v>77198.38</v>
       </c>
       <c r="F57" s="5" t="n">
-        <v>21031.31</v>
+        <v>25899.75</v>
       </c>
       <c r="G57" s="5" t="n">
         <v>112950</v>
@@ -5743,10 +5743,10 @@
         <v>0</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>0</v>
+        <v>102.6</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>0</v>
+        <v>-102.6</v>
       </c>
       <c r="F8" s="3" t="n">
         <v>0</v>
@@ -5839,13 +5839,13 @@
         <v>54325</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>10856.53</v>
+        <v>15622.37</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>43468.47</v>
+        <v>38702.63</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0.1998440865163369</v>
+        <v>0.2875723884031293</v>
       </c>
     </row>
     <row r="13">
@@ -5906,13 +5906,13 @@
         <v>73362.32000000001</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>21031.31</v>
+        <v>25899.75</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>52331.01</v>
+        <v>47462.57</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.2866772752006752</v>
+        <v>0.3530388624569125</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-04-21 11:30:21
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -721,7 +721,7 @@
         <v>129.6</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>0</v>
+        <v>944.1799999999999</v>
       </c>
       <c r="E4" s="2" t="n">
         <v>0</v>
@@ -3894,7 +3894,7 @@
       </c>
       <c r="D57" s="4" t="inlineStr">
         <is>
-          <t>4 de 55</t>
+          <t>5 de 55</t>
         </is>
       </c>
       <c r="E57" s="4" t="inlineStr">
@@ -4103,7 +4103,7 @@
         <v>4764.43</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>4194</v>
+        <v>5138.18</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>15000</v>
@@ -5524,7 +5524,7 @@
         <v>77198.38</v>
       </c>
       <c r="F57" s="5" t="n">
-        <v>25899.75</v>
+        <v>26843.93</v>
       </c>
       <c r="G57" s="5" t="n">
         <v>112950</v>
@@ -5623,13 +5623,13 @@
         <v>8373</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>5343.73</v>
+        <v>6287.91</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>3029.27</v>
+        <v>2085.09</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>0.6382097217245909</v>
+        <v>0.7509745610892153</v>
       </c>
     </row>
     <row r="4">
@@ -5906,13 +5906,13 @@
         <v>73362.32000000001</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>25899.75</v>
+        <v>26843.93</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>47462.57</v>
+        <v>46518.39</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.3530388624569125</v>
+        <v>0.3659089570776933</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-04-21 15:30:20
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -928,7 +928,7 @@
         <v>0</v>
       </c>
       <c r="M7" s="2" t="n">
-        <v>1772.92</v>
+        <v>2419.19</v>
       </c>
       <c r="N7" s="2" t="n">
         <v>0</v>
@@ -4184,7 +4184,7 @@
         <v>4192.73</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>1772.92</v>
+        <v>2419.19</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>1500</v>
@@ -5524,7 +5524,7 @@
         <v>77198.38</v>
       </c>
       <c r="F57" s="5" t="n">
-        <v>26843.93</v>
+        <v>27490.2</v>
       </c>
       <c r="G57" s="5" t="n">
         <v>112950</v>
@@ -5839,13 +5839,13 @@
         <v>54325</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>15622.37</v>
+        <v>16268.64</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>38702.63</v>
+        <v>38056.36</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0.2875723884031293</v>
+        <v>0.299468752876208</v>
       </c>
     </row>
     <row r="13">
@@ -5906,13 +5906,13 @@
         <v>73362.32000000001</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>26843.93</v>
+        <v>27490.2</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>46518.39</v>
+        <v>45872.12</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.3659089570776933</v>
+        <v>0.3747182477326235</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-04-21 17:30:20
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -1948,7 +1948,7 @@
         <v>0</v>
       </c>
       <c r="M24" s="2" t="n">
-        <v>1206.63</v>
+        <v>1870.28</v>
       </c>
       <c r="N24" s="2" t="n">
         <v>0</v>
@@ -2242,7 +2242,7 @@
         <v>0</v>
       </c>
       <c r="K29" s="2" t="n">
-        <v>0</v>
+        <v>101.52</v>
       </c>
       <c r="L29" s="2" t="n">
         <v>0</v>
@@ -3929,7 +3929,7 @@
       </c>
       <c r="K57" s="4" t="inlineStr">
         <is>
-          <t>1 de 55</t>
+          <t>2 de 55</t>
         </is>
       </c>
       <c r="L57" s="4" t="inlineStr">
@@ -4643,7 +4643,7 @@
         <v>2711.11</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>1206.63</v>
+        <v>1870.28</v>
       </c>
       <c r="G24" s="2" t="n">
         <v>15000</v>
@@ -4778,7 +4778,7 @@
         <v>8735.280000000001</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>477.62</v>
+        <v>579.14</v>
       </c>
       <c r="G29" s="2" t="n">
         <v>6000</v>
@@ -5524,7 +5524,7 @@
         <v>77198.38</v>
       </c>
       <c r="F57" s="5" t="n">
-        <v>27490.2</v>
+        <v>28255.37</v>
       </c>
       <c r="G57" s="5" t="n">
         <v>112950</v>
@@ -5549,7 +5549,7 @@
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="23" customWidth="1" min="5" max="5"/>
-    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5767,13 +5767,13 @@
         <v>1300</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>101.52</v>
+        <v>203.04</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>1198.48</v>
+        <v>1096.96</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>0.07809230769230768</v>
+        <v>0.1561846153846154</v>
       </c>
     </row>
     <row r="10">
@@ -5839,13 +5839,13 @@
         <v>54325</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>16268.64</v>
+        <v>16932.29</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>38056.36</v>
+        <v>37392.71</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0.299468752876208</v>
+        <v>0.3116850437183618</v>
       </c>
     </row>
     <row r="13">
@@ -5906,13 +5906,13 @@
         <v>73362.32000000001</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>27490.2</v>
+        <v>28255.37</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>45872.12</v>
+        <v>45106.95</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.3747182477326235</v>
+        <v>0.3851482613963135</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-04-22 16:30:22
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -2188,7 +2188,7 @@
         <v>0</v>
       </c>
       <c r="M28" s="2" t="n">
-        <v>2952.1</v>
+        <v>3004.07</v>
       </c>
       <c r="N28" s="2" t="n">
         <v>0</v>
@@ -4751,7 +4751,7 @@
         <v>3991.15</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>3054.7</v>
+        <v>3106.67</v>
       </c>
       <c r="G28" s="2" t="n">
         <v>1500</v>
@@ -5524,7 +5524,7 @@
         <v>77198.38</v>
       </c>
       <c r="F57" s="5" t="n">
-        <v>28204.39</v>
+        <v>28256.36</v>
       </c>
       <c r="G57" s="5" t="n">
         <v>112950</v>
@@ -5839,13 +5839,13 @@
         <v>54325</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>16881.31</v>
+        <v>16933.28</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>37443.69</v>
+        <v>37391.72</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0.3107466175793834</v>
+        <v>0.3117032673722964</v>
       </c>
     </row>
     <row r="13">
@@ -5906,13 +5906,13 @@
         <v>73362.32000000001</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>28204.39</v>
+        <v>28256.36</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>45157.93</v>
+        <v>45105.96</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.3844533542559723</v>
+        <v>0.3851617560622401</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-04-22 17:30:22
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -808,7 +808,7 @@
         <v>1696.3</v>
       </c>
       <c r="M5" s="2" t="n">
-        <v>0.2</v>
+        <v>4983.75</v>
       </c>
       <c r="N5" s="2" t="n">
         <v>0</v>
@@ -1225,7 +1225,7 @@
         <v>0</v>
       </c>
       <c r="L12" s="2" t="n">
-        <v>0</v>
+        <v>261.27</v>
       </c>
       <c r="M12" s="2" t="n">
         <v>0</v>
@@ -2248,7 +2248,7 @@
         <v>0</v>
       </c>
       <c r="M29" s="2" t="n">
-        <v>25.01</v>
+        <v>2305.97</v>
       </c>
       <c r="N29" s="2" t="n">
         <v>0</v>
@@ -2662,7 +2662,7 @@
         <v>0</v>
       </c>
       <c r="K36" s="2" t="n">
-        <v>0</v>
+        <v>45.68</v>
       </c>
       <c r="L36" s="2" t="n">
         <v>0</v>
@@ -3929,12 +3929,12 @@
       </c>
       <c r="K57" s="4" t="inlineStr">
         <is>
-          <t>2 de 55</t>
+          <t>3 de 55</t>
         </is>
       </c>
       <c r="L57" s="4" t="inlineStr">
         <is>
-          <t>2 de 55</t>
+          <t>3 de 55</t>
         </is>
       </c>
       <c r="M57" s="4" t="inlineStr">
@@ -4130,7 +4130,7 @@
         <v>12980.37</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>1696.5</v>
+        <v>6680.05</v>
       </c>
       <c r="G5" s="2" t="n">
         <v>10000</v>
@@ -4319,7 +4319,7 @@
         <v>0</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>0</v>
+        <v>261.27</v>
       </c>
       <c r="G12" s="2" t="n">
         <v>3000</v>
@@ -4778,7 +4778,7 @@
         <v>8735.280000000001</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>579.14</v>
+        <v>2860.1</v>
       </c>
       <c r="G29" s="2" t="n">
         <v>6000</v>
@@ -4967,7 +4967,7 @@
         <v>0</v>
       </c>
       <c r="F36" s="2" t="n">
-        <v>0</v>
+        <v>45.68</v>
       </c>
       <c r="G36" s="2" t="n">
         <v>0</v>
@@ -5524,7 +5524,7 @@
         <v>77198.38</v>
       </c>
       <c r="F57" s="5" t="n">
-        <v>28256.36</v>
+        <v>35827.82</v>
       </c>
       <c r="G57" s="5" t="n">
         <v>112950</v>
@@ -5767,13 +5767,13 @@
         <v>1300</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>203.04</v>
+        <v>248.72</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>1096.96</v>
+        <v>1051.28</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>0.1561846153846154</v>
+        <v>0.1913230769230769</v>
       </c>
     </row>
     <row r="10">
@@ -5815,13 +5815,13 @@
         <v>7260</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>2605.5</v>
+        <v>2866.77</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>4654.5</v>
+        <v>4393.23</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>0.3588842975206611</v>
+        <v>0.3948719008264463</v>
       </c>
     </row>
     <row r="12">
@@ -5839,13 +5839,13 @@
         <v>54325</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>16933.28</v>
+        <v>24197.79</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>37391.72</v>
+        <v>30127.21</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0.3117032673722964</v>
+        <v>0.4454264150943396</v>
       </c>
     </row>
     <row r="13">
@@ -5906,13 +5906,13 @@
         <v>73362.32000000001</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>28256.36</v>
+        <v>35827.82</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>45105.96</v>
+        <v>37534.5</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.3851617560622401</v>
+        <v>0.4883681432103019</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-04-23 16:30:23
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -3748,7 +3748,7 @@
         <v>0</v>
       </c>
       <c r="M54" s="2" t="n">
-        <v>0</v>
+        <v>45.9</v>
       </c>
       <c r="N54" s="2" t="n">
         <v>0</v>
@@ -3939,7 +3939,7 @@
       </c>
       <c r="M57" s="4" t="inlineStr">
         <is>
-          <t>11 de 55</t>
+          <t>12 de 55</t>
         </is>
       </c>
       <c r="N57" s="4" t="inlineStr">
@@ -5453,7 +5453,7 @@
         <v>1296.86</v>
       </c>
       <c r="F54" s="2" t="n">
-        <v>0</v>
+        <v>45.9</v>
       </c>
       <c r="G54" s="2" t="n">
         <v>1000</v>
@@ -5524,7 +5524,7 @@
         <v>77198.38</v>
       </c>
       <c r="F57" s="5" t="n">
-        <v>35827.82</v>
+        <v>35873.72</v>
       </c>
       <c r="G57" s="5" t="n">
         <v>112950</v>
@@ -5839,13 +5839,13 @@
         <v>54325</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>24197.79</v>
+        <v>24243.69</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>30127.21</v>
+        <v>30081.31</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0.4454264150943396</v>
+        <v>0.4462713299585826</v>
       </c>
     </row>
     <row r="13">
@@ -5906,13 +5906,13 @@
         <v>73362.32000000001</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>35827.82</v>
+        <v>35873.72</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>37534.5</v>
+        <v>37488.6</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.4883681432103019</v>
+        <v>0.4889938049941714</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-04-24 15:30:23
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -1588,7 +1588,7 @@
         <v>0</v>
       </c>
       <c r="M18" s="2" t="n">
-        <v>0</v>
+        <v>103.94</v>
       </c>
       <c r="N18" s="2" t="n">
         <v>0</v>
@@ -2968,7 +2968,7 @@
         <v>909.2</v>
       </c>
       <c r="M41" s="2" t="n">
-        <v>66.09999999999999</v>
+        <v>410.38</v>
       </c>
       <c r="N41" s="2" t="n">
         <v>0</v>
@@ -3939,7 +3939,7 @@
       </c>
       <c r="M57" s="4" t="inlineStr">
         <is>
-          <t>12 de 55</t>
+          <t>13 de 55</t>
         </is>
       </c>
       <c r="N57" s="4" t="inlineStr">
@@ -4481,7 +4481,7 @@
         <v>0</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>0</v>
+        <v>103.94</v>
       </c>
       <c r="G18" s="2" t="n">
         <v>3000</v>
@@ -5102,7 +5102,7 @@
         <v>224.96</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>3428.8</v>
+        <v>3773.08</v>
       </c>
       <c r="G41" s="2" t="n">
         <v>3500</v>
@@ -5524,7 +5524,7 @@
         <v>77198.38</v>
       </c>
       <c r="F57" s="5" t="n">
-        <v>35873.72</v>
+        <v>36321.94</v>
       </c>
       <c r="G57" s="5" t="n">
         <v>112950</v>
@@ -5839,13 +5839,13 @@
         <v>54325</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>24243.69</v>
+        <v>24691.91</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>30081.31</v>
+        <v>29633.09</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0.4462713299585826</v>
+        <v>0.4545220432581684</v>
       </c>
     </row>
     <row r="13">
@@ -5906,13 +5906,13 @@
         <v>73362.32000000001</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>35873.72</v>
+        <v>36321.94</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>37488.6</v>
+        <v>37040.38</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.4889938049941714</v>
+        <v>0.4951034809149983</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-04-28 15:30:18
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -808,7 +808,7 @@
         <v>1696.3</v>
       </c>
       <c r="M5" s="2" t="n">
-        <v>4983.75</v>
+        <v>5045.45</v>
       </c>
       <c r="N5" s="2" t="n">
         <v>0</v>
@@ -4130,7 +4130,7 @@
         <v>12980.37</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>6680.05</v>
+        <v>6741.75</v>
       </c>
       <c r="G5" s="2" t="n">
         <v>10000</v>
@@ -5524,7 +5524,7 @@
         <v>77198.38</v>
       </c>
       <c r="F57" s="5" t="n">
-        <v>45521.14</v>
+        <v>45582.84</v>
       </c>
       <c r="G57" s="5" t="n">
         <v>112950</v>
@@ -5839,13 +5839,13 @@
         <v>54325</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>33328.71</v>
+        <v>33390.41</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>20996.29</v>
+        <v>20934.59</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0.6135059364933272</v>
+        <v>0.6146416935112748</v>
       </c>
     </row>
     <row r="13">
@@ -5906,13 +5906,13 @@
         <v>73362.32000000001</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>45521.14</v>
+        <v>45582.84</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>27841.18</v>
+        <v>27779.48</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.6204975524220062</v>
+        <v>0.6213385836216739</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-04-28 16:30:19
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -1288,7 +1288,7 @@
         <v>0</v>
       </c>
       <c r="M13" s="2" t="n">
-        <v>0</v>
+        <v>4948.24</v>
       </c>
       <c r="N13" s="2" t="n">
         <v>0</v>
@@ -3939,7 +3939,7 @@
       </c>
       <c r="M57" s="4" t="inlineStr">
         <is>
-          <t>14 de 55</t>
+          <t>15 de 55</t>
         </is>
       </c>
       <c r="N57" s="4" t="inlineStr">
@@ -4346,7 +4346,7 @@
         <v>0</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>0</v>
+        <v>4948.24</v>
       </c>
       <c r="G13" s="2" t="n">
         <v>6000</v>
@@ -5524,7 +5524,7 @@
         <v>77198.38</v>
       </c>
       <c r="F57" s="5" t="n">
-        <v>45582.84</v>
+        <v>50531.08</v>
       </c>
       <c r="G57" s="5" t="n">
         <v>112950</v>
@@ -5839,13 +5839,13 @@
         <v>54325</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>33390.41</v>
+        <v>38338.65</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>20934.59</v>
+        <v>15986.35</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0.6146416935112748</v>
+        <v>0.7057275655775426</v>
       </c>
     </row>
     <row r="13">
@@ -5906,13 +5906,13 @@
         <v>73362.32000000001</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>45582.84</v>
+        <v>50531.08</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>27779.48</v>
+        <v>22831.24</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.6213385836216739</v>
+        <v>0.6887879227374488</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-04-29 09:30:20
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -724,7 +724,7 @@
         <v>944.1799999999999</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>0</v>
+        <v>64.81999999999999</v>
       </c>
       <c r="F4" s="2" t="n">
         <v>0</v>
@@ -3899,7 +3899,7 @@
       </c>
       <c r="E57" s="4" t="inlineStr">
         <is>
-          <t>0 de 55</t>
+          <t>1 de 55</t>
         </is>
       </c>
       <c r="F57" s="4" t="inlineStr">
@@ -4103,7 +4103,7 @@
         <v>4764.43</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>5822.67</v>
+        <v>5887.49</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>15000</v>
@@ -5524,7 +5524,7 @@
         <v>77198.38</v>
       </c>
       <c r="F57" s="5" t="n">
-        <v>50513.8</v>
+        <v>50578.62</v>
       </c>
       <c r="G57" s="5" t="n">
         <v>112950</v>
@@ -5647,13 +5647,13 @@
         <v>199.5</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>0</v>
+        <v>64.81999999999999</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>199.5</v>
+        <v>134.68</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>0</v>
+        <v>0.3249122807017544</v>
       </c>
     </row>
     <row r="5">
@@ -5906,13 +5906,13 @@
         <v>73362.32000000001</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>50513.8</v>
+        <v>50578.62</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>22848.52</v>
+        <v>22783.7</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.6885523794776391</v>
+        <v>0.6894359393214391</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-04-30 11:30:21
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -805,7 +805,7 @@
         <v>0</v>
       </c>
       <c r="L5" s="2" t="n">
-        <v>1696.3</v>
+        <v>2857.36</v>
       </c>
       <c r="M5" s="2" t="n">
         <v>5028.17</v>
@@ -1225,7 +1225,7 @@
         <v>0</v>
       </c>
       <c r="L12" s="2" t="n">
-        <v>261.27</v>
+        <v>783.8200000000001</v>
       </c>
       <c r="M12" s="2" t="n">
         <v>0</v>
@@ -2257,7 +2257,7 @@
         <v>0</v>
       </c>
       <c r="P29" s="2" t="n">
-        <v>0</v>
+        <v>84.23999999999999</v>
       </c>
       <c r="Q29" s="2" t="n">
         <v>0</v>
@@ -3088,7 +3088,7 @@
         <v>0</v>
       </c>
       <c r="M43" s="2" t="n">
-        <v>0</v>
+        <v>1736.38</v>
       </c>
       <c r="N43" s="2" t="n">
         <v>0</v>
@@ -3939,7 +3939,7 @@
       </c>
       <c r="M57" s="4" t="inlineStr">
         <is>
-          <t>15 de 55</t>
+          <t>16 de 55</t>
         </is>
       </c>
       <c r="N57" s="4" t="inlineStr">
@@ -3954,7 +3954,7 @@
       </c>
       <c r="P57" s="4" t="inlineStr">
         <is>
-          <t>1 de 55</t>
+          <t>2 de 55</t>
         </is>
       </c>
       <c r="Q57" s="4" t="inlineStr">
@@ -4130,7 +4130,7 @@
         <v>12980.37</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>6724.47</v>
+        <v>7885.53</v>
       </c>
       <c r="G5" s="2" t="n">
         <v>10000</v>
@@ -4319,7 +4319,7 @@
         <v>0</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>261.27</v>
+        <v>783.8200000000001</v>
       </c>
       <c r="G12" s="2" t="n">
         <v>3000</v>
@@ -4778,7 +4778,7 @@
         <v>8735.280000000001</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>2860.1</v>
+        <v>2944.34</v>
       </c>
       <c r="G29" s="2" t="n">
         <v>6000</v>
@@ -4967,7 +4967,7 @@
         <v>0</v>
       </c>
       <c r="F36" s="2" t="n">
-        <v>45.68</v>
+        <v>134.89</v>
       </c>
       <c r="G36" s="2" t="n">
         <v>0</v>
@@ -5156,7 +5156,7 @@
         <v>1994.04</v>
       </c>
       <c r="F43" s="2" t="n">
-        <v>81.22</v>
+        <v>1817.6</v>
       </c>
       <c r="G43" s="2" t="n">
         <v>2000</v>
@@ -5524,7 +5524,7 @@
         <v>77198.38</v>
       </c>
       <c r="F57" s="5" t="n">
-        <v>51123.9</v>
+        <v>54717.34</v>
       </c>
       <c r="G57" s="5" t="n">
         <v>112950</v>
@@ -5719,13 +5719,13 @@
         <v>250</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>1558.83</v>
+        <v>1643.07</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>-1308.83</v>
+        <v>-1393.07</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>6.23532</v>
+        <v>6.57228</v>
       </c>
     </row>
     <row r="8">
@@ -5791,13 +5791,13 @@
         <v>550</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0</v>
+        <v>89.20999999999999</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>550</v>
+        <v>460.79</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>0</v>
+        <v>0.1622</v>
       </c>
     </row>
     <row r="11">
@@ -5815,13 +5815,13 @@
         <v>7260</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>3449.47</v>
+        <v>5133.08</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>3810.53</v>
+        <v>2126.92</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>0.475133608815427</v>
+        <v>0.7070358126721763</v>
       </c>
     </row>
     <row r="12">
@@ -5839,13 +5839,13 @@
         <v>54325</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>38866.65</v>
+        <v>40603.03</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>15458.35</v>
+        <v>13721.97</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0.715446847676024</v>
+        <v>0.7474096640589047</v>
       </c>
     </row>
     <row r="13">
@@ -5906,13 +5906,13 @@
         <v>73362.32000000001</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>51123.9</v>
+        <v>54717.34</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>22238.42</v>
+        <v>18644.98</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.6968686377420997</v>
+        <v>0.7458507310019639</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-05-05 17:30:21
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -724,7 +724,7 @@
         <v>0</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>0</v>
+        <v>73.09</v>
       </c>
       <c r="F4" s="2" t="n">
         <v>0</v>
@@ -1444,7 +1444,7 @@
         <v>0</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>0</v>
+        <v>453.71</v>
       </c>
       <c r="F16" s="2" t="n">
         <v>0</v>
@@ -1681,7 +1681,7 @@
         <v>0</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>0</v>
+        <v>314.73</v>
       </c>
       <c r="E20" s="2" t="n">
         <v>0</v>
@@ -1708,7 +1708,7 @@
         <v>0</v>
       </c>
       <c r="M20" s="2" t="n">
-        <v>0</v>
+        <v>1891.81</v>
       </c>
       <c r="N20" s="2" t="n">
         <v>0</v>
@@ -1918,10 +1918,10 @@
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>0</v>
+        <v>293.76</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>0</v>
+        <v>786.8200000000001</v>
       </c>
       <c r="E24" s="2" t="n">
         <v>0</v>
@@ -3889,57 +3889,57 @@
     <row r="57">
       <c r="C57" s="4" t="inlineStr">
         <is>
+          <t>1 de 55</t>
+        </is>
+      </c>
+      <c r="D57" s="4" t="inlineStr">
+        <is>
+          <t>2 de 55</t>
+        </is>
+      </c>
+      <c r="E57" s="4" t="inlineStr">
+        <is>
+          <t>2 de 55</t>
+        </is>
+      </c>
+      <c r="F57" s="4" t="inlineStr">
+        <is>
           <t>0 de 55</t>
         </is>
       </c>
-      <c r="D57" s="4" t="inlineStr">
+      <c r="G57" s="4" t="inlineStr">
         <is>
           <t>0 de 55</t>
         </is>
       </c>
-      <c r="E57" s="4" t="inlineStr">
+      <c r="H57" s="4" t="inlineStr">
         <is>
           <t>0 de 55</t>
         </is>
       </c>
-      <c r="F57" s="4" t="inlineStr">
+      <c r="I57" s="4" t="inlineStr">
         <is>
           <t>0 de 55</t>
         </is>
       </c>
-      <c r="G57" s="4" t="inlineStr">
+      <c r="J57" s="4" t="inlineStr">
         <is>
           <t>0 de 55</t>
         </is>
       </c>
-      <c r="H57" s="4" t="inlineStr">
+      <c r="K57" s="4" t="inlineStr">
         <is>
           <t>0 de 55</t>
         </is>
       </c>
-      <c r="I57" s="4" t="inlineStr">
+      <c r="L57" s="4" t="inlineStr">
         <is>
           <t>0 de 55</t>
         </is>
       </c>
-      <c r="J57" s="4" t="inlineStr">
-        <is>
-          <t>0 de 55</t>
-        </is>
-      </c>
-      <c r="K57" s="4" t="inlineStr">
-        <is>
-          <t>0 de 55</t>
-        </is>
-      </c>
-      <c r="L57" s="4" t="inlineStr">
-        <is>
-          <t>0 de 55</t>
-        </is>
-      </c>
       <c r="M57" s="4" t="inlineStr">
         <is>
-          <t>0 de 55</t>
+          <t>1 de 55</t>
         </is>
       </c>
       <c r="N57" s="4" t="inlineStr">
@@ -3987,7 +3987,7 @@
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -4103,7 +4103,7 @@
         <v>5887.49</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>0</v>
+        <v>73.09</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>15000</v>
@@ -4427,7 +4427,7 @@
         <v>3550.11</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>0</v>
+        <v>453.71</v>
       </c>
       <c r="G16" s="2" t="n">
         <v>6000</v>
@@ -4535,7 +4535,7 @@
         <v>0</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>0</v>
+        <v>2206.54</v>
       </c>
       <c r="G20" s="2" t="n">
         <v>500</v>
@@ -4643,7 +4643,7 @@
         <v>2398.13</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>0</v>
+        <v>1080.58</v>
       </c>
       <c r="G24" s="2" t="n">
         <v>15000</v>
@@ -5632,7 +5632,7 @@
         <v>55560.07</v>
       </c>
       <c r="F61" s="5" t="n">
-        <v>0</v>
+        <v>3813.92</v>
       </c>
       <c r="G61" s="5" t="n">
         <v>115950</v>

</xml_diff>

<commit_message>
Actualización automática 2026-05-07 13:30:22
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -3748,7 +3748,7 @@
         <v>0</v>
       </c>
       <c r="M54" s="2" t="n">
-        <v>0</v>
+        <v>1621.56</v>
       </c>
       <c r="N54" s="2" t="n">
         <v>0</v>
@@ -3939,7 +3939,7 @@
       </c>
       <c r="M57" s="4" t="inlineStr">
         <is>
-          <t>2 de 55</t>
+          <t>3 de 55</t>
         </is>
       </c>
       <c r="N57" s="4" t="inlineStr">
@@ -5912,7 +5912,7 @@
         <v>137.71</v>
       </c>
       <c r="F71" s="2" t="n">
-        <v>0</v>
+        <v>1621.56</v>
       </c>
       <c r="G71" s="2" t="n">
         <v>1000</v>
@@ -5983,7 +5983,7 @@
         <v>55422.36</v>
       </c>
       <c r="F74" s="5" t="n">
-        <v>3905.22</v>
+        <v>5526.78</v>
       </c>
       <c r="G74" s="5" t="n">
         <v>113950</v>

</xml_diff>

<commit_message>
Actualización automática 2026-05-11 16:30:26
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -724,7 +724,7 @@
         <v>0</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>8.27</v>
+        <v>73.09</v>
       </c>
       <c r="F4" s="2" t="n">
         <v>0</v>
@@ -748,7 +748,7 @@
         <v>0</v>
       </c>
       <c r="M4" s="2" t="n">
-        <v>66.09999999999999</v>
+        <v>112.48</v>
       </c>
       <c r="N4" s="2" t="n">
         <v>0</v>
@@ -1756,7 +1756,7 @@
         <v>0</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>0</v>
+        <v>91</v>
       </c>
       <c r="J21" s="2" t="n">
         <v>0</v>
@@ -1888,7 +1888,7 @@
         <v>0</v>
       </c>
       <c r="M23" s="2" t="n">
-        <v>0</v>
+        <v>1154.74</v>
       </c>
       <c r="N23" s="2" t="n">
         <v>0</v>
@@ -2593,10 +2593,10 @@
         <v>0</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>0</v>
+        <v>55.3</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>0</v>
+        <v>20.3</v>
       </c>
       <c r="J35" s="2" t="n">
         <v>0</v>
@@ -2608,7 +2608,7 @@
         <v>0</v>
       </c>
       <c r="M35" s="2" t="n">
-        <v>0</v>
+        <v>9576.4</v>
       </c>
       <c r="N35" s="2" t="n">
         <v>0</v>
@@ -3914,32 +3914,32 @@
       </c>
       <c r="H57" s="4" t="inlineStr">
         <is>
+          <t>1 de 55</t>
+        </is>
+      </c>
+      <c r="I57" s="4" t="inlineStr">
+        <is>
+          <t>3 de 55</t>
+        </is>
+      </c>
+      <c r="J57" s="4" t="inlineStr">
+        <is>
           <t>0 de 55</t>
         </is>
       </c>
-      <c r="I57" s="4" t="inlineStr">
-        <is>
-          <t>1 de 55</t>
-        </is>
-      </c>
-      <c r="J57" s="4" t="inlineStr">
+      <c r="K57" s="4" t="inlineStr">
         <is>
           <t>0 de 55</t>
         </is>
       </c>
-      <c r="K57" s="4" t="inlineStr">
+      <c r="L57" s="4" t="inlineStr">
         <is>
           <t>0 de 55</t>
         </is>
       </c>
-      <c r="L57" s="4" t="inlineStr">
-        <is>
-          <t>0 de 55</t>
-        </is>
-      </c>
       <c r="M57" s="4" t="inlineStr">
         <is>
-          <t>3 de 55</t>
+          <t>5 de 55</t>
         </is>
       </c>
       <c r="N57" s="4" t="inlineStr">
@@ -4103,7 +4103,7 @@
         <v>5887.49</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>74.37</v>
+        <v>185.57</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>15000</v>
@@ -4697,7 +4697,7 @@
         <v>0</v>
       </c>
       <c r="F26" s="2" t="n">
-        <v>0</v>
+        <v>91</v>
       </c>
       <c r="G26" s="2" t="n">
         <v>0</v>
@@ -4778,7 +4778,7 @@
         <v>2398.13</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>1080.58</v>
+        <v>2235.32</v>
       </c>
       <c r="G29" s="2" t="n">
         <v>15000</v>
@@ -5237,7 +5237,7 @@
         <v>1535.44</v>
       </c>
       <c r="F46" s="2" t="n">
-        <v>0</v>
+        <v>9652</v>
       </c>
       <c r="G46" s="2" t="n">
         <v>10000</v>
@@ -5983,7 +5983,7 @@
         <v>55422.36</v>
       </c>
       <c r="F74" s="5" t="n">
-        <v>5445.07</v>
+        <v>16454.01</v>
       </c>
       <c r="G74" s="5" t="n">
         <v>113950</v>

</xml_diff>

<commit_message>
Actualización automática 2026-05-11 17:30:18
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -2542,7 +2542,7 @@
         <v>0</v>
       </c>
       <c r="K34" s="2" t="n">
-        <v>0</v>
+        <v>50.76</v>
       </c>
       <c r="L34" s="2" t="n">
         <v>0</v>
@@ -2602,7 +2602,7 @@
         <v>0</v>
       </c>
       <c r="K35" s="2" t="n">
-        <v>0</v>
+        <v>45.68</v>
       </c>
       <c r="L35" s="2" t="n">
         <v>0</v>
@@ -3929,7 +3929,7 @@
       </c>
       <c r="K57" s="4" t="inlineStr">
         <is>
-          <t>0 de 55</t>
+          <t>2 de 55</t>
         </is>
       </c>
       <c r="L57" s="4" t="inlineStr">
@@ -5210,7 +5210,7 @@
         <v>134.89</v>
       </c>
       <c r="F45" s="2" t="n">
-        <v>0</v>
+        <v>50.76</v>
       </c>
       <c r="G45" s="2" t="n">
         <v>0</v>
@@ -5237,7 +5237,7 @@
         <v>1535.44</v>
       </c>
       <c r="F46" s="2" t="n">
-        <v>9652</v>
+        <v>9697.68</v>
       </c>
       <c r="G46" s="2" t="n">
         <v>10000</v>
@@ -5983,7 +5983,7 @@
         <v>55422.36</v>
       </c>
       <c r="F74" s="5" t="n">
-        <v>16454.01</v>
+        <v>16550.45</v>
       </c>
       <c r="G74" s="5" t="n">
         <v>113950</v>

</xml_diff>

<commit_message>
Actualización automática 2026-05-12 17:30:18
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -868,7 +868,7 @@
         <v>0</v>
       </c>
       <c r="M6" s="2" t="n">
-        <v>0</v>
+        <v>2157.05</v>
       </c>
       <c r="N6" s="2" t="n">
         <v>0</v>
@@ -1201,7 +1201,7 @@
         <v>0</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>0</v>
+        <v>393.41</v>
       </c>
       <c r="E12" s="2" t="n">
         <v>0</v>
@@ -1408,7 +1408,7 @@
         <v>0</v>
       </c>
       <c r="M15" s="2" t="n">
-        <v>0</v>
+        <v>1026.04</v>
       </c>
       <c r="N15" s="2" t="n">
         <v>0</v>
@@ -3894,52 +3894,52 @@
       </c>
       <c r="D57" s="4" t="inlineStr">
         <is>
+          <t>3 de 55</t>
+        </is>
+      </c>
+      <c r="E57" s="4" t="inlineStr">
+        <is>
           <t>2 de 55</t>
         </is>
       </c>
-      <c r="E57" s="4" t="inlineStr">
+      <c r="F57" s="4" t="inlineStr">
+        <is>
+          <t>0 de 55</t>
+        </is>
+      </c>
+      <c r="G57" s="4" t="inlineStr">
+        <is>
+          <t>0 de 55</t>
+        </is>
+      </c>
+      <c r="H57" s="4" t="inlineStr">
+        <is>
+          <t>1 de 55</t>
+        </is>
+      </c>
+      <c r="I57" s="4" t="inlineStr">
+        <is>
+          <t>3 de 55</t>
+        </is>
+      </c>
+      <c r="J57" s="4" t="inlineStr">
+        <is>
+          <t>0 de 55</t>
+        </is>
+      </c>
+      <c r="K57" s="4" t="inlineStr">
         <is>
           <t>2 de 55</t>
         </is>
       </c>
-      <c r="F57" s="4" t="inlineStr">
+      <c r="L57" s="4" t="inlineStr">
         <is>
           <t>0 de 55</t>
         </is>
       </c>
-      <c r="G57" s="4" t="inlineStr">
-        <is>
-          <t>0 de 55</t>
-        </is>
-      </c>
-      <c r="H57" s="4" t="inlineStr">
-        <is>
-          <t>1 de 55</t>
-        </is>
-      </c>
-      <c r="I57" s="4" t="inlineStr">
-        <is>
-          <t>3 de 55</t>
-        </is>
-      </c>
-      <c r="J57" s="4" t="inlineStr">
-        <is>
-          <t>0 de 55</t>
-        </is>
-      </c>
-      <c r="K57" s="4" t="inlineStr">
-        <is>
-          <t>2 de 55</t>
-        </is>
-      </c>
-      <c r="L57" s="4" t="inlineStr">
-        <is>
-          <t>0 de 55</t>
-        </is>
-      </c>
       <c r="M57" s="4" t="inlineStr">
         <is>
-          <t>5 de 55</t>
+          <t>7 de 55</t>
         </is>
       </c>
       <c r="N57" s="4" t="inlineStr">
@@ -4184,7 +4184,7 @@
         <v>0</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>0</v>
+        <v>2157.05</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>1500</v>
@@ -4373,7 +4373,7 @@
         <v>783.8200000000001</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>0</v>
+        <v>393.41</v>
       </c>
       <c r="G14" s="2" t="n">
         <v>3000</v>
@@ -4454,7 +4454,7 @@
         <v>3550.11</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>453.71</v>
+        <v>1479.75</v>
       </c>
       <c r="G17" s="2" t="n">
         <v>6000</v>
@@ -5983,7 +5983,7 @@
         <v>55422.36</v>
       </c>
       <c r="F74" s="5" t="n">
-        <v>16550.45</v>
+        <v>20126.95</v>
       </c>
       <c r="G74" s="5" t="n">
         <v>113950</v>

</xml_diff>

<commit_message>
Actualización automática 2026-05-13 08:30:19
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -3028,7 +3028,7 @@
         <v>0</v>
       </c>
       <c r="M42" s="2" t="n">
-        <v>0</v>
+        <v>-78.92</v>
       </c>
       <c r="N42" s="2" t="n">
         <v>0</v>
@@ -5480,7 +5480,7 @@
         <v>1817.6</v>
       </c>
       <c r="F55" s="2" t="n">
-        <v>0</v>
+        <v>-78.92</v>
       </c>
       <c r="G55" s="2" t="n">
         <v>2000</v>
@@ -5983,7 +5983,7 @@
         <v>55422.36</v>
       </c>
       <c r="F74" s="5" t="n">
-        <v>20126.95</v>
+        <v>20048.03</v>
       </c>
       <c r="G74" s="5" t="n">
         <v>113950</v>

</xml_diff>

<commit_message>
Actualización automática 2026-05-15 17:30:17
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -2368,7 +2368,7 @@
         <v>0</v>
       </c>
       <c r="M31" s="2" t="n">
-        <v>0</v>
+        <v>-56.22</v>
       </c>
       <c r="N31" s="2" t="n">
         <v>0</v>
@@ -5102,7 +5102,7 @@
         <v>1508.89</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>0</v>
+        <v>-56.22</v>
       </c>
       <c r="G41" s="2" t="n">
         <v>3000</v>
@@ -5983,7 +5983,7 @@
         <v>55422.36</v>
       </c>
       <c r="F74" s="5" t="n">
-        <v>40017.09</v>
+        <v>39960.87</v>
       </c>
       <c r="G74" s="5" t="n">
         <v>113950</v>

</xml_diff>

<commit_message>
Actualización automática 2026-05-18 17:30:19
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -483,7 +483,7 @@
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
     <col width="25" customWidth="1" min="11" max="11"/>
     <col width="24" customWidth="1" min="12" max="12"/>
     <col width="17" customWidth="1" min="13" max="13"/>
@@ -781,7 +781,7 @@
         <v>0</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>0</v>
+        <v>314.73</v>
       </c>
       <c r="E5" s="2" t="n">
         <v>0</v>
@@ -865,7 +865,7 @@
         <v>0</v>
       </c>
       <c r="L6" s="2" t="n">
-        <v>0</v>
+        <v>454.6</v>
       </c>
       <c r="M6" s="2" t="n">
         <v>2157.05</v>
@@ -1384,7 +1384,7 @@
         <v>0</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>453.71</v>
+        <v>651.09</v>
       </c>
       <c r="F15" s="2" t="n">
         <v>0</v>
@@ -1408,7 +1408,7 @@
         <v>0</v>
       </c>
       <c r="M15" s="2" t="n">
-        <v>1026.04</v>
+        <v>4076.83</v>
       </c>
       <c r="N15" s="2" t="n">
         <v>0</v>
@@ -1828,7 +1828,7 @@
         <v>0</v>
       </c>
       <c r="M22" s="2" t="n">
-        <v>14049.28</v>
+        <v>19773.06</v>
       </c>
       <c r="N22" s="2" t="n">
         <v>0</v>
@@ -2581,7 +2581,7 @@
         <v>0</v>
       </c>
       <c r="D35" s="2" t="n">
-        <v>0</v>
+        <v>3294.69</v>
       </c>
       <c r="E35" s="2" t="n">
         <v>0</v>
@@ -3559,7 +3559,7 @@
         <v>0</v>
       </c>
       <c r="J51" s="2" t="n">
-        <v>0</v>
+        <v>43.2</v>
       </c>
       <c r="K51" s="2" t="n">
         <v>0</v>
@@ -3894,47 +3894,47 @@
       </c>
       <c r="D57" s="4" t="inlineStr">
         <is>
+          <t>6 de 55</t>
+        </is>
+      </c>
+      <c r="E57" s="4" t="inlineStr">
+        <is>
+          <t>2 de 55</t>
+        </is>
+      </c>
+      <c r="F57" s="4" t="inlineStr">
+        <is>
+          <t>0 de 55</t>
+        </is>
+      </c>
+      <c r="G57" s="4" t="inlineStr">
+        <is>
+          <t>0 de 55</t>
+        </is>
+      </c>
+      <c r="H57" s="4" t="inlineStr">
+        <is>
+          <t>1 de 55</t>
+        </is>
+      </c>
+      <c r="I57" s="4" t="inlineStr">
+        <is>
           <t>4 de 55</t>
         </is>
       </c>
-      <c r="E57" s="4" t="inlineStr">
+      <c r="J57" s="4" t="inlineStr">
+        <is>
+          <t>1 de 55</t>
+        </is>
+      </c>
+      <c r="K57" s="4" t="inlineStr">
         <is>
           <t>2 de 55</t>
         </is>
       </c>
-      <c r="F57" s="4" t="inlineStr">
-        <is>
-          <t>0 de 55</t>
-        </is>
-      </c>
-      <c r="G57" s="4" t="inlineStr">
-        <is>
-          <t>0 de 55</t>
-        </is>
-      </c>
-      <c r="H57" s="4" t="inlineStr">
-        <is>
-          <t>1 de 55</t>
-        </is>
-      </c>
-      <c r="I57" s="4" t="inlineStr">
-        <is>
-          <t>4 de 55</t>
-        </is>
-      </c>
-      <c r="J57" s="4" t="inlineStr">
-        <is>
-          <t>0 de 55</t>
-        </is>
-      </c>
-      <c r="K57" s="4" t="inlineStr">
+      <c r="L57" s="4" t="inlineStr">
         <is>
           <t>2 de 55</t>
-        </is>
-      </c>
-      <c r="L57" s="4" t="inlineStr">
-        <is>
-          <t>1 de 55</t>
         </is>
       </c>
       <c r="M57" s="4" t="inlineStr">
@@ -4130,7 +4130,7 @@
         <v>7885.53</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>85.44</v>
+        <v>400.17</v>
       </c>
       <c r="G5" s="2" t="n">
         <v>10000</v>
@@ -4184,7 +4184,7 @@
         <v>0</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>2157.05</v>
+        <v>2611.65</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>1500</v>
@@ -4454,7 +4454,7 @@
         <v>3550.11</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>1479.75</v>
+        <v>4727.92</v>
       </c>
       <c r="G17" s="2" t="n">
         <v>6000</v>
@@ -4724,7 +4724,7 @@
         <v>1601.85</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>14049.28</v>
+        <v>19773.06</v>
       </c>
       <c r="G27" s="2" t="n">
         <v>0</v>
@@ -5237,7 +5237,7 @@
         <v>1535.44</v>
       </c>
       <c r="F46" s="2" t="n">
-        <v>9837</v>
+        <v>13131.69</v>
       </c>
       <c r="G46" s="2" t="n">
         <v>10000</v>
@@ -5777,7 +5777,7 @@
         <v>0</v>
       </c>
       <c r="F66" s="2" t="n">
-        <v>0</v>
+        <v>43.2</v>
       </c>
       <c r="G66" s="2" t="n">
         <v>0</v>
@@ -5983,7 +5983,7 @@
         <v>55422.36</v>
       </c>
       <c r="F74" s="5" t="n">
-        <v>39960.87</v>
+        <v>53040.04</v>
       </c>
       <c r="G74" s="5" t="n">
         <v>113950</v>

</xml_diff>

<commit_message>
Actualización automática 2026-06-02 08:30:20
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -748,7 +748,7 @@
         <v>0</v>
       </c>
       <c r="M4" s="2" t="n">
-        <v>0</v>
+        <v>1308.7</v>
       </c>
       <c r="N4" s="2" t="n">
         <v>0</v>
@@ -2641,7 +2641,7 @@
         <v>0</v>
       </c>
       <c r="D36" s="2" t="n">
-        <v>0</v>
+        <v>1652.32</v>
       </c>
       <c r="E36" s="2" t="n">
         <v>0</v>
@@ -2656,7 +2656,7 @@
         <v>0</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>0</v>
+        <v>251.27</v>
       </c>
       <c r="J36" s="2" t="n">
         <v>0</v>
@@ -2668,7 +2668,7 @@
         <v>0</v>
       </c>
       <c r="M36" s="2" t="n">
-        <v>0</v>
+        <v>810.3099999999999</v>
       </c>
       <c r="N36" s="2" t="n">
         <v>0</v>
@@ -3894,52 +3894,52 @@
       </c>
       <c r="D57" s="4" t="inlineStr">
         <is>
+          <t>1 de 55</t>
+        </is>
+      </c>
+      <c r="E57" s="4" t="inlineStr">
+        <is>
           <t>0 de 55</t>
         </is>
       </c>
-      <c r="E57" s="4" t="inlineStr">
+      <c r="F57" s="4" t="inlineStr">
         <is>
           <t>0 de 55</t>
         </is>
       </c>
-      <c r="F57" s="4" t="inlineStr">
+      <c r="G57" s="4" t="inlineStr">
         <is>
           <t>0 de 55</t>
         </is>
       </c>
-      <c r="G57" s="4" t="inlineStr">
+      <c r="H57" s="4" t="inlineStr">
         <is>
           <t>0 de 55</t>
         </is>
       </c>
-      <c r="H57" s="4" t="inlineStr">
+      <c r="I57" s="4" t="inlineStr">
+        <is>
+          <t>1 de 55</t>
+        </is>
+      </c>
+      <c r="J57" s="4" t="inlineStr">
         <is>
           <t>0 de 55</t>
         </is>
       </c>
-      <c r="I57" s="4" t="inlineStr">
+      <c r="K57" s="4" t="inlineStr">
         <is>
           <t>0 de 55</t>
         </is>
       </c>
-      <c r="J57" s="4" t="inlineStr">
+      <c r="L57" s="4" t="inlineStr">
         <is>
           <t>0 de 55</t>
         </is>
       </c>
-      <c r="K57" s="4" t="inlineStr">
-        <is>
-          <t>0 de 55</t>
-        </is>
-      </c>
-      <c r="L57" s="4" t="inlineStr">
-        <is>
-          <t>0 de 55</t>
-        </is>
-      </c>
       <c r="M57" s="4" t="inlineStr">
         <is>
-          <t>0 de 55</t>
+          <t>2 de 55</t>
         </is>
       </c>
       <c r="N57" s="4" t="inlineStr">
@@ -3987,7 +3987,7 @@
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -4103,7 +4103,7 @@
         <v>299.83</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>0</v>
+        <v>1308.7</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>15000</v>
@@ -5264,7 +5264,7 @@
         <v>909.79</v>
       </c>
       <c r="F47" s="2" t="n">
-        <v>0</v>
+        <v>2713.9</v>
       </c>
       <c r="G47" s="2" t="n">
         <v>8000</v>
@@ -5983,7 +5983,7 @@
         <v>96052.77</v>
       </c>
       <c r="F74" s="5" t="n">
-        <v>0</v>
+        <v>4022.6</v>
       </c>
       <c r="G74" s="5" t="n">
         <v>113950</v>

</xml_diff>

<commit_message>
Actualización automática 2026-06-02 12:30:19
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -3748,7 +3748,7 @@
         <v>0</v>
       </c>
       <c r="M54" s="2" t="n">
-        <v>0</v>
+        <v>39.46</v>
       </c>
       <c r="N54" s="2" t="n">
         <v>0</v>
@@ -3939,7 +3939,7 @@
       </c>
       <c r="M57" s="4" t="inlineStr">
         <is>
-          <t>2 de 55</t>
+          <t>3 de 55</t>
         </is>
       </c>
       <c r="N57" s="4" t="inlineStr">
@@ -5912,7 +5912,7 @@
         <v>2084.9</v>
       </c>
       <c r="F71" s="2" t="n">
-        <v>0</v>
+        <v>39.46</v>
       </c>
       <c r="G71" s="2" t="n">
         <v>1000</v>
@@ -5983,7 +5983,7 @@
         <v>96052.77</v>
       </c>
       <c r="F74" s="5" t="n">
-        <v>4022.6</v>
+        <v>4062.06</v>
       </c>
       <c r="G74" s="5" t="n">
         <v>113950</v>

</xml_diff>

<commit_message>
Actualización automática 2026-06-04 11:29:04
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -3979,7 +3979,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G74"/>
+  <dimension ref="A1:G76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5915,7 +5915,7 @@
         <v>39.46</v>
       </c>
       <c r="G71" s="2" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
     </row>
     <row r="72">
@@ -5926,23 +5926,23 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>WONG SANCHEZ PAULA SOFIA</t>
+          <t>WONG SANCHEZ CLAUDIA PAULINA</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
-        <v>0</v>
+        <v>1296.86</v>
       </c>
       <c r="D72" s="2" t="n">
-        <v>0</v>
+        <v>137.71</v>
       </c>
       <c r="E72" s="2" t="n">
-        <v>0</v>
+        <v>2084.9</v>
       </c>
       <c r="F72" s="2" t="n">
-        <v>0</v>
+        <v>39.46</v>
       </c>
       <c r="G72" s="2" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="73">
@@ -5953,40 +5953,94 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
+          <t>WONG SANCHEZ PAULA SOFIA</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D73" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E73" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F73" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G73" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>GUERRERO FAREZ FABIAN MAURICIO</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
           <t>ZUÑIGA CORONEL MARCIA LUZMILA</t>
         </is>
       </c>
-      <c r="C73" s="2" t="n">
+      <c r="C74" s="2" t="n">
         <v>295.2</v>
       </c>
-      <c r="D73" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E73" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F73" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G73" s="2" t="n">
+      <c r="D74" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E74" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F74" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G74" s="2" t="n">
         <v>1000</v>
       </c>
     </row>
-    <row r="74">
-      <c r="C74" s="5" t="n">
-        <v>77198.38</v>
-      </c>
-      <c r="D74" s="5" t="n">
-        <v>55422.36</v>
-      </c>
-      <c r="E74" s="5" t="n">
-        <v>96052.77</v>
-      </c>
-      <c r="F74" s="5" t="n">
-        <v>4455.47</v>
-      </c>
-      <c r="G74" s="5" t="n">
-        <v>113950</v>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>GUERRERO FAREZ FABIAN MAURICIO</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>ZUÑIGA CORONEL MARCIA LUZMILA</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="n">
+        <v>295.2</v>
+      </c>
+      <c r="D75" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E75" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F75" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G75" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="C76" s="5" t="n">
+        <v>78790.44</v>
+      </c>
+      <c r="D76" s="5" t="n">
+        <v>55560.07</v>
+      </c>
+      <c r="E76" s="5" t="n">
+        <v>98137.67</v>
+      </c>
+      <c r="F76" s="5" t="n">
+        <v>4494.93</v>
+      </c>
+      <c r="G76" s="5" t="n">
+        <v>114450</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-06-04 16:30:23
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -3358,7 +3358,7 @@
         </is>
       </c>
       <c r="C48" s="2" t="n">
-        <v>0</v>
+        <v>118.96</v>
       </c>
       <c r="D48" s="2" t="n">
         <v>0</v>
@@ -3748,7 +3748,7 @@
         <v>0</v>
       </c>
       <c r="M54" s="2" t="n">
-        <v>39.46</v>
+        <v>78.92</v>
       </c>
       <c r="N54" s="2" t="n">
         <v>0</v>
@@ -3889,7 +3889,7 @@
     <row r="57">
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>0 de 55</t>
+          <t>1 de 55</t>
         </is>
       </c>
       <c r="D57" s="4" t="inlineStr">
@@ -5669,7 +5669,7 @@
         <v>0</v>
       </c>
       <c r="F62" s="2" t="n">
-        <v>0</v>
+        <v>118.96</v>
       </c>
       <c r="G62" s="2" t="n">
         <v>1500</v>
@@ -5912,7 +5912,7 @@
         <v>2084.9</v>
       </c>
       <c r="F71" s="2" t="n">
-        <v>39.46</v>
+        <v>78.92</v>
       </c>
       <c r="G71" s="2" t="n">
         <v>500</v>
@@ -5939,7 +5939,7 @@
         <v>2084.9</v>
       </c>
       <c r="F72" s="2" t="n">
-        <v>39.46</v>
+        <v>78.92</v>
       </c>
       <c r="G72" s="2" t="n">
         <v>1000</v>
@@ -6037,7 +6037,7 @@
         <v>98137.67</v>
       </c>
       <c r="F76" s="5" t="n">
-        <v>4494.93</v>
+        <v>4692.81</v>
       </c>
       <c r="G76" s="5" t="n">
         <v>114450</v>

</xml_diff>

<commit_message>
Actualización automática 2026-06-08 11:30:21
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -736,7 +736,7 @@
         <v>0</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>0</v>
+        <v>84.91</v>
       </c>
       <c r="J4" s="2" t="n">
         <v>0</v>
@@ -3919,7 +3919,7 @@
       </c>
       <c r="I57" s="4" t="inlineStr">
         <is>
-          <t>1 de 55</t>
+          <t>2 de 55</t>
         </is>
       </c>
       <c r="J57" s="4" t="inlineStr">
@@ -4103,7 +4103,7 @@
         <v>299.83</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>1308.7</v>
+        <v>1393.61</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>15000</v>
@@ -6037,7 +6037,7 @@
         <v>98137.67</v>
       </c>
       <c r="F76" s="5" t="n">
-        <v>4692.81</v>
+        <v>4777.72</v>
       </c>
       <c r="G76" s="5" t="n">
         <v>114450</v>

</xml_diff>

<commit_message>
Actualización automática 2026-06-09 17:30:21
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -781,7 +781,7 @@
         <v>0</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>0</v>
+        <v>496.63</v>
       </c>
       <c r="E5" s="2" t="n">
         <v>0</v>
@@ -805,7 +805,7 @@
         <v>0</v>
       </c>
       <c r="L5" s="2" t="n">
-        <v>0</v>
+        <v>466.39</v>
       </c>
       <c r="M5" s="2" t="n">
         <v>0</v>
@@ -2161,7 +2161,7 @@
         <v>0</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>0</v>
+        <v>1264.46</v>
       </c>
       <c r="E28" s="2" t="n">
         <v>0</v>
@@ -2377,7 +2377,7 @@
         <v>0</v>
       </c>
       <c r="P31" s="2" t="n">
-        <v>0</v>
+        <v>1168.59</v>
       </c>
       <c r="Q31" s="2" t="n">
         <v>0</v>
@@ -2731,7 +2731,7 @@
         <v>0</v>
       </c>
       <c r="N37" s="2" t="n">
-        <v>0</v>
+        <v>1714.5</v>
       </c>
       <c r="O37" s="2" t="n">
         <v>0</v>
@@ -3748,7 +3748,7 @@
         <v>0</v>
       </c>
       <c r="M54" s="2" t="n">
-        <v>78.92</v>
+        <v>812.35</v>
       </c>
       <c r="N54" s="2" t="n">
         <v>0</v>
@@ -3894,67 +3894,67 @@
       </c>
       <c r="D57" s="4" t="inlineStr">
         <is>
+          <t>3 de 55</t>
+        </is>
+      </c>
+      <c r="E57" s="4" t="inlineStr">
+        <is>
+          <t>0 de 55</t>
+        </is>
+      </c>
+      <c r="F57" s="4" t="inlineStr">
+        <is>
+          <t>0 de 55</t>
+        </is>
+      </c>
+      <c r="G57" s="4" t="inlineStr">
+        <is>
+          <t>0 de 55</t>
+        </is>
+      </c>
+      <c r="H57" s="4" t="inlineStr">
+        <is>
+          <t>0 de 55</t>
+        </is>
+      </c>
+      <c r="I57" s="4" t="inlineStr">
+        <is>
+          <t>2 de 55</t>
+        </is>
+      </c>
+      <c r="J57" s="4" t="inlineStr">
+        <is>
+          <t>0 de 55</t>
+        </is>
+      </c>
+      <c r="K57" s="4" t="inlineStr">
+        <is>
+          <t>0 de 55</t>
+        </is>
+      </c>
+      <c r="L57" s="4" t="inlineStr">
+        <is>
           <t>1 de 55</t>
         </is>
       </c>
-      <c r="E57" s="4" t="inlineStr">
+      <c r="M57" s="4" t="inlineStr">
+        <is>
+          <t>3 de 55</t>
+        </is>
+      </c>
+      <c r="N57" s="4" t="inlineStr">
+        <is>
+          <t>1 de 55</t>
+        </is>
+      </c>
+      <c r="O57" s="4" t="inlineStr">
         <is>
           <t>0 de 55</t>
         </is>
       </c>
-      <c r="F57" s="4" t="inlineStr">
-        <is>
-          <t>0 de 55</t>
-        </is>
-      </c>
-      <c r="G57" s="4" t="inlineStr">
-        <is>
-          <t>0 de 55</t>
-        </is>
-      </c>
-      <c r="H57" s="4" t="inlineStr">
-        <is>
-          <t>0 de 55</t>
-        </is>
-      </c>
-      <c r="I57" s="4" t="inlineStr">
-        <is>
-          <t>2 de 55</t>
-        </is>
-      </c>
-      <c r="J57" s="4" t="inlineStr">
-        <is>
-          <t>0 de 55</t>
-        </is>
-      </c>
-      <c r="K57" s="4" t="inlineStr">
-        <is>
-          <t>0 de 55</t>
-        </is>
-      </c>
-      <c r="L57" s="4" t="inlineStr">
-        <is>
-          <t>0 de 55</t>
-        </is>
-      </c>
-      <c r="M57" s="4" t="inlineStr">
-        <is>
-          <t>3 de 55</t>
-        </is>
-      </c>
-      <c r="N57" s="4" t="inlineStr">
-        <is>
-          <t>0 de 55</t>
-        </is>
-      </c>
-      <c r="O57" s="4" t="inlineStr">
-        <is>
-          <t>0 de 55</t>
-        </is>
-      </c>
       <c r="P57" s="4" t="inlineStr">
         <is>
-          <t>0 de 55</t>
+          <t>1 de 55</t>
         </is>
       </c>
       <c r="Q57" s="4" t="inlineStr">
@@ -4130,7 +4130,7 @@
         <v>12753.16</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>0</v>
+        <v>963.02</v>
       </c>
       <c r="G5" s="2" t="n">
         <v>10000</v>
@@ -5021,7 +5021,7 @@
         <v>1827.98</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>0</v>
+        <v>1264.46</v>
       </c>
       <c r="G38" s="2" t="n">
         <v>6000</v>
@@ -5102,7 +5102,7 @@
         <v>-18.09</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>0</v>
+        <v>1168.59</v>
       </c>
       <c r="G41" s="2" t="n">
         <v>3000</v>
@@ -5210,7 +5210,7 @@
         <v>186.76</v>
       </c>
       <c r="F45" s="2" t="n">
-        <v>0</v>
+        <v>97.11</v>
       </c>
       <c r="G45" s="2" t="n">
         <v>0</v>
@@ -5318,7 +5318,7 @@
         <v>0</v>
       </c>
       <c r="F49" s="2" t="n">
-        <v>0</v>
+        <v>1714.5</v>
       </c>
       <c r="G49" s="2" t="n">
         <v>200</v>
@@ -5426,7 +5426,7 @@
         <v>0</v>
       </c>
       <c r="F53" s="2" t="n">
-        <v>0</v>
+        <v>669.0599999999999</v>
       </c>
       <c r="G53" s="2" t="n">
         <v>1000</v>
@@ -5912,7 +5912,7 @@
         <v>2084.9</v>
       </c>
       <c r="F71" s="2" t="n">
-        <v>78.92</v>
+        <v>812.35</v>
       </c>
       <c r="G71" s="2" t="n">
         <v>500</v>
@@ -5939,7 +5939,7 @@
         <v>2084.9</v>
       </c>
       <c r="F72" s="2" t="n">
-        <v>78.92</v>
+        <v>812.35</v>
       </c>
       <c r="G72" s="2" t="n">
         <v>1000</v>
@@ -6037,7 +6037,7 @@
         <v>98137.67</v>
       </c>
       <c r="F76" s="5" t="n">
-        <v>4777.72</v>
+        <v>12121.32</v>
       </c>
       <c r="G76" s="5" t="n">
         <v>114450</v>

</xml_diff>

<commit_message>
Actualización automática 2026-06-10 08:30:20
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R57"/>
+  <dimension ref="A1:R56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3654,7 +3654,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>WONG HEREDIA VLADIMIR GERARDO</t>
+          <t>WONG SANCHEZ CLAUDIA PAULINA</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
@@ -3688,7 +3688,7 @@
         <v>0</v>
       </c>
       <c r="M53" s="2" t="n">
-        <v>0</v>
+        <v>812.35</v>
       </c>
       <c r="N53" s="2" t="n">
         <v>0</v>
@@ -3714,7 +3714,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>WONG SANCHEZ CLAUDIA PAULINA</t>
+          <t>WONG SANCHEZ PAULA SOFIA</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
@@ -3748,7 +3748,7 @@
         <v>0</v>
       </c>
       <c r="M54" s="2" t="n">
-        <v>812.35</v>
+        <v>0</v>
       </c>
       <c r="N54" s="2" t="n">
         <v>0</v>
@@ -3774,7 +3774,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>WONG SANCHEZ PAULA SOFIA</t>
+          <t>ZUÑIGA CORONEL MARCIA LUZMILA</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
@@ -3827,144 +3827,84 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>GUERRERO FAREZ FABIAN MAURICIO</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>ZUÑIGA CORONEL MARCIA LUZMILA</t>
-        </is>
-      </c>
-      <c r="C56" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D56" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E56" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F56" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G56" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H56" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I56" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J56" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K56" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L56" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M56" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N56" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O56" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P56" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q56" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R56" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="C57" s="4" t="inlineStr">
-        <is>
-          <t>1 de 55</t>
-        </is>
-      </c>
-      <c r="D57" s="4" t="inlineStr">
-        <is>
-          <t>3 de 55</t>
-        </is>
-      </c>
-      <c r="E57" s="4" t="inlineStr">
-        <is>
-          <t>0 de 55</t>
-        </is>
-      </c>
-      <c r="F57" s="4" t="inlineStr">
-        <is>
-          <t>0 de 55</t>
-        </is>
-      </c>
-      <c r="G57" s="4" t="inlineStr">
-        <is>
-          <t>0 de 55</t>
-        </is>
-      </c>
-      <c r="H57" s="4" t="inlineStr">
-        <is>
-          <t>0 de 55</t>
-        </is>
-      </c>
-      <c r="I57" s="4" t="inlineStr">
-        <is>
-          <t>2 de 55</t>
-        </is>
-      </c>
-      <c r="J57" s="4" t="inlineStr">
-        <is>
-          <t>0 de 55</t>
-        </is>
-      </c>
-      <c r="K57" s="4" t="inlineStr">
-        <is>
-          <t>0 de 55</t>
-        </is>
-      </c>
-      <c r="L57" s="4" t="inlineStr">
-        <is>
-          <t>1 de 55</t>
-        </is>
-      </c>
-      <c r="M57" s="4" t="inlineStr">
-        <is>
-          <t>3 de 55</t>
-        </is>
-      </c>
-      <c r="N57" s="4" t="inlineStr">
-        <is>
-          <t>1 de 55</t>
-        </is>
-      </c>
-      <c r="O57" s="4" t="inlineStr">
-        <is>
-          <t>0 de 55</t>
-        </is>
-      </c>
-      <c r="P57" s="4" t="inlineStr">
-        <is>
-          <t>1 de 55</t>
-        </is>
-      </c>
-      <c r="Q57" s="4" t="inlineStr">
-        <is>
-          <t>0 de 55</t>
-        </is>
-      </c>
-      <c r="R57" s="4" t="inlineStr">
-        <is>
-          <t>0 de 55</t>
+      <c r="C56" s="4" t="inlineStr">
+        <is>
+          <t>1 de 54</t>
+        </is>
+      </c>
+      <c r="D56" s="4" t="inlineStr">
+        <is>
+          <t>3 de 54</t>
+        </is>
+      </c>
+      <c r="E56" s="4" t="inlineStr">
+        <is>
+          <t>0 de 54</t>
+        </is>
+      </c>
+      <c r="F56" s="4" t="inlineStr">
+        <is>
+          <t>0 de 54</t>
+        </is>
+      </c>
+      <c r="G56" s="4" t="inlineStr">
+        <is>
+          <t>0 de 54</t>
+        </is>
+      </c>
+      <c r="H56" s="4" t="inlineStr">
+        <is>
+          <t>0 de 54</t>
+        </is>
+      </c>
+      <c r="I56" s="4" t="inlineStr">
+        <is>
+          <t>2 de 54</t>
+        </is>
+      </c>
+      <c r="J56" s="4" t="inlineStr">
+        <is>
+          <t>0 de 54</t>
+        </is>
+      </c>
+      <c r="K56" s="4" t="inlineStr">
+        <is>
+          <t>0 de 54</t>
+        </is>
+      </c>
+      <c r="L56" s="4" t="inlineStr">
+        <is>
+          <t>1 de 54</t>
+        </is>
+      </c>
+      <c r="M56" s="4" t="inlineStr">
+        <is>
+          <t>3 de 54</t>
+        </is>
+      </c>
+      <c r="N56" s="4" t="inlineStr">
+        <is>
+          <t>1 de 54</t>
+        </is>
+      </c>
+      <c r="O56" s="4" t="inlineStr">
+        <is>
+          <t>0 de 54</t>
+        </is>
+      </c>
+      <c r="P56" s="4" t="inlineStr">
+        <is>
+          <t>1 de 54</t>
+        </is>
+      </c>
+      <c r="Q56" s="4" t="inlineStr">
+        <is>
+          <t>0 de 54</t>
+        </is>
+      </c>
+      <c r="R56" s="4" t="inlineStr">
+        <is>
+          <t>0 de 54</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática 2026-06-11 15:30:22
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -1528,7 +1528,7 @@
         <v>0</v>
       </c>
       <c r="M17" s="2" t="n">
-        <v>0</v>
+        <v>39.39</v>
       </c>
       <c r="N17" s="2" t="n">
         <v>0</v>
@@ -3879,7 +3879,7 @@
       </c>
       <c r="M56" s="4" t="inlineStr">
         <is>
-          <t>3 de 54</t>
+          <t>4 de 54</t>
         </is>
       </c>
       <c r="N56" s="4" t="inlineStr">
@@ -4529,7 +4529,7 @@
         <v>915.88</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>0</v>
+        <v>39.39</v>
       </c>
       <c r="G22" s="2" t="n">
         <v>3000</v>
@@ -5977,7 +5977,7 @@
         <v>98137.67</v>
       </c>
       <c r="F76" s="5" t="n">
-        <v>12121.32</v>
+        <v>12160.71</v>
       </c>
       <c r="G76" s="5" t="n">
         <v>114450</v>
@@ -6268,13 +6268,13 @@
         <v>72100</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>2931.36</v>
+        <v>2970.75</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>69168.64</v>
+        <v>69129.25</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>0.04065686546463246</v>
+        <v>0.04120319001386963</v>
       </c>
     </row>
     <row r="12">
@@ -6311,13 +6311,13 @@
         <v>83903.5</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>11308.97</v>
+        <v>11348.36</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>72594.53</v>
+        <v>72555.14</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.1347854380329784</v>
+        <v>0.1352549059336023</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-06-12 14:30:22
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -1288,7 +1288,7 @@
         <v>0</v>
       </c>
       <c r="M13" s="2" t="n">
-        <v>0</v>
+        <v>547.9</v>
       </c>
       <c r="N13" s="2" t="n">
         <v>0</v>
@@ -1528,7 +1528,7 @@
         <v>0</v>
       </c>
       <c r="M17" s="2" t="n">
-        <v>39.39</v>
+        <v>62.13</v>
       </c>
       <c r="N17" s="2" t="n">
         <v>0</v>
@@ -3879,7 +3879,7 @@
       </c>
       <c r="M56" s="4" t="inlineStr">
         <is>
-          <t>6 de 54</t>
+          <t>7 de 54</t>
         </is>
       </c>
       <c r="N56" s="4" t="inlineStr">
@@ -4340,7 +4340,7 @@
         <v>0</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>0</v>
+        <v>547.9</v>
       </c>
       <c r="G15" s="2" t="n">
         <v>6000</v>
@@ -4529,7 +4529,7 @@
         <v>915.88</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>39.39</v>
+        <v>62.13</v>
       </c>
       <c r="G22" s="2" t="n">
         <v>3000</v>
@@ -5977,7 +5977,7 @@
         <v>98137.67</v>
       </c>
       <c r="F76" s="5" t="n">
-        <v>12072.96</v>
+        <v>12643.6</v>
       </c>
       <c r="G76" s="5" t="n">
         <v>114450</v>
@@ -6268,13 +6268,13 @@
         <v>72100</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>2866.26</v>
+        <v>3436.9</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>69233.74000000001</v>
+        <v>68663.10000000001</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>0.03975395284327324</v>
+        <v>0.04766851595006935</v>
       </c>
     </row>
     <row r="12">
@@ -6311,13 +6311,13 @@
         <v>83903.5</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>11243.87</v>
+        <v>11814.51</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>72659.63</v>
+        <v>72088.99000000001</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.1340095466816045</v>
+        <v>0.1408106932368733</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-06-15 16:30:21
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -1528,7 +1528,7 @@
         <v>0</v>
       </c>
       <c r="M17" s="2" t="n">
-        <v>62.13</v>
+        <v>40.1</v>
       </c>
       <c r="N17" s="2" t="n">
         <v>0</v>
@@ -4529,7 +4529,7 @@
         <v>915.88</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>62.13</v>
+        <v>40.1</v>
       </c>
       <c r="G22" s="2" t="n">
         <v>3000</v>
@@ -5977,7 +5977,7 @@
         <v>98137.67</v>
       </c>
       <c r="F76" s="5" t="n">
-        <v>12643.6</v>
+        <v>12621.57</v>
       </c>
       <c r="G76" s="5" t="n">
         <v>114450</v>
@@ -6268,13 +6268,13 @@
         <v>72100</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>3436.9</v>
+        <v>3414.87</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>68663.10000000001</v>
+        <v>68685.13</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>0.04766851595006935</v>
+        <v>0.04736296809986131</v>
       </c>
     </row>
     <row r="12">
@@ -6311,13 +6311,13 @@
         <v>83903.5</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>11814.51</v>
+        <v>11792.48</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>72088.99000000001</v>
+        <v>72111.02</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.1408106932368733</v>
+        <v>0.1405481296966158</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-06-15 17:12:22
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -928,7 +928,7 @@
         <v>0</v>
       </c>
       <c r="M7" s="2" t="n">
-        <v>16.74</v>
+        <v>982.99</v>
       </c>
       <c r="N7" s="2" t="n">
         <v>0</v>
@@ -4151,7 +4151,7 @@
         <v>549.08</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>16.74</v>
+        <v>982.99</v>
       </c>
       <c r="G8" s="2" t="n">
         <v>1500</v>
@@ -5977,7 +5977,7 @@
         <v>98137.67</v>
       </c>
       <c r="F76" s="5" t="n">
-        <v>12621.57</v>
+        <v>13587.82</v>
       </c>
       <c r="G76" s="5" t="n">
         <v>114450</v>
@@ -6268,13 +6268,13 @@
         <v>72100</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>3414.87</v>
+        <v>4381.12</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>68685.13</v>
+        <v>67718.88</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>0.04736296809986131</v>
+        <v>0.06076449375866851</v>
       </c>
     </row>
     <row r="12">
@@ -6311,13 +6311,13 @@
         <v>83903.5</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>11792.48</v>
+        <v>12758.73</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>72111.02</v>
+        <v>71144.77</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.1405481296966158</v>
+        <v>0.1520643358143582</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-06-17 15:30:20
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -2341,7 +2341,7 @@
         <v>0</v>
       </c>
       <c r="D31" s="2" t="n">
-        <v>0</v>
+        <v>487.47</v>
       </c>
       <c r="E31" s="2" t="n">
         <v>0</v>
@@ -2377,7 +2377,7 @@
         <v>0</v>
       </c>
       <c r="P31" s="2" t="n">
-        <v>1168.59</v>
+        <v>1238.71</v>
       </c>
       <c r="Q31" s="2" t="n">
         <v>0</v>
@@ -2542,7 +2542,7 @@
         <v>0</v>
       </c>
       <c r="K34" s="2" t="n">
-        <v>0</v>
+        <v>18.27</v>
       </c>
       <c r="L34" s="2" t="n">
         <v>0</v>
@@ -3834,7 +3834,7 @@
       </c>
       <c r="D56" s="4" t="inlineStr">
         <is>
-          <t>3 de 54</t>
+          <t>4 de 54</t>
         </is>
       </c>
       <c r="E56" s="4" t="inlineStr">
@@ -3869,7 +3869,7 @@
       </c>
       <c r="K56" s="4" t="inlineStr">
         <is>
-          <t>1 de 54</t>
+          <t>2 de 54</t>
         </is>
       </c>
       <c r="L56" s="4" t="inlineStr">
@@ -5042,7 +5042,7 @@
         <v>-18.09</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>1168.59</v>
+        <v>1726.18</v>
       </c>
       <c r="G41" s="2" t="n">
         <v>3000</v>
@@ -5150,7 +5150,7 @@
         <v>186.76</v>
       </c>
       <c r="F45" s="2" t="n">
-        <v>97.11</v>
+        <v>115.38</v>
       </c>
       <c r="G45" s="2" t="n">
         <v>0</v>
@@ -5977,7 +5977,7 @@
         <v>98137.67</v>
       </c>
       <c r="F76" s="5" t="n">
-        <v>13655.32</v>
+        <v>14231.18</v>
       </c>
       <c r="G76" s="5" t="n">
         <v>114450</v>
@@ -6001,7 +6001,7 @@
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
     <col width="25" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -6076,13 +6076,13 @@
         <v>7350</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>3806.82</v>
+        <v>4294.29</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>3543.18</v>
+        <v>3055.71</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>0.5179346938775511</v>
+        <v>0.5842571428571428</v>
       </c>
     </row>
     <row r="4">
@@ -6172,13 +6172,13 @@
         <v>250</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>1168.59</v>
+        <v>1238.71</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>-918.5899999999999</v>
+        <v>-988.71</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>4.67436</v>
+        <v>4.95484</v>
       </c>
     </row>
     <row r="8">
@@ -6220,13 +6220,13 @@
         <v>800</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>50.76</v>
+        <v>69.03</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>749.24</v>
+        <v>730.97</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>0.06344999999999999</v>
+        <v>0.0862875</v>
       </c>
     </row>
     <row r="10">
@@ -6311,13 +6311,13 @@
         <v>83903.5</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>12826.23</v>
+        <v>13402.09</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>71077.27</v>
+        <v>70501.41</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.1528688314551836</v>
+        <v>0.1597321923400097</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-06-17 17:30:20
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -471,11 +471,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R56"/>
+  <dimension ref="A1:R57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
     <col width="25" customWidth="1" min="3" max="3"/>
     <col width="24" customWidth="1" min="4" max="4"/>
     <col width="26" customWidth="1" min="5" max="5"/>
@@ -2608,7 +2608,7 @@
         <v>0</v>
       </c>
       <c r="M35" s="2" t="n">
-        <v>0</v>
+        <v>113.72</v>
       </c>
       <c r="N35" s="2" t="n">
         <v>0</v>
@@ -3534,7 +3534,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>SOLANO DE LA SALA PAZ GONZALO PATRICIO</t>
+          <t>SANDIEGO NEUMATICOS &amp; SERVICIOS CIA LTDA</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
@@ -3568,7 +3568,7 @@
         <v>0</v>
       </c>
       <c r="M51" s="2" t="n">
-        <v>0</v>
+        <v>762.85</v>
       </c>
       <c r="N51" s="2" t="n">
         <v>0</v>
@@ -3594,7 +3594,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>TORO BLACIO MARIA DEL CISNE</t>
+          <t>SOLANO DE LA SALA PAZ GONZALO PATRICIO</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
@@ -3654,7 +3654,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>WONG SANCHEZ CLAUDIA PAULINA</t>
+          <t>TORO BLACIO MARIA DEL CISNE</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
@@ -3688,7 +3688,7 @@
         <v>0</v>
       </c>
       <c r="M53" s="2" t="n">
-        <v>829.09</v>
+        <v>0</v>
       </c>
       <c r="N53" s="2" t="n">
         <v>0</v>
@@ -3714,7 +3714,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>WONG SANCHEZ PAULA SOFIA</t>
+          <t>WONG SANCHEZ CLAUDIA PAULINA</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
@@ -3748,7 +3748,7 @@
         <v>0</v>
       </c>
       <c r="M54" s="2" t="n">
-        <v>0</v>
+        <v>829.09</v>
       </c>
       <c r="N54" s="2" t="n">
         <v>0</v>
@@ -3774,137 +3774,197 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
+          <t>WONG SANCHEZ PAULA SOFIA</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R55" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>GUERRERO FAREZ FABIAN MAURICIO</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
           <t>ZUÑIGA CORONEL MARCIA LUZMILA</t>
         </is>
       </c>
-      <c r="C55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R55" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="C56" s="4" t="inlineStr">
-        <is>
-          <t>1 de 54</t>
-        </is>
-      </c>
-      <c r="D56" s="4" t="inlineStr">
-        <is>
-          <t>4 de 54</t>
-        </is>
-      </c>
-      <c r="E56" s="4" t="inlineStr">
-        <is>
-          <t>0 de 54</t>
-        </is>
-      </c>
-      <c r="F56" s="4" t="inlineStr">
-        <is>
-          <t>0 de 54</t>
-        </is>
-      </c>
-      <c r="G56" s="4" t="inlineStr">
-        <is>
-          <t>0 de 54</t>
-        </is>
-      </c>
-      <c r="H56" s="4" t="inlineStr">
-        <is>
-          <t>0 de 54</t>
-        </is>
-      </c>
-      <c r="I56" s="4" t="inlineStr">
-        <is>
-          <t>2 de 54</t>
-        </is>
-      </c>
-      <c r="J56" s="4" t="inlineStr">
-        <is>
-          <t>0 de 54</t>
-        </is>
-      </c>
-      <c r="K56" s="4" t="inlineStr">
-        <is>
-          <t>2 de 54</t>
-        </is>
-      </c>
-      <c r="L56" s="4" t="inlineStr">
-        <is>
-          <t>1 de 54</t>
-        </is>
-      </c>
-      <c r="M56" s="4" t="inlineStr">
-        <is>
-          <t>7 de 54</t>
-        </is>
-      </c>
-      <c r="N56" s="4" t="inlineStr">
-        <is>
-          <t>1 de 54</t>
-        </is>
-      </c>
-      <c r="O56" s="4" t="inlineStr">
-        <is>
-          <t>0 de 54</t>
-        </is>
-      </c>
-      <c r="P56" s="4" t="inlineStr">
-        <is>
-          <t>1 de 54</t>
-        </is>
-      </c>
-      <c r="Q56" s="4" t="inlineStr">
-        <is>
-          <t>0 de 54</t>
-        </is>
-      </c>
-      <c r="R56" s="4" t="inlineStr">
-        <is>
-          <t>0 de 54</t>
+      <c r="C56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R56" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="C57" s="4" t="inlineStr">
+        <is>
+          <t>1 de 55</t>
+        </is>
+      </c>
+      <c r="D57" s="4" t="inlineStr">
+        <is>
+          <t>4 de 55</t>
+        </is>
+      </c>
+      <c r="E57" s="4" t="inlineStr">
+        <is>
+          <t>0 de 55</t>
+        </is>
+      </c>
+      <c r="F57" s="4" t="inlineStr">
+        <is>
+          <t>0 de 55</t>
+        </is>
+      </c>
+      <c r="G57" s="4" t="inlineStr">
+        <is>
+          <t>0 de 55</t>
+        </is>
+      </c>
+      <c r="H57" s="4" t="inlineStr">
+        <is>
+          <t>0 de 55</t>
+        </is>
+      </c>
+      <c r="I57" s="4" t="inlineStr">
+        <is>
+          <t>2 de 55</t>
+        </is>
+      </c>
+      <c r="J57" s="4" t="inlineStr">
+        <is>
+          <t>0 de 55</t>
+        </is>
+      </c>
+      <c r="K57" s="4" t="inlineStr">
+        <is>
+          <t>2 de 55</t>
+        </is>
+      </c>
+      <c r="L57" s="4" t="inlineStr">
+        <is>
+          <t>1 de 55</t>
+        </is>
+      </c>
+      <c r="M57" s="4" t="inlineStr">
+        <is>
+          <t>9 de 55</t>
+        </is>
+      </c>
+      <c r="N57" s="4" t="inlineStr">
+        <is>
+          <t>1 de 55</t>
+        </is>
+      </c>
+      <c r="O57" s="4" t="inlineStr">
+        <is>
+          <t>0 de 55</t>
+        </is>
+      </c>
+      <c r="P57" s="4" t="inlineStr">
+        <is>
+          <t>1 de 55</t>
+        </is>
+      </c>
+      <c r="Q57" s="4" t="inlineStr">
+        <is>
+          <t>0 de 55</t>
+        </is>
+      </c>
+      <c r="R57" s="4" t="inlineStr">
+        <is>
+          <t>0 de 55</t>
         </is>
       </c>
     </row>
@@ -3919,7 +3979,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G76"/>
+  <dimension ref="A1:G77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5177,7 +5237,7 @@
         <v>14045.74</v>
       </c>
       <c r="F46" s="2" t="n">
-        <v>50.76</v>
+        <v>164.48</v>
       </c>
       <c r="G46" s="2" t="n">
         <v>10000</v>
@@ -5704,7 +5764,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>SOLANO DE LA SALA PAZ GONZALO PATRICIO</t>
+          <t>SANDIEGO NEUMATICOS &amp; SERVICIOS CIA LTDA</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
@@ -5714,10 +5774,10 @@
         <v>0</v>
       </c>
       <c r="E66" s="2" t="n">
-        <v>1136.67</v>
+        <v>0</v>
       </c>
       <c r="F66" s="2" t="n">
-        <v>0</v>
+        <v>762.85</v>
       </c>
       <c r="G66" s="2" t="n">
         <v>0</v>
@@ -5731,7 +5791,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>TOLEDO AREVALO DIEGO ANIBAL</t>
+          <t>SOLANO DE LA SALA PAZ GONZALO PATRICIO</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
@@ -5741,7 +5801,7 @@
         <v>0</v>
       </c>
       <c r="E67" s="2" t="n">
-        <v>0</v>
+        <v>1136.67</v>
       </c>
       <c r="F67" s="2" t="n">
         <v>0</v>
@@ -5758,7 +5818,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>TORO AGUILAR JOSE HONORIO</t>
+          <t>TOLEDO AREVALO DIEGO ANIBAL</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
@@ -5785,23 +5845,23 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>TORO BLACIO MARIA DEL CISNE</t>
+          <t>TORO AGUILAR JOSE HONORIO</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
-        <v>834.48</v>
+        <v>0</v>
       </c>
       <c r="D69" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E69" s="2" t="n">
-        <v>38.13</v>
+        <v>0</v>
       </c>
       <c r="F69" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G69" s="2" t="n">
-        <v>1650</v>
+        <v>0</v>
       </c>
     </row>
     <row r="70">
@@ -5812,23 +5872,23 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>WONG HEREDIA VLADIMIR GERARDO</t>
+          <t>TORO BLACIO MARIA DEL CISNE</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
-        <v>0</v>
+        <v>834.48</v>
       </c>
       <c r="D70" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E70" s="2" t="n">
-        <v>0</v>
+        <v>38.13</v>
       </c>
       <c r="F70" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G70" s="2" t="n">
-        <v>0</v>
+        <v>1650</v>
       </c>
     </row>
     <row r="71">
@@ -5839,23 +5899,23 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>WONG SANCHEZ CLAUDIA PAULINA</t>
+          <t>WONG HEREDIA VLADIMIR GERARDO</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
-        <v>1296.86</v>
+        <v>0</v>
       </c>
       <c r="D71" s="2" t="n">
-        <v>137.71</v>
+        <v>0</v>
       </c>
       <c r="E71" s="2" t="n">
-        <v>2084.9</v>
+        <v>0</v>
       </c>
       <c r="F71" s="2" t="n">
-        <v>829.09</v>
+        <v>0</v>
       </c>
       <c r="G71" s="2" t="n">
-        <v>500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="72">
@@ -5882,7 +5942,7 @@
         <v>829.09</v>
       </c>
       <c r="G72" s="2" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
     </row>
     <row r="73">
@@ -5893,23 +5953,23 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>WONG SANCHEZ PAULA SOFIA</t>
+          <t>WONG SANCHEZ CLAUDIA PAULINA</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
-        <v>0</v>
+        <v>1296.86</v>
       </c>
       <c r="D73" s="2" t="n">
-        <v>0</v>
+        <v>137.71</v>
       </c>
       <c r="E73" s="2" t="n">
-        <v>0</v>
+        <v>2084.9</v>
       </c>
       <c r="F73" s="2" t="n">
-        <v>0</v>
+        <v>829.09</v>
       </c>
       <c r="G73" s="2" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="74">
@@ -5920,11 +5980,11 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>ZUÑIGA CORONEL MARCIA LUZMILA</t>
+          <t>WONG SANCHEZ PAULA SOFIA</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
-        <v>295.2</v>
+        <v>0</v>
       </c>
       <c r="D74" s="2" t="n">
         <v>0</v>
@@ -5936,7 +5996,7 @@
         <v>0</v>
       </c>
       <c r="G74" s="2" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="75">
@@ -5963,23 +6023,50 @@
         <v>0</v>
       </c>
       <c r="G75" s="2" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="76">
-      <c r="C76" s="5" t="n">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>GUERRERO FAREZ FABIAN MAURICIO</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>ZUÑIGA CORONEL MARCIA LUZMILA</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="n">
+        <v>295.2</v>
+      </c>
+      <c r="D76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G76" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="C77" s="5" t="n">
         <v>78790.44</v>
       </c>
-      <c r="D76" s="5" t="n">
+      <c r="D77" s="5" t="n">
         <v>55560.07</v>
       </c>
-      <c r="E76" s="5" t="n">
+      <c r="E77" s="5" t="n">
         <v>98137.67</v>
       </c>
-      <c r="F76" s="5" t="n">
-        <v>14231.18</v>
-      </c>
-      <c r="G76" s="5" t="n">
+      <c r="F77" s="5" t="n">
+        <v>15107.75</v>
+      </c>
+      <c r="G77" s="5" t="n">
         <v>114450</v>
       </c>
     </row>
@@ -6268,13 +6355,13 @@
         <v>72100</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>4397.86</v>
+        <v>5274.43</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>67702.14</v>
+        <v>66825.57000000001</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>0.06099667128987517</v>
+        <v>0.07315436893203883</v>
       </c>
     </row>
     <row r="12">
@@ -6311,13 +6398,13 @@
         <v>83903.5</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>13402.09</v>
+        <v>14278.66</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>70501.41</v>
+        <v>69624.84000000001</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.1597321923400097</v>
+        <v>0.1701795515085783</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-06-18 16:30:21
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -1408,7 +1408,7 @@
         <v>0</v>
       </c>
       <c r="M15" s="2" t="n">
-        <v>0</v>
+        <v>15.48</v>
       </c>
       <c r="N15" s="2" t="n">
         <v>0</v>
@@ -3939,7 +3939,7 @@
       </c>
       <c r="M57" s="4" t="inlineStr">
         <is>
-          <t>9 de 55</t>
+          <t>10 de 55</t>
         </is>
       </c>
       <c r="N57" s="4" t="inlineStr">
@@ -4454,7 +4454,7 @@
         <v>11354.85</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>0</v>
+        <v>15.48</v>
       </c>
       <c r="G17" s="2" t="n">
         <v>6000</v>
@@ -6064,7 +6064,7 @@
         <v>98137.67</v>
       </c>
       <c r="F77" s="5" t="n">
-        <v>15107.75</v>
+        <v>15123.23</v>
       </c>
       <c r="G77" s="5" t="n">
         <v>114450</v>
@@ -6355,13 +6355,13 @@
         <v>72100</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>5274.43</v>
+        <v>5289.91</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>66825.57000000001</v>
+        <v>66810.09</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>0.07315436893203883</v>
+        <v>0.07336907073509015</v>
       </c>
     </row>
     <row r="12">
@@ -6398,13 +6398,13 @@
         <v>83903.5</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>14278.66</v>
+        <v>14294.14</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>69624.84000000001</v>
+        <v>69609.36</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.1701795515085783</v>
+        <v>0.1703640491755409</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-06-23 09:30:19
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -2377,7 +2377,7 @@
         <v>0</v>
       </c>
       <c r="P31" s="2" t="n">
-        <v>1238.71</v>
+        <v>1227.02</v>
       </c>
       <c r="Q31" s="2" t="n">
         <v>0</v>
@@ -5102,7 +5102,7 @@
         <v>-18.09</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>1726.18</v>
+        <v>1714.49</v>
       </c>
       <c r="G41" s="2" t="n">
         <v>3000</v>
@@ -6064,7 +6064,7 @@
         <v>98137.67</v>
       </c>
       <c r="F77" s="5" t="n">
-        <v>15155.45</v>
+        <v>15143.76</v>
       </c>
       <c r="G77" s="5" t="n">
         <v>114450</v>
@@ -6259,13 +6259,13 @@
         <v>250</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>1238.71</v>
+        <v>1227.02</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>-988.71</v>
+        <v>-977.02</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>4.95484</v>
+        <v>4.90808</v>
       </c>
     </row>
     <row r="8">
@@ -6398,13 +6398,13 @@
         <v>83903.5</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>14326.36</v>
+        <v>14314.67</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>69577.14</v>
+        <v>69588.83</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.1707480617614283</v>
+        <v>0.1706087350348913</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-06-23 17:30:21
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -2161,7 +2161,7 @@
         <v>0</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>1264.46</v>
+        <v>1517.35</v>
       </c>
       <c r="E28" s="2" t="n">
         <v>0</v>
@@ -5021,7 +5021,7 @@
         <v>1827.98</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>1264.46</v>
+        <v>1517.35</v>
       </c>
       <c r="G38" s="2" t="n">
         <v>6000</v>
@@ -6064,7 +6064,7 @@
         <v>98137.67</v>
       </c>
       <c r="F77" s="5" t="n">
-        <v>15143.76</v>
+        <v>15396.65</v>
       </c>
       <c r="G77" s="5" t="n">
         <v>114450</v>
@@ -6163,13 +6163,13 @@
         <v>7350</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>4294.29</v>
+        <v>4547.18</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>3055.71</v>
+        <v>2802.82</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>0.5842571428571428</v>
+        <v>0.6186639455782313</v>
       </c>
     </row>
     <row r="4">
@@ -6398,13 +6398,13 @@
         <v>83903.5</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>14314.67</v>
+        <v>14567.56</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>69588.83</v>
+        <v>69335.94</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.1706087350348913</v>
+        <v>0.1736227928513114</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-06-26 08:30:19
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R57"/>
+  <dimension ref="A1:R56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2814,7 +2814,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>PALLARES RIVERA WASHINGTON RAMIRO</t>
+          <t>PEREZ ROSALES EDGAR RICARDO</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
@@ -2874,7 +2874,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>PEREZ ROSALES EDGAR RICARDO</t>
+          <t>PEÑALOZA LOPEZ RONALD STALIN</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
@@ -2934,7 +2934,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>PEÑALOZA LOPEZ RONALD STALIN</t>
+          <t>QUEZADA VEGA JAIME PATRICIO</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
@@ -2994,7 +2994,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>QUEZADA VEGA JAIME PATRICIO</t>
+          <t>QUINCHE ALCIVAR ARGENTINA DEL ROCIO</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
@@ -3054,7 +3054,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>QUINCHE ALCIVAR ARGENTINA DEL ROCIO</t>
+          <t>RAMIREZ APOLO JOBANI DE JESUS</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
@@ -3114,7 +3114,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>RAMIREZ APOLO JOBANI DE JESUS</t>
+          <t>REYES MOSCOSO NARCISA DE JESUS</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
@@ -3174,7 +3174,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>REYES MOSCOSO NARCISA DE JESUS</t>
+          <t>ROJAS SANCHEZ LADY MARGOT</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
@@ -3234,7 +3234,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>ROJAS SANCHEZ LADY MARGOT</t>
+          <t>ROMERO RODAS SILVIA MARELIS</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
@@ -3294,11 +3294,11 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>ROMERO RODAS SILVIA MARELIS</t>
+          <t>RUIZ TINIZARAY YOHANNA MARYURI</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
-        <v>0</v>
+        <v>118.96</v>
       </c>
       <c r="D47" s="2" t="n">
         <v>0</v>
@@ -3354,11 +3354,11 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>RUIZ TINIZARAY YOHANNA MARYURI</t>
+          <t>SALAS NOBLECILLA MARIA SUSANA</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
-        <v>118.96</v>
+        <v>0</v>
       </c>
       <c r="D48" s="2" t="n">
         <v>0</v>
@@ -3414,7 +3414,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>SALAS NOBLECILLA MARIA SUSANA</t>
+          <t>SALDARRIAGA ECHEVERRIA BRYAN STEVEN</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
@@ -3474,7 +3474,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>SALDARRIAGA ECHEVERRIA BRYAN STEVEN</t>
+          <t>SANDIEGO NEUMATICOS &amp; SERVICIOS CIA LTDA</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
@@ -3508,7 +3508,7 @@
         <v>0</v>
       </c>
       <c r="M50" s="2" t="n">
-        <v>0</v>
+        <v>762.85</v>
       </c>
       <c r="N50" s="2" t="n">
         <v>0</v>
@@ -3534,7 +3534,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>SANDIEGO NEUMATICOS &amp; SERVICIOS CIA LTDA</t>
+          <t>SOLANO DE LA SALA PAZ GONZALO PATRICIO</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
@@ -3568,7 +3568,7 @@
         <v>0</v>
       </c>
       <c r="M51" s="2" t="n">
-        <v>762.85</v>
+        <v>0</v>
       </c>
       <c r="N51" s="2" t="n">
         <v>0</v>
@@ -3594,7 +3594,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>SOLANO DE LA SALA PAZ GONZALO PATRICIO</t>
+          <t>TORO BLACIO MARIA DEL CISNE</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
@@ -3654,7 +3654,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>TORO BLACIO MARIA DEL CISNE</t>
+          <t>WONG SANCHEZ CLAUDIA PAULINA</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
@@ -3688,7 +3688,7 @@
         <v>0</v>
       </c>
       <c r="M53" s="2" t="n">
-        <v>0</v>
+        <v>829.09</v>
       </c>
       <c r="N53" s="2" t="n">
         <v>0</v>
@@ -3714,7 +3714,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>WONG SANCHEZ CLAUDIA PAULINA</t>
+          <t>WONG SANCHEZ PAULA SOFIA</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
@@ -3748,7 +3748,7 @@
         <v>0</v>
       </c>
       <c r="M54" s="2" t="n">
-        <v>829.09</v>
+        <v>0</v>
       </c>
       <c r="N54" s="2" t="n">
         <v>0</v>
@@ -3774,7 +3774,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>WONG SANCHEZ PAULA SOFIA</t>
+          <t>ZUÑIGA CORONEL MARCIA LUZMILA</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
@@ -3827,144 +3827,84 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>GUERRERO FAREZ FABIAN MAURICIO</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>ZUÑIGA CORONEL MARCIA LUZMILA</t>
-        </is>
-      </c>
-      <c r="C56" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D56" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E56" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F56" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G56" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H56" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I56" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J56" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K56" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L56" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M56" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N56" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O56" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P56" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q56" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R56" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="C57" s="4" t="inlineStr">
-        <is>
-          <t>1 de 55</t>
-        </is>
-      </c>
-      <c r="D57" s="4" t="inlineStr">
-        <is>
-          <t>4 de 55</t>
-        </is>
-      </c>
-      <c r="E57" s="4" t="inlineStr">
-        <is>
-          <t>0 de 55</t>
-        </is>
-      </c>
-      <c r="F57" s="4" t="inlineStr">
-        <is>
-          <t>0 de 55</t>
-        </is>
-      </c>
-      <c r="G57" s="4" t="inlineStr">
-        <is>
-          <t>0 de 55</t>
-        </is>
-      </c>
-      <c r="H57" s="4" t="inlineStr">
-        <is>
-          <t>0 de 55</t>
-        </is>
-      </c>
-      <c r="I57" s="4" t="inlineStr">
-        <is>
-          <t>2 de 55</t>
-        </is>
-      </c>
-      <c r="J57" s="4" t="inlineStr">
-        <is>
-          <t>0 de 55</t>
-        </is>
-      </c>
-      <c r="K57" s="4" t="inlineStr">
-        <is>
-          <t>3 de 55</t>
-        </is>
-      </c>
-      <c r="L57" s="4" t="inlineStr">
-        <is>
-          <t>1 de 55</t>
-        </is>
-      </c>
-      <c r="M57" s="4" t="inlineStr">
-        <is>
-          <t>11 de 55</t>
-        </is>
-      </c>
-      <c r="N57" s="4" t="inlineStr">
-        <is>
-          <t>1 de 55</t>
-        </is>
-      </c>
-      <c r="O57" s="4" t="inlineStr">
-        <is>
-          <t>0 de 55</t>
-        </is>
-      </c>
-      <c r="P57" s="4" t="inlineStr">
-        <is>
-          <t>1 de 55</t>
-        </is>
-      </c>
-      <c r="Q57" s="4" t="inlineStr">
-        <is>
-          <t>0 de 55</t>
-        </is>
-      </c>
-      <c r="R57" s="4" t="inlineStr">
-        <is>
-          <t>0 de 55</t>
+      <c r="C56" s="4" t="inlineStr">
+        <is>
+          <t>1 de 54</t>
+        </is>
+      </c>
+      <c r="D56" s="4" t="inlineStr">
+        <is>
+          <t>4 de 54</t>
+        </is>
+      </c>
+      <c r="E56" s="4" t="inlineStr">
+        <is>
+          <t>0 de 54</t>
+        </is>
+      </c>
+      <c r="F56" s="4" t="inlineStr">
+        <is>
+          <t>0 de 54</t>
+        </is>
+      </c>
+      <c r="G56" s="4" t="inlineStr">
+        <is>
+          <t>0 de 54</t>
+        </is>
+      </c>
+      <c r="H56" s="4" t="inlineStr">
+        <is>
+          <t>0 de 54</t>
+        </is>
+      </c>
+      <c r="I56" s="4" t="inlineStr">
+        <is>
+          <t>2 de 54</t>
+        </is>
+      </c>
+      <c r="J56" s="4" t="inlineStr">
+        <is>
+          <t>0 de 54</t>
+        </is>
+      </c>
+      <c r="K56" s="4" t="inlineStr">
+        <is>
+          <t>3 de 54</t>
+        </is>
+      </c>
+      <c r="L56" s="4" t="inlineStr">
+        <is>
+          <t>1 de 54</t>
+        </is>
+      </c>
+      <c r="M56" s="4" t="inlineStr">
+        <is>
+          <t>11 de 54</t>
+        </is>
+      </c>
+      <c r="N56" s="4" t="inlineStr">
+        <is>
+          <t>1 de 54</t>
+        </is>
+      </c>
+      <c r="O56" s="4" t="inlineStr">
+        <is>
+          <t>0 de 54</t>
+        </is>
+      </c>
+      <c r="P56" s="4" t="inlineStr">
+        <is>
+          <t>1 de 54</t>
+        </is>
+      </c>
+      <c r="Q56" s="4" t="inlineStr">
+        <is>
+          <t>0 de 54</t>
+        </is>
+      </c>
+      <c r="R56" s="4" t="inlineStr">
+        <is>
+          <t>0 de 54</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática 2026-06-29 08:30:22
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R56"/>
+  <dimension ref="A1:R55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2394,7 +2394,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>MONTESDEOCA ROBLES MARIA HILDA</t>
+          <t>OCHOA CUEVA LUIS DAVID</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
@@ -2454,7 +2454,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>OCHOA CUEVA LUIS DAVID</t>
+          <t>OJEDA GONZALEZ EDWIN FERNANDO</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
@@ -2482,7 +2482,7 @@
         <v>0</v>
       </c>
       <c r="K33" s="2" t="n">
-        <v>0</v>
+        <v>18.27</v>
       </c>
       <c r="L33" s="2" t="n">
         <v>0</v>
@@ -2514,7 +2514,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>OJEDA GONZALEZ EDWIN FERNANDO</t>
+          <t>ORTEGA ROMAN KLEBER ERWIN</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
@@ -2542,13 +2542,13 @@
         <v>0</v>
       </c>
       <c r="K34" s="2" t="n">
-        <v>18.27</v>
+        <v>50.76</v>
       </c>
       <c r="L34" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M34" s="2" t="n">
-        <v>0</v>
+        <v>113.72</v>
       </c>
       <c r="N34" s="2" t="n">
         <v>0</v>
@@ -2574,14 +2574,14 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>ORTEGA ROMAN KLEBER ERWIN</t>
+          <t>ORTEGA ROMAN LUIS FERNANDO</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D35" s="2" t="n">
-        <v>0</v>
+        <v>2045.73</v>
       </c>
       <c r="E35" s="2" t="n">
         <v>0</v>
@@ -2596,19 +2596,19 @@
         <v>0</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>0</v>
+        <v>251.27</v>
       </c>
       <c r="J35" s="2" t="n">
         <v>0</v>
       </c>
       <c r="K35" s="2" t="n">
-        <v>50.76</v>
+        <v>0</v>
       </c>
       <c r="L35" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M35" s="2" t="n">
-        <v>113.72</v>
+        <v>810.3099999999999</v>
       </c>
       <c r="N35" s="2" t="n">
         <v>0</v>
@@ -2634,14 +2634,14 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>ORTEGA ROMAN LUIS FERNANDO</t>
+          <t>PACHECO NIVICELA DORIS PRICILA</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D36" s="2" t="n">
-        <v>2045.73</v>
+        <v>0</v>
       </c>
       <c r="E36" s="2" t="n">
         <v>0</v>
@@ -2656,7 +2656,7 @@
         <v>0</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>251.27</v>
+        <v>0</v>
       </c>
       <c r="J36" s="2" t="n">
         <v>0</v>
@@ -2668,10 +2668,10 @@
         <v>0</v>
       </c>
       <c r="M36" s="2" t="n">
-        <v>810.3099999999999</v>
+        <v>0</v>
       </c>
       <c r="N36" s="2" t="n">
-        <v>0</v>
+        <v>1714.5</v>
       </c>
       <c r="O36" s="2" t="n">
         <v>0</v>
@@ -2694,7 +2694,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>PACHECO NIVICELA DORIS PRICILA</t>
+          <t>PACHECO NIVICELA SANDRA ELISABETH</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
@@ -2731,7 +2731,7 @@
         <v>0</v>
       </c>
       <c r="N37" s="2" t="n">
-        <v>1714.5</v>
+        <v>0</v>
       </c>
       <c r="O37" s="2" t="n">
         <v>0</v>
@@ -2754,7 +2754,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>PACHECO NIVICELA SANDRA ELISABETH</t>
+          <t>PEREZ ROSALES EDGAR RICARDO</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
@@ -2814,7 +2814,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>PEREZ ROSALES EDGAR RICARDO</t>
+          <t>PEÑALOZA LOPEZ RONALD STALIN</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
@@ -2874,7 +2874,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>PEÑALOZA LOPEZ RONALD STALIN</t>
+          <t>QUEZADA VEGA JAIME PATRICIO</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
@@ -2934,7 +2934,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>QUEZADA VEGA JAIME PATRICIO</t>
+          <t>QUINCHE ALCIVAR ARGENTINA DEL ROCIO</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
@@ -2994,7 +2994,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>QUINCHE ALCIVAR ARGENTINA DEL ROCIO</t>
+          <t>RAMIREZ APOLO JOBANI DE JESUS</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
@@ -3054,7 +3054,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>RAMIREZ APOLO JOBANI DE JESUS</t>
+          <t>REYES MOSCOSO NARCISA DE JESUS</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
@@ -3114,7 +3114,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>REYES MOSCOSO NARCISA DE JESUS</t>
+          <t>ROJAS SANCHEZ LADY MARGOT</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
@@ -3174,7 +3174,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>ROJAS SANCHEZ LADY MARGOT</t>
+          <t>ROMERO RODAS SILVIA MARELIS</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
@@ -3208,7 +3208,7 @@
         <v>0</v>
       </c>
       <c r="M45" s="2" t="n">
-        <v>0</v>
+        <v>90.98</v>
       </c>
       <c r="N45" s="2" t="n">
         <v>0</v>
@@ -3234,11 +3234,11 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>ROMERO RODAS SILVIA MARELIS</t>
+          <t>RUIZ TINIZARAY YOHANNA MARYURI</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
-        <v>0</v>
+        <v>118.96</v>
       </c>
       <c r="D46" s="2" t="n">
         <v>0</v>
@@ -3268,7 +3268,7 @@
         <v>0</v>
       </c>
       <c r="M46" s="2" t="n">
-        <v>90.98</v>
+        <v>0</v>
       </c>
       <c r="N46" s="2" t="n">
         <v>0</v>
@@ -3294,11 +3294,11 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>RUIZ TINIZARAY YOHANNA MARYURI</t>
+          <t>SALAS NOBLECILLA MARIA SUSANA</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
-        <v>118.96</v>
+        <v>0</v>
       </c>
       <c r="D47" s="2" t="n">
         <v>0</v>
@@ -3354,7 +3354,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>SALAS NOBLECILLA MARIA SUSANA</t>
+          <t>SALDARRIAGA ECHEVERRIA BRYAN STEVEN</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
@@ -3414,7 +3414,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>SALDARRIAGA ECHEVERRIA BRYAN STEVEN</t>
+          <t>SANDIEGO NEUMATICOS &amp; SERVICIOS CIA LTDA</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
@@ -3448,7 +3448,7 @@
         <v>0</v>
       </c>
       <c r="M49" s="2" t="n">
-        <v>0</v>
+        <v>762.85</v>
       </c>
       <c r="N49" s="2" t="n">
         <v>0</v>
@@ -3474,7 +3474,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>SANDIEGO NEUMATICOS &amp; SERVICIOS CIA LTDA</t>
+          <t>SOLANO DE LA SALA PAZ GONZALO PATRICIO</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
@@ -3508,7 +3508,7 @@
         <v>0</v>
       </c>
       <c r="M50" s="2" t="n">
-        <v>762.85</v>
+        <v>0</v>
       </c>
       <c r="N50" s="2" t="n">
         <v>0</v>
@@ -3534,7 +3534,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>SOLANO DE LA SALA PAZ GONZALO PATRICIO</t>
+          <t>TORO BLACIO MARIA DEL CISNE</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
@@ -3594,7 +3594,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>TORO BLACIO MARIA DEL CISNE</t>
+          <t>WONG SANCHEZ CLAUDIA PAULINA</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
@@ -3628,7 +3628,7 @@
         <v>0</v>
       </c>
       <c r="M52" s="2" t="n">
-        <v>0</v>
+        <v>829.09</v>
       </c>
       <c r="N52" s="2" t="n">
         <v>0</v>
@@ -3654,7 +3654,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>WONG SANCHEZ CLAUDIA PAULINA</t>
+          <t>WONG SANCHEZ PAULA SOFIA</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
@@ -3688,7 +3688,7 @@
         <v>0</v>
       </c>
       <c r="M53" s="2" t="n">
-        <v>829.09</v>
+        <v>0</v>
       </c>
       <c r="N53" s="2" t="n">
         <v>0</v>
@@ -3714,7 +3714,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>WONG SANCHEZ PAULA SOFIA</t>
+          <t>ZUÑIGA CORONEL MARCIA LUZMILA</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
@@ -3767,144 +3767,84 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>GUERRERO FAREZ FABIAN MAURICIO</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>ZUÑIGA CORONEL MARCIA LUZMILA</t>
-        </is>
-      </c>
-      <c r="C55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R55" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="C56" s="4" t="inlineStr">
-        <is>
-          <t>1 de 54</t>
-        </is>
-      </c>
-      <c r="D56" s="4" t="inlineStr">
-        <is>
-          <t>4 de 54</t>
-        </is>
-      </c>
-      <c r="E56" s="4" t="inlineStr">
-        <is>
-          <t>0 de 54</t>
-        </is>
-      </c>
-      <c r="F56" s="4" t="inlineStr">
-        <is>
-          <t>0 de 54</t>
-        </is>
-      </c>
-      <c r="G56" s="4" t="inlineStr">
-        <is>
-          <t>0 de 54</t>
-        </is>
-      </c>
-      <c r="H56" s="4" t="inlineStr">
-        <is>
-          <t>0 de 54</t>
-        </is>
-      </c>
-      <c r="I56" s="4" t="inlineStr">
-        <is>
-          <t>2 de 54</t>
-        </is>
-      </c>
-      <c r="J56" s="4" t="inlineStr">
-        <is>
-          <t>0 de 54</t>
-        </is>
-      </c>
-      <c r="K56" s="4" t="inlineStr">
-        <is>
-          <t>3 de 54</t>
-        </is>
-      </c>
-      <c r="L56" s="4" t="inlineStr">
-        <is>
-          <t>1 de 54</t>
-        </is>
-      </c>
-      <c r="M56" s="4" t="inlineStr">
-        <is>
-          <t>12 de 54</t>
-        </is>
-      </c>
-      <c r="N56" s="4" t="inlineStr">
-        <is>
-          <t>1 de 54</t>
-        </is>
-      </c>
-      <c r="O56" s="4" t="inlineStr">
-        <is>
-          <t>0 de 54</t>
-        </is>
-      </c>
-      <c r="P56" s="4" t="inlineStr">
-        <is>
-          <t>1 de 54</t>
-        </is>
-      </c>
-      <c r="Q56" s="4" t="inlineStr">
-        <is>
-          <t>0 de 54</t>
-        </is>
-      </c>
-      <c r="R56" s="4" t="inlineStr">
-        <is>
-          <t>0 de 54</t>
+      <c r="C55" s="4" t="inlineStr">
+        <is>
+          <t>1 de 53</t>
+        </is>
+      </c>
+      <c r="D55" s="4" t="inlineStr">
+        <is>
+          <t>4 de 53</t>
+        </is>
+      </c>
+      <c r="E55" s="4" t="inlineStr">
+        <is>
+          <t>0 de 53</t>
+        </is>
+      </c>
+      <c r="F55" s="4" t="inlineStr">
+        <is>
+          <t>0 de 53</t>
+        </is>
+      </c>
+      <c r="G55" s="4" t="inlineStr">
+        <is>
+          <t>0 de 53</t>
+        </is>
+      </c>
+      <c r="H55" s="4" t="inlineStr">
+        <is>
+          <t>0 de 53</t>
+        </is>
+      </c>
+      <c r="I55" s="4" t="inlineStr">
+        <is>
+          <t>2 de 53</t>
+        </is>
+      </c>
+      <c r="J55" s="4" t="inlineStr">
+        <is>
+          <t>0 de 53</t>
+        </is>
+      </c>
+      <c r="K55" s="4" t="inlineStr">
+        <is>
+          <t>3 de 53</t>
+        </is>
+      </c>
+      <c r="L55" s="4" t="inlineStr">
+        <is>
+          <t>1 de 53</t>
+        </is>
+      </c>
+      <c r="M55" s="4" t="inlineStr">
+        <is>
+          <t>12 de 53</t>
+        </is>
+      </c>
+      <c r="N55" s="4" t="inlineStr">
+        <is>
+          <t>1 de 53</t>
+        </is>
+      </c>
+      <c r="O55" s="4" t="inlineStr">
+        <is>
+          <t>0 de 53</t>
+        </is>
+      </c>
+      <c r="P55" s="4" t="inlineStr">
+        <is>
+          <t>1 de 53</t>
+        </is>
+      </c>
+      <c r="Q55" s="4" t="inlineStr">
+        <is>
+          <t>0 de 53</t>
+        </is>
+      </c>
+      <c r="R55" s="4" t="inlineStr">
+        <is>
+          <t>0 de 53</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática 2026-06-29 17:30:20
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -1408,7 +1408,7 @@
         <v>0</v>
       </c>
       <c r="M15" s="2" t="n">
-        <v>15.48</v>
+        <v>2910.78</v>
       </c>
       <c r="N15" s="2" t="n">
         <v>0</v>
@@ -4253,7 +4253,7 @@
         <v>11354.85</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>15.48</v>
+        <v>2910.78</v>
       </c>
       <c r="G14" s="2" t="n">
         <v>6000</v>
@@ -5458,7 +5458,7 @@
         <v>98137.67</v>
       </c>
       <c r="F59" s="5" t="n">
-        <v>18541.95</v>
+        <v>21437.25</v>
       </c>
       <c r="G59" s="5" t="n">
         <v>114450</v>
@@ -5481,9 +5481,9 @@
     <col width="32" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5749,13 +5749,13 @@
         <v>72100</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>7178.17</v>
+        <v>10073.47</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>64921.83</v>
+        <v>62026.53</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>0.09955852981969487</v>
+        <v>0.1397152565880721</v>
       </c>
     </row>
     <row r="12">
@@ -5792,13 +5792,13 @@
         <v>83903.5</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>17712.86</v>
+        <v>20608.16</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>66190.64</v>
+        <v>63295.34</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.2111099060229907</v>
+        <v>0.2456174057101313</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-06-30 08:30:18
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -1621,7 +1621,7 @@
         <v>0</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>0</v>
+        <v>92.08</v>
       </c>
       <c r="E19" s="2" t="n">
         <v>0</v>
@@ -1648,7 +1648,7 @@
         <v>0</v>
       </c>
       <c r="M19" s="2" t="n">
-        <v>0</v>
+        <v>1680.59</v>
       </c>
       <c r="N19" s="2" t="n">
         <v>0</v>
@@ -3774,7 +3774,7 @@
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>4 de 53</t>
+          <t>5 de 53</t>
         </is>
       </c>
       <c r="E55" s="4" t="inlineStr">
@@ -3819,7 +3819,7 @@
       </c>
       <c r="M55" s="4" t="inlineStr">
         <is>
-          <t>12 de 53</t>
+          <t>13 de 53</t>
         </is>
       </c>
       <c r="N55" s="4" t="inlineStr">
@@ -4361,7 +4361,7 @@
         <v>2189.65</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>0</v>
+        <v>1772.67</v>
       </c>
       <c r="G18" s="2" t="n">
         <v>500</v>
@@ -5458,7 +5458,7 @@
         <v>98137.67</v>
       </c>
       <c r="F59" s="5" t="n">
-        <v>21437.25</v>
+        <v>23209.92</v>
       </c>
       <c r="G59" s="5" t="n">
         <v>114450</v>
@@ -5557,13 +5557,13 @@
         <v>7350</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>5808.58</v>
+        <v>5900.66</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>1541.42</v>
+        <v>1449.34</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>0.7902829931972789</v>
+        <v>0.8028108843537415</v>
       </c>
     </row>
     <row r="4">
@@ -5749,13 +5749,13 @@
         <v>72100</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>10073.47</v>
+        <v>11754.06</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>62026.53</v>
+        <v>60345.94</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>0.1397152565880721</v>
+        <v>0.1630244105409154</v>
       </c>
     </row>
     <row r="12">
@@ -5792,13 +5792,13 @@
         <v>83903.5</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>20608.16</v>
+        <v>22380.83</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>63295.34</v>
+        <v>61522.67000000001</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.2456174057101313</v>
+        <v>0.2667448914526808</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-06-30 13:30:18
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -748,7 +748,7 @@
         <v>0</v>
       </c>
       <c r="M4" s="2" t="n">
-        <v>3073.76</v>
+        <v>3704.63</v>
       </c>
       <c r="N4" s="2" t="n">
         <v>0</v>
@@ -2482,7 +2482,7 @@
         <v>0</v>
       </c>
       <c r="K33" s="2" t="n">
-        <v>18.27</v>
+        <v>170.55</v>
       </c>
       <c r="L33" s="2" t="n">
         <v>0</v>
@@ -3956,7 +3956,7 @@
         <v>299.83</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>3158.67</v>
+        <v>3789.54</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>15000</v>
@@ -4793,7 +4793,7 @@
         <v>186.76</v>
       </c>
       <c r="F34" s="2" t="n">
-        <v>115.38</v>
+        <v>306.5</v>
       </c>
       <c r="G34" s="2" t="n">
         <v>0</v>
@@ -5458,7 +5458,7 @@
         <v>98137.67</v>
       </c>
       <c r="F59" s="5" t="n">
-        <v>23209.92</v>
+        <v>24031.91</v>
       </c>
       <c r="G59" s="5" t="n">
         <v>114450</v>
@@ -5701,13 +5701,13 @@
         <v>800</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>155.32</v>
+        <v>307.6</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>644.6800000000001</v>
+        <v>492.4</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>0.19415</v>
+        <v>0.3845</v>
       </c>
     </row>
     <row r="10">
@@ -5725,13 +5725,13 @@
         <v>220</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>766.17</v>
+        <v>805.01</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>-546.17</v>
+        <v>-585.01</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>3.482590909090909</v>
+        <v>3.659136363636363</v>
       </c>
     </row>
     <row r="11">
@@ -5749,13 +5749,13 @@
         <v>72100</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>11754.06</v>
+        <v>12384.93</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>60345.94</v>
+        <v>59715.07</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>0.1630244105409154</v>
+        <v>0.1717743411927878</v>
       </c>
     </row>
     <row r="12">
@@ -5792,13 +5792,13 @@
         <v>83903.5</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>22380.83</v>
+        <v>23202.82</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>61522.67000000001</v>
+        <v>60700.68</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.2667448914526808</v>
+        <v>0.2765417414053049</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-07-07 16:30:17
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -745,7 +745,7 @@
         <v>0</v>
       </c>
       <c r="L4" s="2" t="n">
-        <v>0</v>
+        <v>1748.09</v>
       </c>
       <c r="M4" s="2" t="n">
         <v>0</v>
@@ -805,7 +805,7 @@
         <v>0</v>
       </c>
       <c r="L5" s="2" t="n">
-        <v>0</v>
+        <v>304.94</v>
       </c>
       <c r="M5" s="2" t="n">
         <v>0</v>
@@ -2908,7 +2908,7 @@
         <v>0</v>
       </c>
       <c r="M40" s="2" t="n">
-        <v>0</v>
+        <v>1388.57</v>
       </c>
       <c r="N40" s="2" t="n">
         <v>0</v>
@@ -3148,7 +3148,7 @@
         <v>0</v>
       </c>
       <c r="M44" s="2" t="n">
-        <v>0</v>
+        <v>1030.52</v>
       </c>
       <c r="N44" s="2" t="n">
         <v>0</v>
@@ -3814,12 +3814,12 @@
       </c>
       <c r="L55" s="4" t="inlineStr">
         <is>
-          <t>0 de 53</t>
+          <t>2 de 53</t>
         </is>
       </c>
       <c r="M55" s="4" t="inlineStr">
         <is>
-          <t>4 de 53</t>
+          <t>6 de 53</t>
         </is>
       </c>
       <c r="N55" s="4" t="inlineStr">
@@ -3956,7 +3956,7 @@
         <v>3789.54</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>0</v>
+        <v>1748.09</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>15000</v>
@@ -3983,7 +3983,7 @@
         <v>1581.4</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>312.26</v>
+        <v>617.2</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>10000</v>
@@ -5009,7 +5009,7 @@
         <v>0</v>
       </c>
       <c r="F42" s="2" t="n">
-        <v>0</v>
+        <v>1388.57</v>
       </c>
       <c r="G42" s="2" t="n">
         <v>2000</v>
@@ -5117,7 +5117,7 @@
         <v>0</v>
       </c>
       <c r="F46" s="2" t="n">
-        <v>0</v>
+        <v>1030.52</v>
       </c>
       <c r="G46" s="2" t="n">
         <v>1500</v>
@@ -5458,7 +5458,7 @@
         <v>23521.41</v>
       </c>
       <c r="F59" s="5" t="n">
-        <v>4586.91</v>
+        <v>9059.030000000001</v>
       </c>
       <c r="G59" s="5" t="n">
         <v>114450</v>

</xml_diff>

<commit_message>
Actualización automática 2026-07-07 17:30:16
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -805,7 +805,7 @@
         <v>0</v>
       </c>
       <c r="L5" s="2" t="n">
-        <v>304.94</v>
+        <v>924.0599999999999</v>
       </c>
       <c r="M5" s="2" t="n">
         <v>0</v>
@@ -2284,7 +2284,7 @@
         <v>0</v>
       </c>
       <c r="E30" s="2" t="n">
-        <v>0</v>
+        <v>131.59</v>
       </c>
       <c r="F30" s="2" t="n">
         <v>0</v>
@@ -2296,7 +2296,7 @@
         <v>0</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>0</v>
+        <v>48.33</v>
       </c>
       <c r="J30" s="2" t="n">
         <v>0</v>
@@ -3148,7 +3148,7 @@
         <v>0</v>
       </c>
       <c r="M44" s="2" t="n">
-        <v>1030.52</v>
+        <v>4377.51</v>
       </c>
       <c r="N44" s="2" t="n">
         <v>0</v>
@@ -3779,27 +3779,27 @@
       </c>
       <c r="E55" s="4" t="inlineStr">
         <is>
+          <t>1 de 53</t>
+        </is>
+      </c>
+      <c r="F55" s="4" t="inlineStr">
+        <is>
           <t>0 de 53</t>
         </is>
       </c>
-      <c r="F55" s="4" t="inlineStr">
+      <c r="G55" s="4" t="inlineStr">
         <is>
           <t>0 de 53</t>
         </is>
       </c>
-      <c r="G55" s="4" t="inlineStr">
+      <c r="H55" s="4" t="inlineStr">
         <is>
           <t>0 de 53</t>
         </is>
       </c>
-      <c r="H55" s="4" t="inlineStr">
-        <is>
-          <t>0 de 53</t>
-        </is>
-      </c>
       <c r="I55" s="4" t="inlineStr">
         <is>
-          <t>0 de 53</t>
+          <t>1 de 53</t>
         </is>
       </c>
       <c r="J55" s="4" t="inlineStr">
@@ -3983,7 +3983,7 @@
         <v>1581.4</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>617.2</v>
+        <v>1236.32</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>10000</v>
@@ -4685,7 +4685,7 @@
         <v>16.74</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>0</v>
+        <v>179.92</v>
       </c>
       <c r="G30" s="2" t="n">
         <v>1500</v>
@@ -5117,7 +5117,7 @@
         <v>0</v>
       </c>
       <c r="F46" s="2" t="n">
-        <v>1030.52</v>
+        <v>4377.51</v>
       </c>
       <c r="G46" s="2" t="n">
         <v>1500</v>
@@ -5458,7 +5458,7 @@
         <v>23521.41</v>
       </c>
       <c r="F59" s="5" t="n">
-        <v>9059.030000000001</v>
+        <v>13205.06</v>
       </c>
       <c r="G59" s="5" t="n">
         <v>114450</v>

</xml_diff>

<commit_message>
Actualización automática 2026-07-08 13:30:16
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -2113,7 +2113,7 @@
         <v>0</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>0</v>
+        <v>-65.18000000000001</v>
       </c>
       <c r="I27" s="2" t="n">
         <v>0</v>
@@ -4604,7 +4604,7 @@
         <v>0</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>0</v>
+        <v>-65.18000000000001</v>
       </c>
       <c r="G27" s="2" t="n">
         <v>1500</v>
@@ -5458,7 +5458,7 @@
         <v>23521.41</v>
       </c>
       <c r="F59" s="5" t="n">
-        <v>13245.81</v>
+        <v>13180.63</v>
       </c>
       <c r="G59" s="5" t="n">
         <v>114450</v>

</xml_diff>

<commit_message>
Actualización automática 2026-07-10 08:30:15
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -1861,7 +1861,7 @@
         <v>0</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>0</v>
+        <v>1079.4</v>
       </c>
       <c r="E23" s="2" t="n">
         <v>0</v>
@@ -1888,7 +1888,7 @@
         <v>0</v>
       </c>
       <c r="M23" s="2" t="n">
-        <v>0</v>
+        <v>1167.57</v>
       </c>
       <c r="N23" s="2" t="n">
         <v>0</v>
@@ -2608,7 +2608,7 @@
         <v>0</v>
       </c>
       <c r="M35" s="2" t="n">
-        <v>0</v>
+        <v>836.66</v>
       </c>
       <c r="N35" s="2" t="n">
         <v>0</v>
@@ -3145,7 +3145,7 @@
         <v>0</v>
       </c>
       <c r="L44" s="2" t="n">
-        <v>0</v>
+        <v>151.53</v>
       </c>
       <c r="M44" s="2" t="n">
         <v>4377.51</v>
@@ -3774,7 +3774,7 @@
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>2 de 53</t>
+          <t>3 de 53</t>
         </is>
       </c>
       <c r="E55" s="4" t="inlineStr">
@@ -3814,12 +3814,12 @@
       </c>
       <c r="L55" s="4" t="inlineStr">
         <is>
-          <t>2 de 53</t>
+          <t>3 de 53</t>
         </is>
       </c>
       <c r="M55" s="4" t="inlineStr">
         <is>
-          <t>7 de 53</t>
+          <t>9 de 53</t>
         </is>
       </c>
       <c r="N55" s="4" t="inlineStr">
@@ -4469,7 +4469,7 @@
         <v>0</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>0</v>
+        <v>2246.97</v>
       </c>
       <c r="G22" s="2" t="n">
         <v>15000</v>
@@ -4847,7 +4847,7 @@
         <v>3107.31</v>
       </c>
       <c r="F36" s="2" t="n">
-        <v>0</v>
+        <v>836.66</v>
       </c>
       <c r="G36" s="2" t="n">
         <v>8000</v>
@@ -5117,7 +5117,7 @@
         <v>0</v>
       </c>
       <c r="F46" s="2" t="n">
-        <v>4377.51</v>
+        <v>4529.04</v>
       </c>
       <c r="G46" s="2" t="n">
         <v>1500</v>
@@ -5458,7 +5458,7 @@
         <v>23521.41</v>
       </c>
       <c r="F59" s="5" t="n">
-        <v>14317.3</v>
+        <v>17552.46</v>
       </c>
       <c r="G59" s="5" t="n">
         <v>114450</v>

</xml_diff>

<commit_message>
Actualización automática 2026-07-13 17:30:16
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -748,7 +748,7 @@
         <v>1748.09</v>
       </c>
       <c r="M4" s="2" t="n">
-        <v>0</v>
+        <v>-19.12</v>
       </c>
       <c r="N4" s="2" t="n">
         <v>0</v>
@@ -3956,7 +3956,7 @@
         <v>3789.54</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>2827.99</v>
+        <v>2808.87</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>15000</v>
@@ -5458,7 +5458,7 @@
         <v>23521.41</v>
       </c>
       <c r="F59" s="5" t="n">
-        <v>17552.46</v>
+        <v>17533.34</v>
       </c>
       <c r="G59" s="5" t="n">
         <v>114450</v>

</xml_diff>

<commit_message>
Actualización automática 2026-07-15 15:30:17
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -2188,7 +2188,7 @@
         <v>0</v>
       </c>
       <c r="M28" s="2" t="n">
-        <v>0</v>
+        <v>69.89</v>
       </c>
       <c r="N28" s="2" t="n">
         <v>0</v>
@@ -2548,7 +2548,7 @@
         <v>0</v>
       </c>
       <c r="M34" s="2" t="n">
-        <v>0</v>
+        <v>57.25</v>
       </c>
       <c r="N34" s="2" t="n">
         <v>0</v>
@@ -3819,7 +3819,7 @@
       </c>
       <c r="M55" s="4" t="inlineStr">
         <is>
-          <t>9 de 53</t>
+          <t>11 de 53</t>
         </is>
       </c>
       <c r="N55" s="4" t="inlineStr">
@@ -4631,7 +4631,7 @@
         <v>2107.43</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>0</v>
+        <v>69.89</v>
       </c>
       <c r="G28" s="2" t="n">
         <v>6000</v>
@@ -4820,7 +4820,7 @@
         <v>164.48</v>
       </c>
       <c r="F35" s="2" t="n">
-        <v>4298.83</v>
+        <v>4356.08</v>
       </c>
       <c r="G35" s="2" t="n">
         <v>10000</v>
@@ -5458,7 +5458,7 @@
         <v>23521.41</v>
       </c>
       <c r="F59" s="5" t="n">
-        <v>17533.34</v>
+        <v>17660.48</v>
       </c>
       <c r="G59" s="5" t="n">
         <v>114450</v>
@@ -5773,13 +5773,13 @@
         <v>55052</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>8033.24</v>
+        <v>8160.38</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>47018.76</v>
+        <v>46891.62</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0.1459209474678486</v>
+        <v>0.1482304003487612</v>
       </c>
     </row>
     <row r="13">
@@ -5816,13 +5816,13 @@
         <v>72543.32000000001</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>17479.77</v>
+        <v>17606.91</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>55063.55</v>
+        <v>54936.41</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.2409563003182099</v>
+        <v>0.2427089082771508</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-07-15 17:30:17
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -781,7 +781,7 @@
         <v>312.26</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>0</v>
+        <v>324.98</v>
       </c>
       <c r="E5" s="2" t="n">
         <v>0</v>
@@ -805,7 +805,7 @@
         <v>0</v>
       </c>
       <c r="L5" s="2" t="n">
-        <v>924.0599999999999</v>
+        <v>2380.8</v>
       </c>
       <c r="M5" s="2" t="n">
         <v>0</v>
@@ -1408,7 +1408,7 @@
         <v>0</v>
       </c>
       <c r="M15" s="2" t="n">
-        <v>0</v>
+        <v>7572.51</v>
       </c>
       <c r="N15" s="2" t="n">
         <v>0</v>
@@ -3148,7 +3148,7 @@
         <v>151.53</v>
       </c>
       <c r="M44" s="2" t="n">
-        <v>4377.51</v>
+        <v>7022.33</v>
       </c>
       <c r="N44" s="2" t="n">
         <v>0</v>
@@ -3774,52 +3774,52 @@
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
+          <t>4 de 53</t>
+        </is>
+      </c>
+      <c r="E55" s="4" t="inlineStr">
+        <is>
+          <t>1 de 53</t>
+        </is>
+      </c>
+      <c r="F55" s="4" t="inlineStr">
+        <is>
+          <t>0 de 53</t>
+        </is>
+      </c>
+      <c r="G55" s="4" t="inlineStr">
+        <is>
+          <t>0 de 53</t>
+        </is>
+      </c>
+      <c r="H55" s="4" t="inlineStr">
+        <is>
+          <t>0 de 53</t>
+        </is>
+      </c>
+      <c r="I55" s="4" t="inlineStr">
+        <is>
+          <t>1 de 53</t>
+        </is>
+      </c>
+      <c r="J55" s="4" t="inlineStr">
+        <is>
+          <t>0 de 53</t>
+        </is>
+      </c>
+      <c r="K55" s="4" t="inlineStr">
+        <is>
+          <t>0 de 53</t>
+        </is>
+      </c>
+      <c r="L55" s="4" t="inlineStr">
+        <is>
           <t>3 de 53</t>
         </is>
       </c>
-      <c r="E55" s="4" t="inlineStr">
-        <is>
-          <t>1 de 53</t>
-        </is>
-      </c>
-      <c r="F55" s="4" t="inlineStr">
-        <is>
-          <t>0 de 53</t>
-        </is>
-      </c>
-      <c r="G55" s="4" t="inlineStr">
-        <is>
-          <t>0 de 53</t>
-        </is>
-      </c>
-      <c r="H55" s="4" t="inlineStr">
-        <is>
-          <t>0 de 53</t>
-        </is>
-      </c>
-      <c r="I55" s="4" t="inlineStr">
-        <is>
-          <t>1 de 53</t>
-        </is>
-      </c>
-      <c r="J55" s="4" t="inlineStr">
-        <is>
-          <t>0 de 53</t>
-        </is>
-      </c>
-      <c r="K55" s="4" t="inlineStr">
-        <is>
-          <t>0 de 53</t>
-        </is>
-      </c>
-      <c r="L55" s="4" t="inlineStr">
-        <is>
-          <t>3 de 53</t>
-        </is>
-      </c>
       <c r="M55" s="4" t="inlineStr">
         <is>
-          <t>11 de 53</t>
+          <t>12 de 53</t>
         </is>
       </c>
       <c r="N55" s="4" t="inlineStr">
@@ -3983,7 +3983,7 @@
         <v>1581.4</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>1236.32</v>
+        <v>3018.04</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>10000</v>
@@ -4253,7 +4253,7 @@
         <v>2910.78</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>0</v>
+        <v>7572.51</v>
       </c>
       <c r="G14" s="2" t="n">
         <v>6000</v>
@@ -5117,7 +5117,7 @@
         <v>0</v>
       </c>
       <c r="F46" s="2" t="n">
-        <v>4529.04</v>
+        <v>7173.86</v>
       </c>
       <c r="G46" s="2" t="n">
         <v>1500</v>
@@ -5458,7 +5458,7 @@
         <v>23521.41</v>
       </c>
       <c r="F59" s="5" t="n">
-        <v>17660.48</v>
+        <v>29659.53</v>
       </c>
       <c r="G59" s="5" t="n">
         <v>114450</v>
@@ -5481,8 +5481,8 @@
     <col width="32" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="23" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
     <col width="26" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -5557,13 +5557,13 @@
         <v>6600</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>6508.89</v>
+        <v>6833.87</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>91.10999999999967</v>
+        <v>-233.8699999999999</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>0.9861954545454545</v>
+        <v>1.035434848484849</v>
       </c>
     </row>
     <row r="4">
@@ -5749,13 +5749,13 @@
         <v>7700</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>2823.68</v>
+        <v>4280.42</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>4876.32</v>
+        <v>3419.58</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>0.3667116883116883</v>
+        <v>0.5558987012987013</v>
       </c>
     </row>
     <row r="12">
@@ -5773,13 +5773,13 @@
         <v>55052</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>8160.38</v>
+        <v>18377.71</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>46891.62</v>
+        <v>36674.29</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0.1482304003487612</v>
+        <v>0.3338245658650004</v>
       </c>
     </row>
     <row r="13">
@@ -5816,13 +5816,13 @@
         <v>72543.32000000001</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>17606.91</v>
+        <v>29605.96</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>54936.41</v>
+        <v>42937.36</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.2427089082771508</v>
+        <v>0.4081142136863876</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-07-16 14:30:17
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -1288,7 +1288,7 @@
         <v>0</v>
       </c>
       <c r="M13" s="2" t="n">
-        <v>0</v>
+        <v>126.44</v>
       </c>
       <c r="N13" s="2" t="n">
         <v>0</v>
@@ -2788,7 +2788,7 @@
         <v>0</v>
       </c>
       <c r="M38" s="2" t="n">
-        <v>56.77</v>
+        <v>223.69</v>
       </c>
       <c r="N38" s="2" t="n">
         <v>0</v>
@@ -3819,7 +3819,7 @@
       </c>
       <c r="M55" s="4" t="inlineStr">
         <is>
-          <t>12 de 53</t>
+          <t>13 de 53</t>
         </is>
       </c>
       <c r="N55" s="4" t="inlineStr">
@@ -4199,7 +4199,7 @@
         <v>564.64</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>0</v>
+        <v>126.44</v>
       </c>
       <c r="G12" s="2" t="n">
         <v>6000</v>
@@ -4955,7 +4955,7 @@
         <v>118.96</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>-62.19</v>
+        <v>104.73</v>
       </c>
       <c r="G40" s="2" t="n">
         <v>3500</v>
@@ -5458,7 +5458,7 @@
         <v>23521.41</v>
       </c>
       <c r="F59" s="5" t="n">
-        <v>29659.53</v>
+        <v>29952.89</v>
       </c>
       <c r="G59" s="5" t="n">
         <v>114450</v>
@@ -5773,13 +5773,13 @@
         <v>55052</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>18377.71</v>
+        <v>18671.07</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>36674.29</v>
+        <v>36380.93</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0.3338245658650004</v>
+        <v>0.3391533459274867</v>
       </c>
     </row>
     <row r="13">
@@ -5816,13 +5816,13 @@
         <v>72543.32000000001</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>29605.96</v>
+        <v>29899.32</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>42937.36</v>
+        <v>42644</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.4081142136863876</v>
+        <v>0.4121581421969658</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-07-16 16:30:18
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -718,7 +718,7 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0</v>
+        <v>312.26</v>
       </c>
       <c r="D4" s="2" t="n">
         <v>1079.9</v>
@@ -748,7 +748,7 @@
         <v>1748.09</v>
       </c>
       <c r="M4" s="2" t="n">
-        <v>-19.12</v>
+        <v>32.8</v>
       </c>
       <c r="N4" s="2" t="n">
         <v>0</v>
@@ -1888,7 +1888,7 @@
         <v>0</v>
       </c>
       <c r="M23" s="2" t="n">
-        <v>1167.57</v>
+        <v>1253.45</v>
       </c>
       <c r="N23" s="2" t="n">
         <v>0</v>
@@ -2824,7 +2824,7 @@
         <v>0</v>
       </c>
       <c r="E39" s="2" t="n">
-        <v>0</v>
+        <v>129.61</v>
       </c>
       <c r="F39" s="2" t="n">
         <v>0</v>
@@ -2848,7 +2848,7 @@
         <v>0</v>
       </c>
       <c r="M39" s="2" t="n">
-        <v>0</v>
+        <v>1335.87</v>
       </c>
       <c r="N39" s="2" t="n">
         <v>0</v>
@@ -3241,7 +3241,7 @@
         <v>0</v>
       </c>
       <c r="D46" s="2" t="n">
-        <v>0</v>
+        <v>1819.81</v>
       </c>
       <c r="E46" s="2" t="n">
         <v>0</v>
@@ -3769,49 +3769,49 @@
     <row r="55">
       <c r="C55" s="4" t="inlineStr">
         <is>
+          <t>2 de 53</t>
+        </is>
+      </c>
+      <c r="D55" s="4" t="inlineStr">
+        <is>
+          <t>5 de 53</t>
+        </is>
+      </c>
+      <c r="E55" s="4" t="inlineStr">
+        <is>
+          <t>2 de 53</t>
+        </is>
+      </c>
+      <c r="F55" s="4" t="inlineStr">
+        <is>
+          <t>0 de 53</t>
+        </is>
+      </c>
+      <c r="G55" s="4" t="inlineStr">
+        <is>
+          <t>0 de 53</t>
+        </is>
+      </c>
+      <c r="H55" s="4" t="inlineStr">
+        <is>
+          <t>0 de 53</t>
+        </is>
+      </c>
+      <c r="I55" s="4" t="inlineStr">
+        <is>
           <t>1 de 53</t>
         </is>
       </c>
-      <c r="D55" s="4" t="inlineStr">
-        <is>
-          <t>4 de 53</t>
-        </is>
-      </c>
-      <c r="E55" s="4" t="inlineStr">
-        <is>
-          <t>1 de 53</t>
-        </is>
-      </c>
-      <c r="F55" s="4" t="inlineStr">
+      <c r="J55" s="4" t="inlineStr">
         <is>
           <t>0 de 53</t>
         </is>
       </c>
-      <c r="G55" s="4" t="inlineStr">
+      <c r="K55" s="4" t="inlineStr">
         <is>
           <t>0 de 53</t>
         </is>
       </c>
-      <c r="H55" s="4" t="inlineStr">
-        <is>
-          <t>0 de 53</t>
-        </is>
-      </c>
-      <c r="I55" s="4" t="inlineStr">
-        <is>
-          <t>1 de 53</t>
-        </is>
-      </c>
-      <c r="J55" s="4" t="inlineStr">
-        <is>
-          <t>0 de 53</t>
-        </is>
-      </c>
-      <c r="K55" s="4" t="inlineStr">
-        <is>
-          <t>0 de 53</t>
-        </is>
-      </c>
       <c r="L55" s="4" t="inlineStr">
         <is>
           <t>3 de 53</t>
@@ -3819,7 +3819,7 @@
       </c>
       <c r="M55" s="4" t="inlineStr">
         <is>
-          <t>13 de 53</t>
+          <t>15 de 53</t>
         </is>
       </c>
       <c r="N55" s="4" t="inlineStr">
@@ -3956,7 +3956,7 @@
         <v>3789.54</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>2808.87</v>
+        <v>3173.05</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>15000</v>
@@ -4469,7 +4469,7 @@
         <v>0</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>2246.97</v>
+        <v>2332.85</v>
       </c>
       <c r="G22" s="2" t="n">
         <v>15000</v>
@@ -4982,7 +4982,7 @@
         <v>669.0599999999999</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>0</v>
+        <v>1465.48</v>
       </c>
       <c r="G41" s="2" t="n">
         <v>1000</v>
@@ -5171,7 +5171,7 @@
         <v>118.96</v>
       </c>
       <c r="F48" s="2" t="n">
-        <v>0</v>
+        <v>1819.81</v>
       </c>
       <c r="G48" s="2" t="n">
         <v>1500</v>
@@ -5458,7 +5458,7 @@
         <v>23521.41</v>
       </c>
       <c r="F59" s="5" t="n">
-        <v>29952.89</v>
+        <v>33688.24</v>
       </c>
       <c r="G59" s="5" t="n">
         <v>114450</v>
@@ -5533,13 +5533,13 @@
         <v>436</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>193.3</v>
+        <v>505.56</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>242.7</v>
+        <v>-69.56</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>0.4433486238532111</v>
+        <v>1.15954128440367</v>
       </c>
     </row>
     <row r="3">
@@ -5557,13 +5557,13 @@
         <v>6600</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>6833.87</v>
+        <v>8653.68</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>-233.8699999999999</v>
+        <v>-2053.68</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>1.035434848484849</v>
+        <v>1.311163636363636</v>
       </c>
     </row>
     <row r="4">
@@ -5581,13 +5581,13 @@
         <v>199.5</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>131.59</v>
+        <v>261.2</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>67.91</v>
+        <v>-61.69999999999999</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>0.6595989974937344</v>
+        <v>1.309273182957393</v>
       </c>
     </row>
     <row r="5">
@@ -5773,13 +5773,13 @@
         <v>55052</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>18671.07</v>
+        <v>20144.74</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>36380.93</v>
+        <v>34907.25999999999</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0.3391533459274867</v>
+        <v>0.3659220373465088</v>
       </c>
     </row>
     <row r="13">
@@ -5816,13 +5816,13 @@
         <v>72543.32000000001</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>29899.32</v>
+        <v>33634.67</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>42644</v>
+        <v>38908.64999999999</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.4121581421969658</v>
+        <v>0.4636494442217422</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-07-21 12:30:21
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -1528,7 +1528,7 @@
         <v>0</v>
       </c>
       <c r="M17" s="2" t="n">
-        <v>222.03</v>
+        <v>1355.61</v>
       </c>
       <c r="N17" s="2" t="n">
         <v>0</v>
@@ -4307,7 +4307,7 @@
         <v>-589.36</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>222.03</v>
+        <v>1355.61</v>
       </c>
       <c r="G16" s="2" t="n">
         <v>3000</v>
@@ -5458,7 +5458,7 @@
         <v>23521.41</v>
       </c>
       <c r="F59" s="5" t="n">
-        <v>33886.62</v>
+        <v>35020.2</v>
       </c>
       <c r="G59" s="5" t="n">
         <v>114450</v>
@@ -5481,7 +5481,7 @@
     <col width="32" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="26" customWidth="1" min="6" max="6"/>
   </cols>
@@ -5773,13 +5773,13 @@
         <v>55052</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>20343.12</v>
+        <v>21476.7</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>34708.88</v>
+        <v>33575.3</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0.3695255394899368</v>
+        <v>0.3901166170166388</v>
       </c>
     </row>
     <row r="13">
@@ -5816,13 +5816,13 @@
         <v>72543.32000000001</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>33833.05</v>
+        <v>34966.63</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>38710.27</v>
+        <v>37576.69</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.4663840860881471</v>
+        <v>0.4820103353416965</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-07-23 08:30:18
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -928,7 +928,7 @@
         <v>0</v>
       </c>
       <c r="M7" s="2" t="n">
-        <v>15.48</v>
+        <v>2318.68</v>
       </c>
       <c r="N7" s="2" t="n">
         <v>0</v>
@@ -1585,7 +1585,7 @@
         <v>0</v>
       </c>
       <c r="L18" s="2" t="n">
-        <v>0</v>
+        <v>3234.7</v>
       </c>
       <c r="M18" s="2" t="n">
         <v>74.73</v>
@@ -2188,7 +2188,7 @@
         <v>0</v>
       </c>
       <c r="M28" s="2" t="n">
-        <v>69.89</v>
+        <v>2808.93</v>
       </c>
       <c r="N28" s="2" t="n">
         <v>0</v>
@@ -2521,7 +2521,7 @@
         <v>0</v>
       </c>
       <c r="D34" s="2" t="n">
-        <v>4349.59</v>
+        <v>12655.12</v>
       </c>
       <c r="E34" s="2" t="n">
         <v>0</v>
@@ -3628,7 +3628,7 @@
         <v>0</v>
       </c>
       <c r="M52" s="2" t="n">
-        <v>53.57</v>
+        <v>334.62</v>
       </c>
       <c r="N52" s="2" t="n">
         <v>0</v>
@@ -3814,7 +3814,7 @@
       </c>
       <c r="L55" s="4" t="inlineStr">
         <is>
-          <t>3 de 53</t>
+          <t>4 de 53</t>
         </is>
       </c>
       <c r="M55" s="4" t="inlineStr">
@@ -3867,7 +3867,7 @@
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -4037,7 +4037,7 @@
         <v>982.99</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>15.48</v>
+        <v>2318.68</v>
       </c>
       <c r="G6" s="2" t="n">
         <v>1500</v>
@@ -4334,7 +4334,7 @@
         <v>16.74</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>74.73</v>
+        <v>3309.43</v>
       </c>
       <c r="G17" s="2" t="n">
         <v>1000</v>
@@ -4631,7 +4631,7 @@
         <v>2107.43</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>69.89</v>
+        <v>2808.93</v>
       </c>
       <c r="G28" s="2" t="n">
         <v>6000</v>
@@ -4820,7 +4820,7 @@
         <v>164.48</v>
       </c>
       <c r="F35" s="2" t="n">
-        <v>4356.08</v>
+        <v>12661.61</v>
       </c>
       <c r="G35" s="2" t="n">
         <v>10000</v>
@@ -5333,7 +5333,7 @@
         <v>829.09</v>
       </c>
       <c r="F54" s="2" t="n">
-        <v>53.57</v>
+        <v>334.62</v>
       </c>
       <c r="G54" s="2" t="n">
         <v>500</v>
@@ -5360,7 +5360,7 @@
         <v>829.09</v>
       </c>
       <c r="F55" s="2" t="n">
-        <v>53.57</v>
+        <v>334.62</v>
       </c>
       <c r="G55" s="2" t="n">
         <v>1000</v>
@@ -5458,7 +5458,7 @@
         <v>23521.41</v>
       </c>
       <c r="F59" s="5" t="n">
-        <v>35077.6</v>
+        <v>52222.17</v>
       </c>
       <c r="G59" s="5" t="n">
         <v>114450</v>
@@ -5481,7 +5481,7 @@
     <col width="32" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="26" customWidth="1" min="6" max="6"/>
   </cols>
@@ -5557,13 +5557,13 @@
         <v>6600</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>8653.68</v>
+        <v>16959.21</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>-2053.68</v>
+        <v>-10359.21</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>1.311163636363636</v>
+        <v>2.569577272727273</v>
       </c>
     </row>
     <row r="4">
@@ -5749,13 +5749,13 @@
         <v>7700</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>4280.42</v>
+        <v>7515.12</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>3419.58</v>
+        <v>184.8800000000001</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>0.5558987012987013</v>
+        <v>0.9759896103896104</v>
       </c>
     </row>
     <row r="12">
@@ -5773,13 +5773,13 @@
         <v>55052</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>21476.7</v>
+        <v>26799.99</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>33575.3</v>
+        <v>28252.01</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0.3901166170166388</v>
+        <v>0.4868122865654291</v>
       </c>
     </row>
     <row r="13">
@@ -5816,13 +5816,13 @@
         <v>72543.32000000001</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>35024.03</v>
+        <v>51887.55</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>37519.29</v>
+        <v>20655.77</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.4828015866933026</v>
+        <v>0.7152629628751482</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-07-23 10:30:18
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -2113,7 +2113,7 @@
         <v>0</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>-7.78</v>
+        <v>-65.18000000000001</v>
       </c>
       <c r="I27" s="2" t="n">
         <v>0</v>
@@ -4604,7 +4604,7 @@
         <v>0</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>-7.78</v>
+        <v>-65.18000000000001</v>
       </c>
       <c r="G27" s="2" t="n">
         <v>1500</v>
@@ -5458,7 +5458,7 @@
         <v>23521.41</v>
       </c>
       <c r="F59" s="5" t="n">
-        <v>52222.17</v>
+        <v>52164.77</v>
       </c>
       <c r="G59" s="5" t="n">
         <v>114450</v>
@@ -5677,10 +5677,10 @@
         <v>0</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>-151.1</v>
+        <v>-208.5</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>151.1</v>
+        <v>208.5</v>
       </c>
       <c r="F8" s="3" t="n">
         <v>0</v>
@@ -5816,13 +5816,13 @@
         <v>72543.32000000001</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>51887.55</v>
+        <v>51830.15000000001</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>20655.77</v>
+        <v>20713.17</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.7152629628751482</v>
+        <v>0.7144717115235422</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-07-28 08:30:17
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -748,7 +748,7 @@
         <v>1748.09</v>
       </c>
       <c r="M4" s="2" t="n">
-        <v>32.8</v>
+        <v>1448.77</v>
       </c>
       <c r="N4" s="2" t="n">
         <v>0</v>
@@ -808,7 +808,7 @@
         <v>2380.8</v>
       </c>
       <c r="M5" s="2" t="n">
-        <v>0</v>
+        <v>2830.46</v>
       </c>
       <c r="N5" s="2" t="n">
         <v>0</v>
@@ -1408,7 +1408,7 @@
         <v>0</v>
       </c>
       <c r="M15" s="2" t="n">
-        <v>11288.17</v>
+        <v>12396.76</v>
       </c>
       <c r="N15" s="2" t="n">
         <v>0</v>
@@ -1588,7 +1588,7 @@
         <v>3234.7</v>
       </c>
       <c r="M18" s="2" t="n">
-        <v>74.73</v>
+        <v>1242.3</v>
       </c>
       <c r="N18" s="2" t="n">
         <v>0</v>
@@ -1858,7 +1858,7 @@
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>0</v>
+        <v>312.26</v>
       </c>
       <c r="D23" s="2" t="n">
         <v>1079.4</v>
@@ -1888,7 +1888,7 @@
         <v>0</v>
       </c>
       <c r="M23" s="2" t="n">
-        <v>1253.45</v>
+        <v>2936.28</v>
       </c>
       <c r="N23" s="2" t="n">
         <v>0</v>
@@ -2185,10 +2185,10 @@
         <v>0</v>
       </c>
       <c r="L28" s="2" t="n">
-        <v>0</v>
+        <v>391.91</v>
       </c>
       <c r="M28" s="2" t="n">
-        <v>2808.93</v>
+        <v>3470.95</v>
       </c>
       <c r="N28" s="2" t="n">
         <v>0</v>
@@ -2482,7 +2482,7 @@
         <v>0</v>
       </c>
       <c r="K33" s="2" t="n">
-        <v>0</v>
+        <v>36.2</v>
       </c>
       <c r="L33" s="2" t="n">
         <v>0</v>
@@ -3208,7 +3208,7 @@
         <v>0</v>
       </c>
       <c r="M45" s="2" t="n">
-        <v>0</v>
+        <v>90.98</v>
       </c>
       <c r="N45" s="2" t="n">
         <v>0</v>
@@ -3217,7 +3217,7 @@
         <v>0</v>
       </c>
       <c r="P45" s="2" t="n">
-        <v>0</v>
+        <v>112.96</v>
       </c>
       <c r="Q45" s="2" t="n">
         <v>0</v>
@@ -3769,72 +3769,72 @@
     <row r="55">
       <c r="C55" s="4" t="inlineStr">
         <is>
+          <t>3 de 53</t>
+        </is>
+      </c>
+      <c r="D55" s="4" t="inlineStr">
+        <is>
+          <t>5 de 53</t>
+        </is>
+      </c>
+      <c r="E55" s="4" t="inlineStr">
+        <is>
           <t>2 de 53</t>
         </is>
       </c>
-      <c r="D55" s="4" t="inlineStr">
+      <c r="F55" s="4" t="inlineStr">
+        <is>
+          <t>0 de 53</t>
+        </is>
+      </c>
+      <c r="G55" s="4" t="inlineStr">
+        <is>
+          <t>0 de 53</t>
+        </is>
+      </c>
+      <c r="H55" s="4" t="inlineStr">
+        <is>
+          <t>0 de 53</t>
+        </is>
+      </c>
+      <c r="I55" s="4" t="inlineStr">
+        <is>
+          <t>1 de 53</t>
+        </is>
+      </c>
+      <c r="J55" s="4" t="inlineStr">
+        <is>
+          <t>0 de 53</t>
+        </is>
+      </c>
+      <c r="K55" s="4" t="inlineStr">
+        <is>
+          <t>1 de 53</t>
+        </is>
+      </c>
+      <c r="L55" s="4" t="inlineStr">
         <is>
           <t>5 de 53</t>
         </is>
       </c>
-      <c r="E55" s="4" t="inlineStr">
-        <is>
-          <t>2 de 53</t>
-        </is>
-      </c>
-      <c r="F55" s="4" t="inlineStr">
+      <c r="M55" s="4" t="inlineStr">
+        <is>
+          <t>19 de 53</t>
+        </is>
+      </c>
+      <c r="N55" s="4" t="inlineStr">
         <is>
           <t>0 de 53</t>
         </is>
       </c>
-      <c r="G55" s="4" t="inlineStr">
+      <c r="O55" s="4" t="inlineStr">
         <is>
           <t>0 de 53</t>
         </is>
       </c>
-      <c r="H55" s="4" t="inlineStr">
-        <is>
-          <t>0 de 53</t>
-        </is>
-      </c>
-      <c r="I55" s="4" t="inlineStr">
+      <c r="P55" s="4" t="inlineStr">
         <is>
           <t>1 de 53</t>
-        </is>
-      </c>
-      <c r="J55" s="4" t="inlineStr">
-        <is>
-          <t>0 de 53</t>
-        </is>
-      </c>
-      <c r="K55" s="4" t="inlineStr">
-        <is>
-          <t>0 de 53</t>
-        </is>
-      </c>
-      <c r="L55" s="4" t="inlineStr">
-        <is>
-          <t>4 de 53</t>
-        </is>
-      </c>
-      <c r="M55" s="4" t="inlineStr">
-        <is>
-          <t>17 de 53</t>
-        </is>
-      </c>
-      <c r="N55" s="4" t="inlineStr">
-        <is>
-          <t>0 de 53</t>
-        </is>
-      </c>
-      <c r="O55" s="4" t="inlineStr">
-        <is>
-          <t>0 de 53</t>
-        </is>
-      </c>
-      <c r="P55" s="4" t="inlineStr">
-        <is>
-          <t>0 de 53</t>
         </is>
       </c>
       <c r="Q55" s="4" t="inlineStr">
@@ -3956,7 +3956,7 @@
         <v>3789.54</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>3173.05</v>
+        <v>4589.02</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>15000</v>
@@ -3983,7 +3983,7 @@
         <v>1581.4</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>3018.04</v>
+        <v>5848.5</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>10000</v>
@@ -4253,7 +4253,7 @@
         <v>2910.78</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>11288.17</v>
+        <v>12396.76</v>
       </c>
       <c r="G14" s="2" t="n">
         <v>6000</v>
@@ -4334,7 +4334,7 @@
         <v>16.74</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>3309.43</v>
+        <v>4477</v>
       </c>
       <c r="G17" s="2" t="n">
         <v>1000</v>
@@ -4469,7 +4469,7 @@
         <v>0</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>2332.85</v>
+        <v>4327.94</v>
       </c>
       <c r="G22" s="2" t="n">
         <v>15000</v>
@@ -4631,7 +4631,7 @@
         <v>2107.43</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>2808.93</v>
+        <v>3862.86</v>
       </c>
       <c r="G28" s="2" t="n">
         <v>6000</v>
@@ -4793,7 +4793,7 @@
         <v>306.5</v>
       </c>
       <c r="F34" s="2" t="n">
-        <v>0</v>
+        <v>36.2</v>
       </c>
       <c r="G34" s="2" t="n">
         <v>0</v>
@@ -5144,7 +5144,7 @@
         <v>90.98</v>
       </c>
       <c r="F47" s="2" t="n">
-        <v>0</v>
+        <v>203.94</v>
       </c>
       <c r="G47" s="2" t="n">
         <v>1500</v>
@@ -5458,7 +5458,7 @@
         <v>23521.41</v>
       </c>
       <c r="F59" s="5" t="n">
-        <v>55880.43</v>
+        <v>65692.18000000001</v>
       </c>
       <c r="G59" s="5" t="n">
         <v>114450</v>
@@ -5483,7 +5483,7 @@
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5533,13 +5533,13 @@
         <v>436</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>505.56</v>
+        <v>817.8200000000001</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>-69.56</v>
+        <v>-381.8200000000001</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>1.15954128440367</v>
+        <v>1.875733944954129</v>
       </c>
     </row>
     <row r="3">
@@ -5653,13 +5653,13 @@
         <v>250</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>0</v>
+        <v>112.96</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>250</v>
+        <v>137.04</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>0</v>
+        <v>0.45184</v>
       </c>
     </row>
     <row r="8">
@@ -5701,13 +5701,13 @@
         <v>728</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>-50.76</v>
+        <v>-14.56</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>778.76</v>
+        <v>742.5599999999999</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>-0.06972527472527472</v>
+        <v>-0.02</v>
       </c>
     </row>
     <row r="10">
@@ -5749,13 +5749,13 @@
         <v>7700</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>7515.12</v>
+        <v>7907.03</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>184.8800000000001</v>
+        <v>-207.0299999999997</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>0.9759896103896104</v>
+        <v>1.026887012987013</v>
       </c>
     </row>
     <row r="12">
@@ -5773,13 +5773,13 @@
         <v>55052</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>30515.65</v>
+        <v>39474.07</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>24536.35</v>
+        <v>15577.93</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0.5543059289399114</v>
+        <v>0.7170324420547846</v>
       </c>
     </row>
     <row r="13">
@@ -5816,13 +5816,13 @@
         <v>72543.32000000001</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>55545.81</v>
+        <v>65357.56</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>16997.51</v>
+        <v>7185.760000000002</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.7656915895219574</v>
+        <v>0.9009452558829675</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-07-30 08:30:18
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -748,7 +748,7 @@
         <v>1748.09</v>
       </c>
       <c r="M4" s="2" t="n">
-        <v>1448.77</v>
+        <v>2132.32</v>
       </c>
       <c r="N4" s="2" t="n">
         <v>0</v>
@@ -781,7 +781,7 @@
         <v>312.26</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>324.98</v>
+        <v>1348.91</v>
       </c>
       <c r="E5" s="2" t="n">
         <v>0</v>
@@ -808,7 +808,7 @@
         <v>2380.8</v>
       </c>
       <c r="M5" s="2" t="n">
-        <v>2830.46</v>
+        <v>6779.14</v>
       </c>
       <c r="N5" s="2" t="n">
         <v>0</v>
@@ -1588,7 +1588,7 @@
         <v>3234.7</v>
       </c>
       <c r="M18" s="2" t="n">
-        <v>1242.3</v>
+        <v>2409.87</v>
       </c>
       <c r="N18" s="2" t="n">
         <v>0</v>
@@ -1858,7 +1858,7 @@
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>312.26</v>
+        <v>624.52</v>
       </c>
       <c r="D23" s="2" t="n">
         <v>1079.4</v>
@@ -3148,7 +3148,7 @@
         <v>151.53</v>
       </c>
       <c r="M44" s="2" t="n">
-        <v>7006.72</v>
+        <v>8174.29</v>
       </c>
       <c r="N44" s="2" t="n">
         <v>0</v>
@@ -3956,7 +3956,7 @@
         <v>3789.54</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>4589.02</v>
+        <v>5272.57</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>15000</v>
@@ -3983,7 +3983,7 @@
         <v>1581.4</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>5848.5</v>
+        <v>10821.11</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>10000</v>
@@ -4334,7 +4334,7 @@
         <v>16.74</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>4477</v>
+        <v>5644.57</v>
       </c>
       <c r="G17" s="2" t="n">
         <v>1000</v>
@@ -4469,7 +4469,7 @@
         <v>0</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>4327.94</v>
+        <v>4640.2</v>
       </c>
       <c r="G22" s="2" t="n">
         <v>15000</v>
@@ -5117,7 +5117,7 @@
         <v>0</v>
       </c>
       <c r="F46" s="2" t="n">
-        <v>7158.25</v>
+        <v>8325.82</v>
       </c>
       <c r="G46" s="2" t="n">
         <v>1500</v>
@@ -5458,7 +5458,7 @@
         <v>23521.41</v>
       </c>
       <c r="F59" s="5" t="n">
-        <v>65692.18000000001</v>
+        <v>73995.74000000001</v>
       </c>
       <c r="G59" s="5" t="n">
         <v>114450</v>
@@ -5533,13 +5533,13 @@
         <v>436</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>817.8200000000001</v>
+        <v>1130.08</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>-381.8200000000001</v>
+        <v>-694.0799999999999</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>1.875733944954129</v>
+        <v>2.591926605504587</v>
       </c>
     </row>
     <row r="3">
@@ -5557,13 +5557,13 @@
         <v>6600</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>16959.21</v>
+        <v>17983.14</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>-10359.21</v>
+        <v>-11383.14</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>2.569577272727273</v>
+        <v>2.724718181818182</v>
       </c>
     </row>
     <row r="4">
@@ -5773,13 +5773,13 @@
         <v>55052</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>39474.07</v>
+        <v>46441.44</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>15577.93</v>
+        <v>8610.559999999998</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0.7170324420547846</v>
+        <v>0.8435922400639396</v>
       </c>
     </row>
     <row r="13">
@@ -5816,13 +5816,13 @@
         <v>72543.32000000001</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>65357.56</v>
+        <v>73661.12</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>7185.760000000002</v>
+        <v>-1117.800000000001</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.9009452558829675</v>
+        <v>1.015408724056191</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-08-05 14:30:15
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -1876,7 +1876,7 @@
         <v>0</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>0</v>
+        <v>104.08</v>
       </c>
       <c r="J23" s="2" t="n">
         <v>0</v>
@@ -3799,7 +3799,7 @@
       </c>
       <c r="I55" s="4" t="inlineStr">
         <is>
-          <t>0 de 53</t>
+          <t>1 de 53</t>
         </is>
       </c>
       <c r="J55" s="4" t="inlineStr">
@@ -4469,7 +4469,7 @@
         <v>4640.2</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>1485.99</v>
+        <v>1590.07</v>
       </c>
       <c r="G22" s="2" t="n">
         <v>15000</v>
@@ -5458,7 +5458,7 @@
         <v>85761.95999999999</v>
       </c>
       <c r="F59" s="5" t="n">
-        <v>4251.86</v>
+        <v>4355.94</v>
       </c>
       <c r="G59" s="5" t="n">
         <v>114450</v>

</xml_diff>

<commit_message>
Actualización automática 2026-08-07 09:30:16
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -808,7 +808,7 @@
         <v>841.27</v>
       </c>
       <c r="M5" s="2" t="n">
-        <v>0</v>
+        <v>-35.38</v>
       </c>
       <c r="N5" s="2" t="n">
         <v>0</v>
@@ -3148,7 +3148,7 @@
         <v>0</v>
       </c>
       <c r="M44" s="2" t="n">
-        <v>0</v>
+        <v>-17.69</v>
       </c>
       <c r="N44" s="2" t="n">
         <v>0</v>
@@ -3983,7 +3983,7 @@
         <v>17314.42</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>841.27</v>
+        <v>805.89</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>10000</v>
@@ -5117,7 +5117,7 @@
         <v>8325.82</v>
       </c>
       <c r="F46" s="2" t="n">
-        <v>0</v>
+        <v>-17.69</v>
       </c>
       <c r="G46" s="2" t="n">
         <v>1500</v>
@@ -5458,7 +5458,7 @@
         <v>85761.95999999999</v>
       </c>
       <c r="F59" s="5" t="n">
-        <v>4550.53</v>
+        <v>4497.46</v>
       </c>
       <c r="G59" s="5" t="n">
         <v>114450</v>

</xml_diff>

<commit_message>
Actualización automática 2026-08-11 17:30:23
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -748,7 +748,7 @@
         <v>0</v>
       </c>
       <c r="M4" s="2" t="n">
-        <v>19.46</v>
+        <v>1350.84</v>
       </c>
       <c r="N4" s="2" t="n">
         <v>0</v>
@@ -781,7 +781,7 @@
         <v>0</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>0</v>
+        <v>1153.68</v>
       </c>
       <c r="E5" s="2" t="n">
         <v>0</v>
@@ -1588,7 +1588,7 @@
         <v>0</v>
       </c>
       <c r="M18" s="2" t="n">
-        <v>99.48</v>
+        <v>588.4299999999999</v>
       </c>
       <c r="N18" s="2" t="n">
         <v>0</v>
@@ -1888,7 +1888,7 @@
         <v>0</v>
       </c>
       <c r="M23" s="2" t="n">
-        <v>1485.99</v>
+        <v>2903.5</v>
       </c>
       <c r="N23" s="2" t="n">
         <v>0</v>
@@ -2182,13 +2182,13 @@
         <v>0</v>
       </c>
       <c r="K28" s="2" t="n">
-        <v>0</v>
+        <v>135</v>
       </c>
       <c r="L28" s="2" t="n">
         <v>638.09</v>
       </c>
       <c r="M28" s="2" t="n">
-        <v>0</v>
+        <v>103.36</v>
       </c>
       <c r="N28" s="2" t="n">
         <v>0</v>
@@ -2788,7 +2788,7 @@
         <v>0</v>
       </c>
       <c r="M38" s="2" t="n">
-        <v>6190.38</v>
+        <v>8044.92</v>
       </c>
       <c r="N38" s="2" t="n">
         <v>0</v>
@@ -3774,44 +3774,44 @@
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
+          <t>1 de 53</t>
+        </is>
+      </c>
+      <c r="E55" s="4" t="inlineStr">
+        <is>
           <t>0 de 53</t>
         </is>
       </c>
-      <c r="E55" s="4" t="inlineStr">
+      <c r="F55" s="4" t="inlineStr">
         <is>
           <t>0 de 53</t>
         </is>
       </c>
-      <c r="F55" s="4" t="inlineStr">
+      <c r="G55" s="4" t="inlineStr">
         <is>
           <t>0 de 53</t>
         </is>
       </c>
-      <c r="G55" s="4" t="inlineStr">
+      <c r="H55" s="4" t="inlineStr">
         <is>
           <t>0 de 53</t>
         </is>
       </c>
-      <c r="H55" s="4" t="inlineStr">
+      <c r="I55" s="4" t="inlineStr">
+        <is>
+          <t>1 de 53</t>
+        </is>
+      </c>
+      <c r="J55" s="4" t="inlineStr">
         <is>
           <t>0 de 53</t>
         </is>
       </c>
-      <c r="I55" s="4" t="inlineStr">
+      <c r="K55" s="4" t="inlineStr">
         <is>
           <t>1 de 53</t>
         </is>
       </c>
-      <c r="J55" s="4" t="inlineStr">
-        <is>
-          <t>0 de 53</t>
-        </is>
-      </c>
-      <c r="K55" s="4" t="inlineStr">
-        <is>
-          <t>0 de 53</t>
-        </is>
-      </c>
       <c r="L55" s="4" t="inlineStr">
         <is>
           <t>2 de 53</t>
@@ -3819,7 +3819,7 @@
       </c>
       <c r="M55" s="4" t="inlineStr">
         <is>
-          <t>5 de 53</t>
+          <t>6 de 53</t>
         </is>
       </c>
       <c r="N55" s="4" t="inlineStr">
@@ -3956,7 +3956,7 @@
         <v>8423.200000000001</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>19.46</v>
+        <v>1350.84</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>15000</v>
@@ -3983,7 +3983,7 @@
         <v>17314.42</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>805.89</v>
+        <v>1959.57</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>10000</v>
@@ -4334,7 +4334,7 @@
         <v>5644.57</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>99.48</v>
+        <v>588.4299999999999</v>
       </c>
       <c r="G17" s="2" t="n">
         <v>1000</v>
@@ -4469,7 +4469,7 @@
         <v>4640.2</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>1590.07</v>
+        <v>3007.58</v>
       </c>
       <c r="G22" s="2" t="n">
         <v>15000</v>
@@ -4631,7 +4631,7 @@
         <v>3862.86</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>638.09</v>
+        <v>876.45</v>
       </c>
       <c r="G28" s="2" t="n">
         <v>6000</v>
@@ -4955,7 +4955,7 @@
         <v>104.73</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>6190.38</v>
+        <v>8044.92</v>
       </c>
       <c r="G40" s="2" t="n">
         <v>3500</v>
@@ -5458,7 +5458,7 @@
         <v>85761.95999999999</v>
       </c>
       <c r="F59" s="5" t="n">
-        <v>10687.84</v>
+        <v>17172.26</v>
       </c>
       <c r="G59" s="5" t="n">
         <v>114450</v>
@@ -5481,7 +5481,7 @@
     <col width="32" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
@@ -5557,13 +5557,13 @@
         <v>6600</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>0</v>
+        <v>1153.68</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>6600</v>
+        <v>5446.32</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>0</v>
+        <v>0.1748</v>
       </c>
     </row>
     <row r="4">
@@ -5725,13 +5725,13 @@
         <v>728</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0</v>
+        <v>135</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>728</v>
+        <v>593</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>0</v>
+        <v>0.1854395604395604</v>
       </c>
     </row>
     <row r="11">
@@ -5797,13 +5797,13 @@
         <v>57552</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>9104.4</v>
+        <v>14300.14</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>48447.6</v>
+        <v>43251.86</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.1581943286071726</v>
+        <v>0.2484733805949402</v>
       </c>
     </row>
     <row r="14">
@@ -5840,13 +5840,13 @@
         <v>79852</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>10687.84</v>
+        <v>17172.26</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>69164.16</v>
+        <v>62679.74</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.1338456143866152</v>
+        <v>0.215051094524871</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-08-13 15:30:20
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -1021,7 +1021,7 @@
         <v>0</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0</v>
+        <v>1089.89</v>
       </c>
       <c r="E9" s="2" t="n">
         <v>0</v>
@@ -1201,7 +1201,7 @@
         <v>0</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>0</v>
+        <v>487.47</v>
       </c>
       <c r="E12" s="2" t="n">
         <v>0</v>
@@ -2308,7 +2308,7 @@
         <v>0</v>
       </c>
       <c r="M30" s="2" t="n">
-        <v>0</v>
+        <v>827.54</v>
       </c>
       <c r="N30" s="2" t="n">
         <v>0</v>
@@ -2341,7 +2341,7 @@
         <v>0</v>
       </c>
       <c r="D31" s="2" t="n">
-        <v>0</v>
+        <v>1079.91</v>
       </c>
       <c r="E31" s="2" t="n">
         <v>0</v>
@@ -2368,7 +2368,7 @@
         <v>0</v>
       </c>
       <c r="M31" s="2" t="n">
-        <v>0</v>
+        <v>1296.47</v>
       </c>
       <c r="N31" s="2" t="n">
         <v>0</v>
@@ -3541,7 +3541,7 @@
         <v>0</v>
       </c>
       <c r="D51" s="2" t="n">
-        <v>0</v>
+        <v>406.22</v>
       </c>
       <c r="E51" s="2" t="n">
         <v>0</v>
@@ -3774,44 +3774,44 @@
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
+          <t>5 de 53</t>
+        </is>
+      </c>
+      <c r="E55" s="4" t="inlineStr">
+        <is>
+          <t>0 de 53</t>
+        </is>
+      </c>
+      <c r="F55" s="4" t="inlineStr">
+        <is>
+          <t>0 de 53</t>
+        </is>
+      </c>
+      <c r="G55" s="4" t="inlineStr">
+        <is>
+          <t>0 de 53</t>
+        </is>
+      </c>
+      <c r="H55" s="4" t="inlineStr">
+        <is>
+          <t>0 de 53</t>
+        </is>
+      </c>
+      <c r="I55" s="4" t="inlineStr">
+        <is>
           <t>1 de 53</t>
         </is>
       </c>
-      <c r="E55" s="4" t="inlineStr">
+      <c r="J55" s="4" t="inlineStr">
         <is>
           <t>0 de 53</t>
         </is>
       </c>
-      <c r="F55" s="4" t="inlineStr">
-        <is>
-          <t>0 de 53</t>
-        </is>
-      </c>
-      <c r="G55" s="4" t="inlineStr">
-        <is>
-          <t>0 de 53</t>
-        </is>
-      </c>
-      <c r="H55" s="4" t="inlineStr">
-        <is>
-          <t>0 de 53</t>
-        </is>
-      </c>
-      <c r="I55" s="4" t="inlineStr">
+      <c r="K55" s="4" t="inlineStr">
         <is>
           <t>1 de 53</t>
         </is>
       </c>
-      <c r="J55" s="4" t="inlineStr">
-        <is>
-          <t>0 de 53</t>
-        </is>
-      </c>
-      <c r="K55" s="4" t="inlineStr">
-        <is>
-          <t>1 de 53</t>
-        </is>
-      </c>
       <c r="L55" s="4" t="inlineStr">
         <is>
           <t>2 de 53</t>
@@ -3819,7 +3819,7 @@
       </c>
       <c r="M55" s="4" t="inlineStr">
         <is>
-          <t>6 de 53</t>
+          <t>8 de 53</t>
         </is>
       </c>
       <c r="N55" s="4" t="inlineStr">
@@ -4091,7 +4091,7 @@
         <v>0</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>0</v>
+        <v>1089.89</v>
       </c>
       <c r="G8" s="2" t="n">
         <v>1500</v>
@@ -4172,7 +4172,7 @@
         <v>0</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>0</v>
+        <v>487.47</v>
       </c>
       <c r="G11" s="2" t="n">
         <v>3000</v>
@@ -4685,7 +4685,7 @@
         <v>179.92</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>0</v>
+        <v>827.54</v>
       </c>
       <c r="G30" s="2" t="n">
         <v>1500</v>
@@ -4712,7 +4712,7 @@
         <v>0</v>
       </c>
       <c r="F31" s="2" t="n">
-        <v>0</v>
+        <v>2376.38</v>
       </c>
       <c r="G31" s="2" t="n">
         <v>3000</v>
@@ -5306,7 +5306,7 @@
         <v>0</v>
       </c>
       <c r="F53" s="2" t="n">
-        <v>0</v>
+        <v>406.22</v>
       </c>
       <c r="G53" s="2" t="n">
         <v>1650</v>
@@ -5458,7 +5458,7 @@
         <v>85761.95999999999</v>
       </c>
       <c r="F59" s="5" t="n">
-        <v>17172.26</v>
+        <v>22359.76</v>
       </c>
       <c r="G59" s="5" t="n">
         <v>114450</v>
@@ -5557,13 +5557,13 @@
         <v>6600</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>1153.68</v>
+        <v>4217.17</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>5446.32</v>
+        <v>2382.83</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>0.1748</v>
+        <v>0.6389651515151515</v>
       </c>
     </row>
     <row r="4">
@@ -5797,13 +5797,13 @@
         <v>57552</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>14300.14</v>
+        <v>16424.15</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>43251.86</v>
+        <v>41127.85</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.2484733805949402</v>
+        <v>0.285379309146511</v>
       </c>
     </row>
     <row r="14">
@@ -5840,13 +5840,13 @@
         <v>79852</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>17172.26</v>
+        <v>22359.76</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>62679.74</v>
+        <v>57492.24</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.215051094524871</v>
+        <v>0.2800150278014327</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-08-17 17:30:18
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -718,7 +718,7 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0</v>
+        <v>118.96</v>
       </c>
       <c r="D4" s="2" t="n">
         <v>0</v>
@@ -805,7 +805,7 @@
         <v>0</v>
       </c>
       <c r="L5" s="2" t="n">
-        <v>841.27</v>
+        <v>1755.73</v>
       </c>
       <c r="M5" s="2" t="n">
         <v>-35.38</v>
@@ -1858,7 +1858,7 @@
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>0</v>
+        <v>208.17</v>
       </c>
       <c r="D23" s="2" t="n">
         <v>0</v>
@@ -2185,7 +2185,7 @@
         <v>135</v>
       </c>
       <c r="L28" s="2" t="n">
-        <v>638.09</v>
+        <v>1595.18</v>
       </c>
       <c r="M28" s="2" t="n">
         <v>103.36</v>
@@ -2308,7 +2308,7 @@
         <v>0</v>
       </c>
       <c r="M30" s="2" t="n">
-        <v>827.54</v>
+        <v>1030.52</v>
       </c>
       <c r="N30" s="2" t="n">
         <v>0</v>
@@ -2518,7 +2518,7 @@
         </is>
       </c>
       <c r="C34" s="2" t="n">
-        <v>0</v>
+        <v>312.26</v>
       </c>
       <c r="D34" s="2" t="n">
         <v>0</v>
@@ -2548,7 +2548,7 @@
         <v>0</v>
       </c>
       <c r="M34" s="2" t="n">
-        <v>0</v>
+        <v>6464.07</v>
       </c>
       <c r="N34" s="2" t="n">
         <v>0</v>
@@ -2905,7 +2905,7 @@
         <v>0</v>
       </c>
       <c r="L40" s="2" t="n">
-        <v>0</v>
+        <v>645.35</v>
       </c>
       <c r="M40" s="2" t="n">
         <v>0</v>
@@ -3769,57 +3769,57 @@
     <row r="55">
       <c r="C55" s="4" t="inlineStr">
         <is>
+          <t>3 de 53</t>
+        </is>
+      </c>
+      <c r="D55" s="4" t="inlineStr">
+        <is>
+          <t>5 de 53</t>
+        </is>
+      </c>
+      <c r="E55" s="4" t="inlineStr">
+        <is>
           <t>0 de 53</t>
         </is>
       </c>
-      <c r="D55" s="4" t="inlineStr">
-        <is>
-          <t>5 de 53</t>
-        </is>
-      </c>
-      <c r="E55" s="4" t="inlineStr">
+      <c r="F55" s="4" t="inlineStr">
         <is>
           <t>0 de 53</t>
         </is>
       </c>
-      <c r="F55" s="4" t="inlineStr">
+      <c r="G55" s="4" t="inlineStr">
         <is>
           <t>0 de 53</t>
         </is>
       </c>
-      <c r="G55" s="4" t="inlineStr">
+      <c r="H55" s="4" t="inlineStr">
         <is>
           <t>0 de 53</t>
         </is>
       </c>
-      <c r="H55" s="4" t="inlineStr">
+      <c r="I55" s="4" t="inlineStr">
+        <is>
+          <t>1 de 53</t>
+        </is>
+      </c>
+      <c r="J55" s="4" t="inlineStr">
         <is>
           <t>0 de 53</t>
         </is>
       </c>
-      <c r="I55" s="4" t="inlineStr">
+      <c r="K55" s="4" t="inlineStr">
         <is>
           <t>1 de 53</t>
         </is>
       </c>
-      <c r="J55" s="4" t="inlineStr">
-        <is>
-          <t>0 de 53</t>
-        </is>
-      </c>
-      <c r="K55" s="4" t="inlineStr">
-        <is>
-          <t>1 de 53</t>
-        </is>
-      </c>
       <c r="L55" s="4" t="inlineStr">
         <is>
-          <t>2 de 53</t>
+          <t>3 de 53</t>
         </is>
       </c>
       <c r="M55" s="4" t="inlineStr">
         <is>
-          <t>8 de 53</t>
+          <t>9 de 53</t>
         </is>
       </c>
       <c r="N55" s="4" t="inlineStr">
@@ -3956,7 +3956,7 @@
         <v>8423.200000000001</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>1350.84</v>
+        <v>1469.8</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>15000</v>
@@ -3983,7 +3983,7 @@
         <v>17314.42</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>1959.57</v>
+        <v>2874.03</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>10000</v>
@@ -4469,7 +4469,7 @@
         <v>4640.2</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>3007.58</v>
+        <v>3215.75</v>
       </c>
       <c r="G22" s="2" t="n">
         <v>15000</v>
@@ -4631,7 +4631,7 @@
         <v>3862.86</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>876.45</v>
+        <v>1833.54</v>
       </c>
       <c r="G28" s="2" t="n">
         <v>6000</v>
@@ -4685,7 +4685,7 @@
         <v>179.92</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>827.54</v>
+        <v>1030.52</v>
       </c>
       <c r="G30" s="2" t="n">
         <v>1500</v>
@@ -4820,7 +4820,7 @@
         <v>12800.81</v>
       </c>
       <c r="F35" s="2" t="n">
-        <v>0</v>
+        <v>6776.33</v>
       </c>
       <c r="G35" s="2" t="n">
         <v>10000</v>
@@ -5009,7 +5009,7 @@
         <v>1388.57</v>
       </c>
       <c r="F42" s="2" t="n">
-        <v>0</v>
+        <v>645.35</v>
       </c>
       <c r="G42" s="2" t="n">
         <v>2000</v>
@@ -5458,7 +5458,7 @@
         <v>85761.95999999999</v>
       </c>
       <c r="F59" s="5" t="n">
-        <v>22359.76</v>
+        <v>32183.1</v>
       </c>
       <c r="G59" s="5" t="n">
         <v>114450</v>
@@ -5481,7 +5481,7 @@
     <col width="32" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
@@ -5533,13 +5533,13 @@
         <v>436</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0</v>
+        <v>639.39</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>436</v>
+        <v>-203.39</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>0</v>
+        <v>1.466490825688073</v>
       </c>
     </row>
     <row r="3">
@@ -5773,13 +5773,13 @@
         <v>9700</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>1479.36</v>
+        <v>3996.26</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>8220.639999999999</v>
+        <v>5703.74</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0.1525113402061856</v>
+        <v>0.4119855670103093</v>
       </c>
     </row>
     <row r="13">
@@ -5797,13 +5797,13 @@
         <v>57552</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>16424.15</v>
+        <v>23091.2</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>41127.85</v>
+        <v>34460.8</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.285379309146511</v>
+        <v>0.4012232415902141</v>
       </c>
     </row>
     <row r="14">
@@ -5840,13 +5840,13 @@
         <v>79852</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>22359.76</v>
+        <v>32183.1</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>57492.24</v>
+        <v>47668.9</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.2800150278014327</v>
+        <v>0.4030343635726094</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-08-18 16:30:19
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -2128,7 +2128,7 @@
         <v>0</v>
       </c>
       <c r="M27" s="2" t="n">
-        <v>1362.16</v>
+        <v>1415.23</v>
       </c>
       <c r="N27" s="2" t="n">
         <v>0</v>
@@ -4604,7 +4604,7 @@
         <v>-65.18000000000001</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>1362.16</v>
+        <v>1415.23</v>
       </c>
       <c r="G27" s="2" t="n">
         <v>1500</v>
@@ -5458,7 +5458,7 @@
         <v>85761.95999999999</v>
       </c>
       <c r="F59" s="5" t="n">
-        <v>32183.1</v>
+        <v>32236.17</v>
       </c>
       <c r="G59" s="5" t="n">
         <v>114450</v>
@@ -5481,7 +5481,7 @@
     <col width="32" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
@@ -5797,13 +5797,13 @@
         <v>57552</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>23091.2</v>
+        <v>23144.27</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>34460.8</v>
+        <v>34407.73</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.4012232415902141</v>
+        <v>0.4021453641923826</v>
       </c>
     </row>
     <row r="14">
@@ -5840,13 +5840,13 @@
         <v>79852</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>32183.1</v>
+        <v>32236.17</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>47668.9</v>
+        <v>47615.83</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.4030343635726094</v>
+        <v>0.4036989680909683</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-08-19 14:30:17
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -1528,7 +1528,7 @@
         <v>0</v>
       </c>
       <c r="M17" s="2" t="n">
-        <v>0</v>
+        <v>11.16</v>
       </c>
       <c r="N17" s="2" t="n">
         <v>0</v>
@@ -2788,7 +2788,7 @@
         <v>0</v>
       </c>
       <c r="M38" s="2" t="n">
-        <v>8044.92</v>
+        <v>8056.08</v>
       </c>
       <c r="N38" s="2" t="n">
         <v>0</v>
@@ -3819,7 +3819,7 @@
       </c>
       <c r="M55" s="4" t="inlineStr">
         <is>
-          <t>9 de 53</t>
+          <t>10 de 53</t>
         </is>
       </c>
       <c r="N55" s="4" t="inlineStr">
@@ -4307,7 +4307,7 @@
         <v>1355.61</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>0</v>
+        <v>11.16</v>
       </c>
       <c r="G16" s="2" t="n">
         <v>3000</v>
@@ -4955,7 +4955,7 @@
         <v>104.73</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>8044.92</v>
+        <v>8056.08</v>
       </c>
       <c r="G40" s="2" t="n">
         <v>3500</v>
@@ -5458,7 +5458,7 @@
         <v>85761.95999999999</v>
       </c>
       <c r="F59" s="5" t="n">
-        <v>32236.17</v>
+        <v>32258.49</v>
       </c>
       <c r="G59" s="5" t="n">
         <v>114450</v>
@@ -5797,13 +5797,13 @@
         <v>57552</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>23144.27</v>
+        <v>23166.59</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>34407.73</v>
+        <v>34385.41</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.4021453641923826</v>
+        <v>0.4025331873783708</v>
       </c>
     </row>
     <row r="14">
@@ -5840,13 +5840,13 @@
         <v>79852</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>32236.17</v>
+        <v>32258.49</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>47615.83</v>
+        <v>47593.51</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.4036989680909683</v>
+        <v>0.4039784851976156</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-08-19 15:30:18
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -748,7 +748,7 @@
         <v>0</v>
       </c>
       <c r="M4" s="2" t="n">
-        <v>1350.84</v>
+        <v>1362</v>
       </c>
       <c r="N4" s="2" t="n">
         <v>0</v>
@@ -808,7 +808,7 @@
         <v>1755.73</v>
       </c>
       <c r="M5" s="2" t="n">
-        <v>-35.38</v>
+        <v>11.8</v>
       </c>
       <c r="N5" s="2" t="n">
         <v>0</v>
@@ -1408,7 +1408,7 @@
         <v>0</v>
       </c>
       <c r="M15" s="2" t="n">
-        <v>0</v>
+        <v>11.16</v>
       </c>
       <c r="N15" s="2" t="n">
         <v>0</v>
@@ -1588,7 +1588,7 @@
         <v>0</v>
       </c>
       <c r="M18" s="2" t="n">
-        <v>588.4299999999999</v>
+        <v>599.59</v>
       </c>
       <c r="N18" s="2" t="n">
         <v>0</v>
@@ -2182,7 +2182,7 @@
         <v>0</v>
       </c>
       <c r="K28" s="2" t="n">
-        <v>135</v>
+        <v>216.22</v>
       </c>
       <c r="L28" s="2" t="n">
         <v>1595.18</v>
@@ -2368,7 +2368,7 @@
         <v>0</v>
       </c>
       <c r="M31" s="2" t="n">
-        <v>1296.47</v>
+        <v>1307.63</v>
       </c>
       <c r="N31" s="2" t="n">
         <v>0</v>
@@ -3148,7 +3148,7 @@
         <v>0</v>
       </c>
       <c r="M44" s="2" t="n">
-        <v>-17.69</v>
+        <v>-6.53</v>
       </c>
       <c r="N44" s="2" t="n">
         <v>0</v>
@@ -3819,7 +3819,7 @@
       </c>
       <c r="M55" s="4" t="inlineStr">
         <is>
-          <t>10 de 53</t>
+          <t>12 de 53</t>
         </is>
       </c>
       <c r="N55" s="4" t="inlineStr">
@@ -3956,7 +3956,7 @@
         <v>8423.200000000001</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>1469.8</v>
+        <v>1480.96</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>15000</v>
@@ -3983,7 +3983,7 @@
         <v>17314.42</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>2874.03</v>
+        <v>2921.21</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>10000</v>
@@ -4253,7 +4253,7 @@
         <v>13338.07</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>0</v>
+        <v>11.16</v>
       </c>
       <c r="G14" s="2" t="n">
         <v>6000</v>
@@ -4334,7 +4334,7 @@
         <v>5644.57</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>588.4299999999999</v>
+        <v>599.59</v>
       </c>
       <c r="G17" s="2" t="n">
         <v>1000</v>
@@ -4631,7 +4631,7 @@
         <v>3862.86</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>1833.54</v>
+        <v>1914.76</v>
       </c>
       <c r="G28" s="2" t="n">
         <v>6000</v>
@@ -4712,7 +4712,7 @@
         <v>0</v>
       </c>
       <c r="F31" s="2" t="n">
-        <v>2376.38</v>
+        <v>2387.54</v>
       </c>
       <c r="G31" s="2" t="n">
         <v>3000</v>
@@ -5117,7 +5117,7 @@
         <v>8325.82</v>
       </c>
       <c r="F46" s="2" t="n">
-        <v>-17.69</v>
+        <v>-6.53</v>
       </c>
       <c r="G46" s="2" t="n">
         <v>1500</v>
@@ -5458,7 +5458,7 @@
         <v>85761.95999999999</v>
       </c>
       <c r="F59" s="5" t="n">
-        <v>32258.49</v>
+        <v>32442.69</v>
       </c>
       <c r="G59" s="5" t="n">
         <v>114450</v>
@@ -5725,13 +5725,13 @@
         <v>728</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>135</v>
+        <v>216.22</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>593</v>
+        <v>511.78</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>0.1854395604395604</v>
+        <v>0.2970054945054945</v>
       </c>
     </row>
     <row r="11">
@@ -5797,13 +5797,13 @@
         <v>57552</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>23166.59</v>
+        <v>23269.57</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>34385.41</v>
+        <v>34282.43</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.4025331873783708</v>
+        <v>0.4043225257158743</v>
       </c>
     </row>
     <row r="14">
@@ -5840,13 +5840,13 @@
         <v>79852</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>32258.49</v>
+        <v>32442.69</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>47593.51</v>
+        <v>47409.31</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.4039784851976156</v>
+        <v>0.4062852527175275</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-08-20 17:30:19
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -1222,7 +1222,7 @@
         <v>0</v>
       </c>
       <c r="K12" s="2" t="n">
-        <v>0</v>
+        <v>2294.4</v>
       </c>
       <c r="L12" s="2" t="n">
         <v>0</v>
@@ -1342,7 +1342,7 @@
         <v>0</v>
       </c>
       <c r="K14" s="2" t="n">
-        <v>0</v>
+        <v>676.8</v>
       </c>
       <c r="L14" s="2" t="n">
         <v>0</v>
@@ -3809,7 +3809,7 @@
       </c>
       <c r="K55" s="4" t="inlineStr">
         <is>
-          <t>1 de 53</t>
+          <t>3 de 53</t>
         </is>
       </c>
       <c r="L55" s="4" t="inlineStr">
@@ -4172,7 +4172,7 @@
         <v>0</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>487.47</v>
+        <v>2781.87</v>
       </c>
       <c r="G11" s="2" t="n">
         <v>3000</v>
@@ -4226,7 +4226,7 @@
         <v>0</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>0</v>
+        <v>676.8</v>
       </c>
       <c r="G13" s="2" t="n">
         <v>0</v>
@@ -5458,7 +5458,7 @@
         <v>85761.95999999999</v>
       </c>
       <c r="F59" s="5" t="n">
-        <v>32442.69</v>
+        <v>35413.89</v>
       </c>
       <c r="G59" s="5" t="n">
         <v>114450</v>
@@ -5725,13 +5725,13 @@
         <v>728</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>216.22</v>
+        <v>3187.42</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>511.78</v>
+        <v>-2459.42</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>0.2970054945054945</v>
+        <v>4.378324175824176</v>
       </c>
     </row>
     <row r="11">
@@ -5840,13 +5840,13 @@
         <v>79852</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>32442.69</v>
+        <v>35413.89</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>47409.31</v>
+        <v>44438.11</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.4062852527175275</v>
+        <v>0.4434940890647698</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-08-24 11:30:18
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -2788,7 +2788,7 @@
         <v>0</v>
       </c>
       <c r="M38" s="2" t="n">
-        <v>8056.08</v>
+        <v>8074.62</v>
       </c>
       <c r="N38" s="2" t="n">
         <v>0</v>
@@ -4955,7 +4955,7 @@
         <v>104.73</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>8056.08</v>
+        <v>8074.62</v>
       </c>
       <c r="G40" s="2" t="n">
         <v>3500</v>
@@ -5458,7 +5458,7 @@
         <v>85761.95999999999</v>
       </c>
       <c r="F59" s="5" t="n">
-        <v>35413.89</v>
+        <v>35432.43</v>
       </c>
       <c r="G59" s="5" t="n">
         <v>114450</v>
@@ -5797,13 +5797,13 @@
         <v>57552</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>23269.57</v>
+        <v>23288.11</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>34282.43</v>
+        <v>34263.89</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.4043225257158743</v>
+        <v>0.4046446691687517</v>
       </c>
     </row>
     <row r="14">
@@ -5840,13 +5840,13 @@
         <v>79852</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>35413.89</v>
+        <v>35432.43</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>44438.11</v>
+        <v>44419.57</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.4434940890647698</v>
+        <v>0.4437262685969043</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-08-24 16:30:18
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -1885,7 +1885,7 @@
         <v>0</v>
       </c>
       <c r="L23" s="2" t="n">
-        <v>0</v>
+        <v>322.88</v>
       </c>
       <c r="M23" s="2" t="n">
         <v>2903.5</v>
@@ -2368,7 +2368,7 @@
         <v>0</v>
       </c>
       <c r="M31" s="2" t="n">
-        <v>1307.63</v>
+        <v>2153.58</v>
       </c>
       <c r="N31" s="2" t="n">
         <v>0</v>
@@ -2521,7 +2521,7 @@
         <v>312.26</v>
       </c>
       <c r="D34" s="2" t="n">
-        <v>0</v>
+        <v>2062.32</v>
       </c>
       <c r="E34" s="2" t="n">
         <v>0</v>
@@ -2902,10 +2902,10 @@
         <v>0</v>
       </c>
       <c r="K40" s="2" t="n">
-        <v>0</v>
+        <v>2238.2</v>
       </c>
       <c r="L40" s="2" t="n">
-        <v>645.35</v>
+        <v>1322.56</v>
       </c>
       <c r="M40" s="2" t="n">
         <v>0</v>
@@ -3774,7 +3774,7 @@
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>5 de 53</t>
+          <t>6 de 53</t>
         </is>
       </c>
       <c r="E55" s="4" t="inlineStr">
@@ -3809,12 +3809,12 @@
       </c>
       <c r="K55" s="4" t="inlineStr">
         <is>
-          <t>3 de 53</t>
+          <t>4 de 53</t>
         </is>
       </c>
       <c r="L55" s="4" t="inlineStr">
         <is>
-          <t>3 de 53</t>
+          <t>4 de 53</t>
         </is>
       </c>
       <c r="M55" s="4" t="inlineStr">
@@ -4469,7 +4469,7 @@
         <v>4640.2</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>3215.75</v>
+        <v>3538.63</v>
       </c>
       <c r="G22" s="2" t="n">
         <v>15000</v>
@@ -4712,7 +4712,7 @@
         <v>0</v>
       </c>
       <c r="F31" s="2" t="n">
-        <v>2387.54</v>
+        <v>3233.49</v>
       </c>
       <c r="G31" s="2" t="n">
         <v>3000</v>
@@ -4820,7 +4820,7 @@
         <v>12800.81</v>
       </c>
       <c r="F35" s="2" t="n">
-        <v>6776.33</v>
+        <v>8838.65</v>
       </c>
       <c r="G35" s="2" t="n">
         <v>10000</v>
@@ -5009,7 +5009,7 @@
         <v>1388.57</v>
       </c>
       <c r="F42" s="2" t="n">
-        <v>645.35</v>
+        <v>3560.76</v>
       </c>
       <c r="G42" s="2" t="n">
         <v>2000</v>
@@ -5458,7 +5458,7 @@
         <v>85761.95999999999</v>
       </c>
       <c r="F59" s="5" t="n">
-        <v>35432.43</v>
+        <v>41578.99</v>
       </c>
       <c r="G59" s="5" t="n">
         <v>114450</v>
@@ -5482,7 +5482,7 @@
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -5557,13 +5557,13 @@
         <v>6600</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>4217.17</v>
+        <v>6279.49</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>2382.83</v>
+        <v>320.5100000000002</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>0.6389651515151515</v>
+        <v>0.9514378787878788</v>
       </c>
     </row>
     <row r="4">
@@ -5725,13 +5725,13 @@
         <v>728</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>3187.42</v>
+        <v>5425.62</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>-2459.42</v>
+        <v>-4697.62</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>4.378324175824176</v>
+        <v>7.452774725274725</v>
       </c>
     </row>
     <row r="11">
@@ -5773,13 +5773,13 @@
         <v>9700</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>3996.26</v>
+        <v>4996.35</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>5703.74</v>
+        <v>4703.65</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0.4119855670103093</v>
+        <v>0.5150876288659795</v>
       </c>
     </row>
     <row r="13">
@@ -5797,13 +5797,13 @@
         <v>57552</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>23288.11</v>
+        <v>24134.06</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>34263.89</v>
+        <v>33417.94</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.4046446691687517</v>
+        <v>0.4193435501807062</v>
       </c>
     </row>
     <row r="14">
@@ -5840,13 +5840,13 @@
         <v>79852</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>35432.43</v>
+        <v>41578.99000000001</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>44419.57</v>
+        <v>38273.01</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.4437262685969043</v>
+        <v>0.5207006712417974</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-08-25 15:30:18
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -2788,7 +2788,7 @@
         <v>0</v>
       </c>
       <c r="M38" s="2" t="n">
-        <v>8074.62</v>
+        <v>10503.44</v>
       </c>
       <c r="N38" s="2" t="n">
         <v>0</v>
@@ -3867,7 +3867,7 @@
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -4955,7 +4955,7 @@
         <v>104.73</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>8074.62</v>
+        <v>10503.44</v>
       </c>
       <c r="G40" s="2" t="n">
         <v>3500</v>
@@ -5458,7 +5458,7 @@
         <v>85761.95999999999</v>
       </c>
       <c r="F59" s="5" t="n">
-        <v>41578.99</v>
+        <v>44007.81</v>
       </c>
       <c r="G59" s="5" t="n">
         <v>114450</v>
@@ -5797,13 +5797,13 @@
         <v>57552</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>24134.06</v>
+        <v>26562.88</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>33417.94</v>
+        <v>30989.12</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.4193435501807062</v>
+        <v>0.4615457325549069</v>
       </c>
     </row>
     <row r="14">
@@ -5840,13 +5840,13 @@
         <v>79852</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>41578.99000000001</v>
+        <v>44007.81</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>38273.01</v>
+        <v>35844.19</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.5207006712417974</v>
+        <v>0.5511171918048389</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-08-27 08:30:20
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R55"/>
+  <dimension ref="A1:R54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -922,7 +922,7 @@
         <v>0</v>
       </c>
       <c r="K7" s="2" t="n">
-        <v>0</v>
+        <v>812.16</v>
       </c>
       <c r="L7" s="2" t="n">
         <v>0</v>
@@ -1402,7 +1402,7 @@
         <v>0</v>
       </c>
       <c r="K15" s="2" t="n">
-        <v>0</v>
+        <v>727.5599999999999</v>
       </c>
       <c r="L15" s="2" t="n">
         <v>0</v>
@@ -1888,7 +1888,7 @@
         <v>322.88</v>
       </c>
       <c r="M23" s="2" t="n">
-        <v>2903.5</v>
+        <v>3027.85</v>
       </c>
       <c r="N23" s="2" t="n">
         <v>0</v>
@@ -2521,7 +2521,7 @@
         <v>312.26</v>
       </c>
       <c r="D34" s="2" t="n">
-        <v>2062.32</v>
+        <v>4468.36</v>
       </c>
       <c r="E34" s="2" t="n">
         <v>0</v>
@@ -3654,7 +3654,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>WONG SANCHEZ PAULA SOFIA</t>
+          <t>ZUÑIGA CORONEL MARCIA LUZMILA</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
@@ -3707,144 +3707,84 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>GUERRERO FAREZ FABIAN MAURICIO</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>ZUÑIGA CORONEL MARCIA LUZMILA</t>
-        </is>
-      </c>
-      <c r="C54" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D54" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E54" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F54" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G54" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H54" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I54" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J54" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K54" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L54" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M54" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N54" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O54" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P54" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q54" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R54" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="C55" s="4" t="inlineStr">
-        <is>
-          <t>3 de 53</t>
-        </is>
-      </c>
-      <c r="D55" s="4" t="inlineStr">
-        <is>
-          <t>6 de 53</t>
-        </is>
-      </c>
-      <c r="E55" s="4" t="inlineStr">
-        <is>
-          <t>0 de 53</t>
-        </is>
-      </c>
-      <c r="F55" s="4" t="inlineStr">
-        <is>
-          <t>0 de 53</t>
-        </is>
-      </c>
-      <c r="G55" s="4" t="inlineStr">
-        <is>
-          <t>0 de 53</t>
-        </is>
-      </c>
-      <c r="H55" s="4" t="inlineStr">
-        <is>
-          <t>0 de 53</t>
-        </is>
-      </c>
-      <c r="I55" s="4" t="inlineStr">
-        <is>
-          <t>1 de 53</t>
-        </is>
-      </c>
-      <c r="J55" s="4" t="inlineStr">
-        <is>
-          <t>0 de 53</t>
-        </is>
-      </c>
-      <c r="K55" s="4" t="inlineStr">
-        <is>
-          <t>4 de 53</t>
-        </is>
-      </c>
-      <c r="L55" s="4" t="inlineStr">
-        <is>
-          <t>4 de 53</t>
-        </is>
-      </c>
-      <c r="M55" s="4" t="inlineStr">
-        <is>
-          <t>12 de 53</t>
-        </is>
-      </c>
-      <c r="N55" s="4" t="inlineStr">
-        <is>
-          <t>0 de 53</t>
-        </is>
-      </c>
-      <c r="O55" s="4" t="inlineStr">
-        <is>
-          <t>0 de 53</t>
-        </is>
-      </c>
-      <c r="P55" s="4" t="inlineStr">
-        <is>
-          <t>0 de 53</t>
-        </is>
-      </c>
-      <c r="Q55" s="4" t="inlineStr">
-        <is>
-          <t>0 de 53</t>
-        </is>
-      </c>
-      <c r="R55" s="4" t="inlineStr">
-        <is>
-          <t>0 de 53</t>
+      <c r="C54" s="4" t="inlineStr">
+        <is>
+          <t>3 de 52</t>
+        </is>
+      </c>
+      <c r="D54" s="4" t="inlineStr">
+        <is>
+          <t>6 de 52</t>
+        </is>
+      </c>
+      <c r="E54" s="4" t="inlineStr">
+        <is>
+          <t>0 de 52</t>
+        </is>
+      </c>
+      <c r="F54" s="4" t="inlineStr">
+        <is>
+          <t>0 de 52</t>
+        </is>
+      </c>
+      <c r="G54" s="4" t="inlineStr">
+        <is>
+          <t>0 de 52</t>
+        </is>
+      </c>
+      <c r="H54" s="4" t="inlineStr">
+        <is>
+          <t>0 de 52</t>
+        </is>
+      </c>
+      <c r="I54" s="4" t="inlineStr">
+        <is>
+          <t>1 de 52</t>
+        </is>
+      </c>
+      <c r="J54" s="4" t="inlineStr">
+        <is>
+          <t>0 de 52</t>
+        </is>
+      </c>
+      <c r="K54" s="4" t="inlineStr">
+        <is>
+          <t>6 de 52</t>
+        </is>
+      </c>
+      <c r="L54" s="4" t="inlineStr">
+        <is>
+          <t>4 de 52</t>
+        </is>
+      </c>
+      <c r="M54" s="4" t="inlineStr">
+        <is>
+          <t>12 de 52</t>
+        </is>
+      </c>
+      <c r="N54" s="4" t="inlineStr">
+        <is>
+          <t>0 de 52</t>
+        </is>
+      </c>
+      <c r="O54" s="4" t="inlineStr">
+        <is>
+          <t>0 de 52</t>
+        </is>
+      </c>
+      <c r="P54" s="4" t="inlineStr">
+        <is>
+          <t>0 de 52</t>
+        </is>
+      </c>
+      <c r="Q54" s="4" t="inlineStr">
+        <is>
+          <t>0 de 52</t>
+        </is>
+      </c>
+      <c r="R54" s="4" t="inlineStr">
+        <is>
+          <t>0 de 52</t>
         </is>
       </c>
     </row>
@@ -4037,7 +3977,7 @@
         <v>3259.99</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>0</v>
+        <v>812.16</v>
       </c>
       <c r="G6" s="2" t="n">
         <v>1500</v>
@@ -4253,7 +4193,7 @@
         <v>13338.07</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>11.16</v>
+        <v>738.72</v>
       </c>
       <c r="G14" s="2" t="n">
         <v>6000</v>
@@ -4469,7 +4409,7 @@
         <v>4640.2</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>3538.63</v>
+        <v>3662.98</v>
       </c>
       <c r="G22" s="2" t="n">
         <v>15000</v>
@@ -4820,7 +4760,7 @@
         <v>12800.81</v>
       </c>
       <c r="F35" s="2" t="n">
-        <v>8838.65</v>
+        <v>11244.69</v>
       </c>
       <c r="G35" s="2" t="n">
         <v>10000</v>
@@ -5458,7 +5398,7 @@
         <v>85761.95999999999</v>
       </c>
       <c r="F59" s="5" t="n">
-        <v>44007.81</v>
+        <v>48077.92</v>
       </c>
       <c r="G59" s="5" t="n">
         <v>114450</v>
@@ -5482,7 +5422,7 @@
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="23" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -5557,13 +5497,13 @@
         <v>6600</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>6279.49</v>
+        <v>8685.530000000001</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>320.5100000000002</v>
+        <v>-2085.530000000001</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>0.9514378787878788</v>
+        <v>1.315989393939394</v>
       </c>
     </row>
     <row r="4">
@@ -5725,13 +5665,13 @@
         <v>728</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>5425.62</v>
+        <v>6965.34</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>-4697.62</v>
+        <v>-6237.34</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>7.452774725274725</v>
+        <v>9.567774725274726</v>
       </c>
     </row>
     <row r="11">
@@ -5797,13 +5737,13 @@
         <v>57552</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>26562.88</v>
+        <v>26687.23</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>30989.12</v>
+        <v>30864.77</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.4615457325549069</v>
+        <v>0.4637063872671671</v>
       </c>
     </row>
     <row r="14">
@@ -5840,13 +5780,13 @@
         <v>79852</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>44007.81</v>
+        <v>48077.92</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>35844.19</v>
+        <v>31774.08</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.5511171918048389</v>
+        <v>0.6020878625457096</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-08-27 16:30:21
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -1288,7 +1288,7 @@
         <v>0</v>
       </c>
       <c r="M13" s="2" t="n">
-        <v>0</v>
+        <v>2642.83</v>
       </c>
       <c r="N13" s="2" t="n">
         <v>0</v>
@@ -3759,7 +3759,7 @@
       </c>
       <c r="M54" s="4" t="inlineStr">
         <is>
-          <t>12 de 52</t>
+          <t>13 de 52</t>
         </is>
       </c>
       <c r="N54" s="4" t="inlineStr">
@@ -4139,7 +4139,7 @@
         <v>126.44</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>0</v>
+        <v>2642.83</v>
       </c>
       <c r="G12" s="2" t="n">
         <v>6000</v>
@@ -5398,7 +5398,7 @@
         <v>85761.95999999999</v>
       </c>
       <c r="F59" s="5" t="n">
-        <v>48005.93</v>
+        <v>50648.76</v>
       </c>
       <c r="G59" s="5" t="n">
         <v>114450</v>
@@ -5737,13 +5737,13 @@
         <v>57552</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>26687.23</v>
+        <v>29330.06</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>30864.77</v>
+        <v>28221.94</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.4637063872671671</v>
+        <v>0.509627119822074</v>
       </c>
     </row>
     <row r="14">
@@ -5780,13 +5780,13 @@
         <v>79852</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>48005.93</v>
+        <v>50648.76</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>31846.07</v>
+        <v>29203.24</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.6011863196914291</v>
+        <v>0.6342829234083054</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-08-27 17:30:20
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -1528,7 +1528,7 @@
         <v>0</v>
       </c>
       <c r="M17" s="2" t="n">
-        <v>11.16</v>
+        <v>210.12</v>
       </c>
       <c r="N17" s="2" t="n">
         <v>0</v>
@@ -2782,13 +2782,13 @@
         <v>0</v>
       </c>
       <c r="K38" s="2" t="n">
-        <v>0</v>
+        <v>1488.2</v>
       </c>
       <c r="L38" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M38" s="2" t="n">
-        <v>10503.44</v>
+        <v>11710.62</v>
       </c>
       <c r="N38" s="2" t="n">
         <v>0</v>
@@ -3749,7 +3749,7 @@
       </c>
       <c r="K54" s="4" t="inlineStr">
         <is>
-          <t>6 de 52</t>
+          <t>7 de 52</t>
         </is>
       </c>
       <c r="L54" s="4" t="inlineStr">
@@ -4247,7 +4247,7 @@
         <v>1355.61</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>11.16</v>
+        <v>210.12</v>
       </c>
       <c r="G16" s="2" t="n">
         <v>3000</v>
@@ -4895,7 +4895,7 @@
         <v>104.73</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>10503.44</v>
+        <v>13198.82</v>
       </c>
       <c r="G40" s="2" t="n">
         <v>3500</v>
@@ -5398,7 +5398,7 @@
         <v>85761.95999999999</v>
       </c>
       <c r="F59" s="5" t="n">
-        <v>50648.76</v>
+        <v>53543.1</v>
       </c>
       <c r="G59" s="5" t="n">
         <v>114450</v>
@@ -5421,7 +5421,7 @@
     <col width="32" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
@@ -5665,13 +5665,13 @@
         <v>728</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>6965.34</v>
+        <v>8453.540000000001</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>-6237.34</v>
+        <v>-7725.540000000001</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>9.567774725274726</v>
+        <v>11.6120054945055</v>
       </c>
     </row>
     <row r="11">
@@ -5737,13 +5737,13 @@
         <v>57552</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>29330.06</v>
+        <v>30736.2</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>28221.94</v>
+        <v>26815.8</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.509627119822074</v>
+        <v>0.5340596330275229</v>
       </c>
     </row>
     <row r="14">
@@ -5780,13 +5780,13 @@
         <v>79852</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>50648.76</v>
+        <v>53543.10000000001</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>29203.24</v>
+        <v>26308.9</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.6342829234083054</v>
+        <v>0.6705292290737865</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-01 16:30:16
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -928,7 +928,7 @@
         <v>0</v>
       </c>
       <c r="M7" s="2" t="n">
-        <v>0</v>
+        <v>295.02</v>
       </c>
       <c r="N7" s="2" t="n">
         <v>0</v>
@@ -3759,7 +3759,7 @@
       </c>
       <c r="M54" s="4" t="inlineStr">
         <is>
-          <t>0 de 52</t>
+          <t>1 de 52</t>
         </is>
       </c>
       <c r="N54" s="4" t="inlineStr">
@@ -3977,7 +3977,7 @@
         <v>1082.88</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>0</v>
+        <v>295.02</v>
       </c>
       <c r="G6" s="2" t="n">
         <v>1500</v>
@@ -5398,7 +5398,7 @@
         <v>51483.74</v>
       </c>
       <c r="F59" s="5" t="n">
-        <v>0</v>
+        <v>295.02</v>
       </c>
       <c r="G59" s="5" t="n">
         <v>114450</v>

</xml_diff>

<commit_message>
Actualización automática 2026-09-03 09:03:49
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -3799,7 +3799,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G59"/>
+  <dimension ref="A1:G57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4682,7 +4682,7 @@
         <v>0</v>
       </c>
       <c r="G32" s="2" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33">
@@ -4979,7 +4979,7 @@
         <v>0</v>
       </c>
       <c r="G43" s="2" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44">
@@ -5276,7 +5276,7 @@
         <v>0</v>
       </c>
       <c r="G54" s="2" t="n">
-        <v>500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="55">
@@ -5287,14 +5287,14 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>WONG SANCHEZ CLAUDIA PAULINA</t>
+          <t>WONG SANCHEZ PAULA SOFIA</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
-        <v>829.09</v>
+        <v>0</v>
       </c>
       <c r="D55" s="2" t="n">
-        <v>334.62</v>
+        <v>0</v>
       </c>
       <c r="E55" s="2" t="n">
         <v>0</v>
@@ -5303,7 +5303,7 @@
         <v>0</v>
       </c>
       <c r="G55" s="2" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="56">
@@ -5314,7 +5314,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>WONG SANCHEZ PAULA SOFIA</t>
+          <t>ZUÑIGA CORONEL MARCIA LUZMILA</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
@@ -5334,74 +5334,20 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>GUERRERO FAREZ FABIAN MAURICIO</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>ZUÑIGA CORONEL MARCIA LUZMILA</t>
-        </is>
-      </c>
-      <c r="C57" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D57" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E57" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F57" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G57" s="2" t="n">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>GUERRERO FAREZ FABIAN MAURICIO</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>ZUÑIGA CORONEL MARCIA LUZMILA</t>
-        </is>
-      </c>
-      <c r="C58" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D58" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E58" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F58" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G58" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="C59" s="5" t="n">
-        <v>23521.41</v>
-      </c>
-      <c r="D59" s="5" t="n">
-        <v>85761.95999999999</v>
-      </c>
-      <c r="E59" s="5" t="n">
+      <c r="C57" s="5" t="n">
+        <v>22692.32</v>
+      </c>
+      <c r="D57" s="5" t="n">
+        <v>85427.34</v>
+      </c>
+      <c r="E57" s="5" t="n">
         <v>51483.74</v>
       </c>
-      <c r="F59" s="5" t="n">
+      <c r="F57" s="5" t="n">
         <v>295.02</v>
       </c>
-      <c r="G59" s="5" t="n">
-        <v>114450</v>
+      <c r="G57" s="5" t="n">
+        <v>111450</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-03 09:43:39
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -3799,7 +3799,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G58"/>
+  <dimension ref="A1:G57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5276,7 +5276,7 @@
         <v>0</v>
       </c>
       <c r="G54" s="2" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="55">
@@ -5287,14 +5287,14 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>WONG SANCHEZ CLAUDIA PAULINA</t>
+          <t>WONG SANCHEZ PAULA SOFIA</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
-        <v>829.09</v>
+        <v>0</v>
       </c>
       <c r="D55" s="2" t="n">
-        <v>334.62</v>
+        <v>0</v>
       </c>
       <c r="E55" s="2" t="n">
         <v>0</v>
@@ -5314,7 +5314,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>WONG SANCHEZ PAULA SOFIA</t>
+          <t>ZUÑIGA CORONEL MARCIA LUZMILA</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
@@ -5334,47 +5334,20 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>GUERRERO FAREZ FABIAN MAURICIO</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>ZUÑIGA CORONEL MARCIA LUZMILA</t>
-        </is>
-      </c>
-      <c r="C57" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D57" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E57" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F57" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G57" s="2" t="n">
-        <v>1200</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="C58" s="5" t="n">
-        <v>23521.41</v>
-      </c>
-      <c r="D58" s="5" t="n">
-        <v>85761.95999999999</v>
-      </c>
-      <c r="E58" s="5" t="n">
+      <c r="C57" s="5" t="n">
+        <v>22692.32</v>
+      </c>
+      <c r="D57" s="5" t="n">
+        <v>85427.34</v>
+      </c>
+      <c r="E57" s="5" t="n">
         <v>51483.74</v>
       </c>
-      <c r="F58" s="5" t="n">
+      <c r="F57" s="5" t="n">
         <v>295.02</v>
       </c>
-      <c r="G58" s="5" t="n">
-        <v>79187</v>
+      <c r="G57" s="5" t="n">
+        <v>76987</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-04 08:30:16
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -2905,7 +2905,7 @@
         <v>0</v>
       </c>
       <c r="L40" s="2" t="n">
-        <v>846.52</v>
+        <v>761.87</v>
       </c>
       <c r="M40" s="2" t="n">
         <v>0</v>
@@ -4814,7 +4814,7 @@
         <v>3984.02</v>
       </c>
       <c r="F37" s="2" t="n">
-        <v>846.52</v>
+        <v>761.87</v>
       </c>
       <c r="G37" s="2" t="n">
         <v>2000</v>
@@ -5074,7 +5074,7 @@
         <v>51483.74</v>
       </c>
       <c r="F47" s="5" t="n">
-        <v>11741.51</v>
+        <v>11656.86</v>
       </c>
       <c r="G47" s="5" t="n">
         <v>76987</v>

</xml_diff>

<commit_message>
Actualización automática 2026-09-07 17:30:16
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -805,7 +805,7 @@
         <v>0</v>
       </c>
       <c r="L5" s="2" t="n">
-        <v>2609.32</v>
+        <v>2900.67</v>
       </c>
       <c r="M5" s="2" t="n">
         <v>107.31</v>
@@ -1585,10 +1585,10 @@
         <v>0</v>
       </c>
       <c r="L18" s="2" t="n">
-        <v>2870.07</v>
+        <v>3731.09</v>
       </c>
       <c r="M18" s="2" t="n">
-        <v>0</v>
+        <v>5079.09</v>
       </c>
       <c r="N18" s="2" t="n">
         <v>0</v>
@@ -2548,7 +2548,7 @@
         <v>0</v>
       </c>
       <c r="M34" s="2" t="n">
-        <v>0</v>
+        <v>820.72</v>
       </c>
       <c r="N34" s="2" t="n">
         <v>0</v>
@@ -2608,7 +2608,7 @@
         <v>0</v>
       </c>
       <c r="M35" s="2" t="n">
-        <v>0</v>
+        <v>1207.18</v>
       </c>
       <c r="N35" s="2" t="n">
         <v>0</v>
@@ -2788,7 +2788,7 @@
         <v>0</v>
       </c>
       <c r="M38" s="2" t="n">
-        <v>0</v>
+        <v>967.6799999999999</v>
       </c>
       <c r="N38" s="2" t="n">
         <v>0</v>
@@ -3759,7 +3759,7 @@
       </c>
       <c r="M54" s="4" t="inlineStr">
         <is>
-          <t>3 de 52</t>
+          <t>7 de 52</t>
         </is>
       </c>
       <c r="N54" s="4" t="inlineStr">
@@ -3923,7 +3923,7 @@
         <v>-373.57</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>2716.63</v>
+        <v>3007.98</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>6174</v>
@@ -4247,7 +4247,7 @@
         <v>599.59</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>2870.07</v>
+        <v>8810.18</v>
       </c>
       <c r="G16" s="2" t="n">
         <v>5000</v>
@@ -4652,7 +4652,7 @@
         <v>11244.69</v>
       </c>
       <c r="F31" s="2" t="n">
-        <v>0</v>
+        <v>820.72</v>
       </c>
       <c r="G31" s="2" t="n">
         <v>9000</v>
@@ -4679,7 +4679,7 @@
         <v>0</v>
       </c>
       <c r="F32" s="2" t="n">
-        <v>0</v>
+        <v>1207.18</v>
       </c>
       <c r="G32" s="2" t="n">
         <v>3000</v>
@@ -4760,7 +4760,7 @@
         <v>13198.82</v>
       </c>
       <c r="F35" s="2" t="n">
-        <v>0</v>
+        <v>967.6799999999999</v>
       </c>
       <c r="G35" s="2" t="n">
         <v>2000</v>
@@ -5074,7 +5074,7 @@
         <v>51483.74</v>
       </c>
       <c r="F47" s="5" t="n">
-        <v>11656.86</v>
+        <v>20883.9</v>
       </c>
       <c r="G47" s="5" t="n">
         <v>76987</v>

</xml_diff>

<commit_message>
Actualización automática 2026-09-10 09:30:17
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -2893,10 +2893,10 @@
         <v>0</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>0</v>
+        <v>1242</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>0</v>
+        <v>267.62</v>
       </c>
       <c r="J40" s="2" t="n">
         <v>0</v>
@@ -3734,12 +3734,12 @@
       </c>
       <c r="H54" s="4" t="inlineStr">
         <is>
-          <t>0 de 52</t>
+          <t>1 de 52</t>
         </is>
       </c>
       <c r="I54" s="4" t="inlineStr">
         <is>
-          <t>0 de 52</t>
+          <t>1 de 52</t>
         </is>
       </c>
       <c r="J54" s="4" t="inlineStr">
@@ -4814,7 +4814,7 @@
         <v>3984.02</v>
       </c>
       <c r="F37" s="2" t="n">
-        <v>761.87</v>
+        <v>3497.15</v>
       </c>
       <c r="G37" s="2" t="n">
         <v>2000</v>
@@ -5074,7 +5074,7 @@
         <v>51483.74</v>
       </c>
       <c r="F47" s="5" t="n">
-        <v>20027.88</v>
+        <v>22763.16</v>
       </c>
       <c r="G47" s="5" t="n">
         <v>76987</v>
@@ -5197,13 +5197,13 @@
         <v>5532</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>0</v>
+        <v>1225.66</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>5532</v>
+        <v>4306.34</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>0</v>
+        <v>0.2215582067968185</v>
       </c>
     </row>
     <row r="5">
@@ -5269,13 +5269,13 @@
         <v>2483</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>0</v>
+        <v>1242</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>2483</v>
+        <v>1241</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>0</v>
+        <v>0.500201369311317</v>
       </c>
     </row>
     <row r="8">
@@ -5293,13 +5293,13 @@
         <v>953</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>0</v>
+        <v>267.62</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>953</v>
+        <v>685.38</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>0</v>
+        <v>0.2808184679958027</v>
       </c>
     </row>
     <row r="9">
@@ -5480,13 +5480,13 @@
         <v>85618</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>20027.88</v>
+        <v>22763.16</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>65590.12</v>
+        <v>62854.84</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.2339213716741807</v>
+        <v>0.2658688593520054</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-11 08:30:18
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -748,7 +748,7 @@
         <v>0</v>
       </c>
       <c r="M4" s="2" t="n">
-        <v>0</v>
+        <v>46.44</v>
       </c>
       <c r="N4" s="2" t="n">
         <v>0</v>
@@ -808,7 +808,7 @@
         <v>2900.67</v>
       </c>
       <c r="M5" s="2" t="n">
-        <v>107.31</v>
+        <v>1771.75</v>
       </c>
       <c r="N5" s="2" t="n">
         <v>0</v>
@@ -985,7 +985,7 @@
         <v>0</v>
       </c>
       <c r="L8" s="2" t="n">
-        <v>0</v>
+        <v>253.96</v>
       </c>
       <c r="M8" s="2" t="n">
         <v>0</v>
@@ -1381,7 +1381,7 @@
         <v>0</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>0</v>
+        <v>1093.89</v>
       </c>
       <c r="E15" s="2" t="n">
         <v>0</v>
@@ -1393,7 +1393,7 @@
         <v>0</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>0</v>
+        <v>853.2</v>
       </c>
       <c r="I15" s="2" t="n">
         <v>0</v>
@@ -1408,7 +1408,7 @@
         <v>0</v>
       </c>
       <c r="M15" s="2" t="n">
-        <v>0</v>
+        <v>4505.12</v>
       </c>
       <c r="N15" s="2" t="n">
         <v>0</v>
@@ -2185,10 +2185,10 @@
         <v>0</v>
       </c>
       <c r="L28" s="2" t="n">
-        <v>0</v>
+        <v>397.78</v>
       </c>
       <c r="M28" s="2" t="n">
-        <v>0</v>
+        <v>2481.21</v>
       </c>
       <c r="N28" s="2" t="n">
         <v>0</v>
@@ -3714,52 +3714,52 @@
       </c>
       <c r="D54" s="4" t="inlineStr">
         <is>
+          <t>1 de 52</t>
+        </is>
+      </c>
+      <c r="E54" s="4" t="inlineStr">
+        <is>
           <t>0 de 52</t>
         </is>
       </c>
-      <c r="E54" s="4" t="inlineStr">
+      <c r="F54" s="4" t="inlineStr">
         <is>
           <t>0 de 52</t>
         </is>
       </c>
-      <c r="F54" s="4" t="inlineStr">
+      <c r="G54" s="4" t="inlineStr">
         <is>
           <t>0 de 52</t>
         </is>
       </c>
-      <c r="G54" s="4" t="inlineStr">
+      <c r="H54" s="4" t="inlineStr">
+        <is>
+          <t>2 de 52</t>
+        </is>
+      </c>
+      <c r="I54" s="4" t="inlineStr">
+        <is>
+          <t>1 de 52</t>
+        </is>
+      </c>
+      <c r="J54" s="4" t="inlineStr">
         <is>
           <t>0 de 52</t>
         </is>
       </c>
-      <c r="H54" s="4" t="inlineStr">
-        <is>
-          <t>1 de 52</t>
-        </is>
-      </c>
-      <c r="I54" s="4" t="inlineStr">
-        <is>
-          <t>1 de 52</t>
-        </is>
-      </c>
-      <c r="J54" s="4" t="inlineStr">
+      <c r="K54" s="4" t="inlineStr">
         <is>
           <t>0 de 52</t>
         </is>
       </c>
-      <c r="K54" s="4" t="inlineStr">
-        <is>
-          <t>0 de 52</t>
-        </is>
-      </c>
       <c r="L54" s="4" t="inlineStr">
         <is>
-          <t>4 de 52</t>
+          <t>6 de 52</t>
         </is>
       </c>
       <c r="M54" s="4" t="inlineStr">
         <is>
-          <t>7 de 52</t>
+          <t>10 de 52</t>
         </is>
       </c>
       <c r="N54" s="4" t="inlineStr">
@@ -3896,7 +3896,7 @@
         <v>1480.96</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>0</v>
+        <v>46.44</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>3000</v>
@@ -3923,7 +3923,7 @@
         <v>-373.57</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>3007.98</v>
+        <v>4672.42</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>6174</v>
@@ -4004,7 +4004,7 @@
         <v>0</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>0</v>
+        <v>253.96</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>0</v>
@@ -4193,7 +4193,7 @@
         <v>738.72</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>0</v>
+        <v>6452.21</v>
       </c>
       <c r="G14" s="2" t="n">
         <v>5662</v>
@@ -4517,7 +4517,7 @@
         <v>1914.76</v>
       </c>
       <c r="F26" s="2" t="n">
-        <v>0</v>
+        <v>2878.99</v>
       </c>
       <c r="G26" s="2" t="n">
         <v>3000</v>
@@ -4679,7 +4679,7 @@
         <v>0</v>
       </c>
       <c r="F32" s="2" t="n">
-        <v>1207.18</v>
+        <v>2552.31</v>
       </c>
       <c r="G32" s="2" t="n">
         <v>3000</v>
@@ -5074,7 +5074,7 @@
         <v>51483.74</v>
       </c>
       <c r="F47" s="5" t="n">
-        <v>22763.16</v>
+        <v>35404.33</v>
       </c>
       <c r="G47" s="5" t="n">
         <v>76987</v>
@@ -5098,7 +5098,7 @@
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -5173,13 +5173,13 @@
         <v>6600</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>0</v>
+        <v>1093.89</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>6600</v>
+        <v>5506.11</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>0</v>
+        <v>0.1657409090909091</v>
       </c>
     </row>
     <row r="4">
@@ -5197,13 +5197,13 @@
         <v>5532</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>1225.66</v>
+        <v>2570.79</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>4306.34</v>
+        <v>2961.21</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>0.2215582067968185</v>
+        <v>0.4647125813449024</v>
       </c>
     </row>
     <row r="5">
@@ -5269,13 +5269,13 @@
         <v>2483</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>1242</v>
+        <v>2095.2</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>1241</v>
+        <v>387.8000000000002</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>0.500201369311317</v>
+        <v>0.8438179621425694</v>
       </c>
     </row>
     <row r="8">
@@ -5413,13 +5413,13 @@
         <v>2996</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>6663.25</v>
+        <v>7314.99</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>-3667.25</v>
+        <v>-4318.99</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>2.22404873164219</v>
+        <v>2.441585447263017</v>
       </c>
     </row>
     <row r="14">
@@ -5437,13 +5437,13 @@
         <v>64490</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>13245.67</v>
+        <v>21942.88</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>51244.33</v>
+        <v>42547.12</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.205391068382695</v>
+        <v>0.3402524422391068</v>
       </c>
     </row>
     <row r="15">
@@ -5480,13 +5480,13 @@
         <v>85618</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>22763.16</v>
+        <v>35404.33</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>62854.84</v>
+        <v>50213.67</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.2658688593520054</v>
+        <v>0.4135150318858184</v>
       </c>
     </row>
   </sheetData>

</xml_diff>